<commit_message>
add solution for LeetCode 504 - Base 7
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99395C60-F665-458A-B3F4-5D8F82498F07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35895BA2-C0BE-47F0-93C2-4E8CD082F796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DSA Tracker" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="92">
   <si>
     <t>No.</t>
   </si>
@@ -1039,9 +1039,15 @@
       <c r="G8" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
+      <c r="H8" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="I8" s="2">
+        <v>30</v>
+      </c>
+      <c r="J8" s="12">
+        <v>46227</v>
+      </c>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>

</xml_diff>

<commit_message>
Add Two Sum solution : Leetcode :0001
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35895BA2-C0BE-47F0-93C2-4E8CD082F796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E555ABB6-7F81-4F98-8BC1-E160FA79800E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="92">
   <si>
     <t>No.</t>
   </si>
@@ -305,7 +305,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -339,6 +339,13 @@
     </font>
     <font>
       <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
@@ -435,7 +442,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -968,7 +975,7 @@
         <v>27</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I6" s="2">
         <v>10</v>
@@ -1013,7 +1020,9 @@
       <c r="J7" s="13">
         <v>46227</v>
       </c>
-      <c r="K7" s="6"/>
+      <c r="K7" s="13">
+        <v>46228</v>
+      </c>
       <c r="L7" s="6"/>
       <c r="M7" s="6"/>
     </row>
@@ -1040,7 +1049,7 @@
         <v>38</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I8" s="2">
         <v>30</v>
@@ -1048,7 +1057,9 @@
       <c r="J8" s="12">
         <v>46227</v>
       </c>
-      <c r="K8" s="2"/>
+      <c r="K8" s="12">
+        <v>46228</v>
+      </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
     </row>
@@ -1074,9 +1085,15 @@
       <c r="G9" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6"/>
+      <c r="H9" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="I9" s="6">
+        <v>90</v>
+      </c>
+      <c r="J9" s="13">
+        <v>46228</v>
+      </c>
       <c r="K9" s="6"/>
       <c r="L9" s="6"/>
       <c r="M9" s="6"/>
@@ -1132,9 +1149,15 @@
       <c r="G11" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
+      <c r="H11" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="I11" s="6">
+        <v>20</v>
+      </c>
+      <c r="J11" s="13">
+        <v>46228</v>
+      </c>
       <c r="K11" s="6"/>
       <c r="L11" s="6"/>
       <c r="M11" s="6"/>

</xml_diff>

<commit_message>
Solve LeetCode 283: Move Zeroes using two-pointer approach
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E555ABB6-7F81-4F98-8BC1-E160FA79800E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C0EBA48-010A-483B-A4D6-20035F98F278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="92">
   <si>
     <t>No.</t>
   </si>
@@ -1089,12 +1089,14 @@
         <v>91</v>
       </c>
       <c r="I9" s="6">
-        <v>90</v>
+        <v>10</v>
       </c>
       <c r="J9" s="13">
         <v>46228</v>
       </c>
-      <c r="K9" s="6"/>
+      <c r="K9" s="13">
+        <v>46229</v>
+      </c>
       <c r="L9" s="6"/>
       <c r="M9" s="6"/>
     </row>
@@ -1158,7 +1160,9 @@
       <c r="J11" s="13">
         <v>46228</v>
       </c>
-      <c r="K11" s="6"/>
+      <c r="K11" s="13">
+        <v>46229</v>
+      </c>
       <c r="L11" s="6"/>
       <c r="M11" s="6"/>
     </row>
@@ -1213,9 +1217,15 @@
       <c r="G13" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
+      <c r="H13" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="I13" s="6">
+        <v>30</v>
+      </c>
+      <c r="J13" s="13">
+        <v>46229</v>
+      </c>
       <c r="K13" s="6"/>
       <c r="L13" s="6"/>
       <c r="M13" s="6"/>

</xml_diff>

<commit_message>
Solve LeetCode 169: Majority Element using Boyer-Moore Voting Algorithm
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C0EBA48-010A-483B-A4D6-20035F98F278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C22EB971-0C7F-42C5-8ACD-FCD9A09E5E17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="DSA Tracker" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DSA Tracker'!$A$1:$M$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DSA Tracker'!$A$1:$M$38</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="130">
   <si>
     <t>No.</t>
   </si>
@@ -31,21 +31,21 @@
     <t>Topic</t>
   </si>
   <si>
-    <t>Subtopic</t>
+    <t>What to Learn First</t>
   </si>
   <si>
     <t>Problem</t>
   </si>
   <si>
+    <t>Algorithm Used</t>
+  </si>
+  <si>
     <t>LeetCode Link</t>
   </si>
   <si>
     <t>Difficulty</t>
   </si>
   <si>
-    <t>Similar Pepcoding Topic</t>
-  </si>
-  <si>
     <t>Solved Alone?</t>
   </si>
   <si>
@@ -55,257 +55,371 @@
     <t>Date Solved</t>
   </si>
   <si>
-    <t>Revision 1 (1 day)</t>
-  </si>
-  <si>
-    <t>Revision 2 (1 week)</t>
-  </si>
-  <si>
-    <t>Revision 3 (1 month)</t>
-  </si>
-  <si>
-    <t>Basics</t>
-  </si>
-  <si>
-    <t>Getting Started</t>
+    <t>Revision 1</t>
+  </si>
+  <si>
+    <t>Revision 2</t>
+  </si>
+  <si>
+    <t>Revision 3</t>
+  </si>
+  <si>
+    <t>Math &amp; Basics</t>
+  </si>
+  <si>
+    <t>Basic Math &amp; Loops</t>
+  </si>
+  <si>
+    <t>Subtract the Product and Sum of Digits of an Integer</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/subtract-the-product-and-sum-of-digits-of-an-integer/</t>
+  </si>
+  <si>
+    <t>Easy</t>
+  </si>
+  <si>
+    <t>Number of Steps to Reduce a Number to Zero</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/number-of-steps-to-reduce-a-number-to-zero/</t>
+  </si>
+  <si>
+    <t>Power of Two</t>
+  </si>
+  <si>
+    <t>Bitwise or Repeated Division</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/power-of-two/</t>
   </si>
   <si>
     <t>Fibonacci Number</t>
   </si>
   <si>
+    <t>Recursion or DP</t>
+  </si>
+  <si>
     <t>https://leetcode.com/problems/fibonacci-number/</t>
   </si>
   <si>
-    <t>Easy</t>
-  </si>
-  <si>
-    <t>Fibonacci Numbers</t>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>22-07-2026</t>
+  </si>
+  <si>
+    <t>23-07-2026</t>
   </si>
   <si>
     <t>Climbing Stairs</t>
   </si>
   <si>
+    <t>Fibonacci Sequence</t>
+  </si>
+  <si>
     <t>https://leetcode.com/problems/climbing-stairs/</t>
   </si>
   <si>
-    <t>Math</t>
+    <t>Palindrome Number</t>
+  </si>
+  <si>
+    <t>Digit Extraction</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/palindrome-number/</t>
+  </si>
+  <si>
+    <t>24-07-2026</t>
+  </si>
+  <si>
+    <t>Reverse Integer</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/reverse-integer/</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Count Primes</t>
+  </si>
+  <si>
+    <t>Sieve of Eratosthenes</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/count-primes/</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>25-07-2026</t>
+  </si>
+  <si>
+    <t>Base 7</t>
+  </si>
+  <si>
+    <t>Base Conversion</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/base-7/</t>
+  </si>
+  <si>
+    <t>Add Binary</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/add-binary/</t>
+  </si>
+  <si>
+    <t>26-07-2026</t>
+  </si>
+  <si>
+    <t>Arrays</t>
+  </si>
+  <si>
+    <t>Basic Array Traversal</t>
+  </si>
+  <si>
+    <t>Build Array from Permutation</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/build-array-from-permutation/</t>
+  </si>
+  <si>
+    <t>Concatenation of Array</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/concatenation-of-array/</t>
+  </si>
+  <si>
+    <t>Running Sum of 1d Array</t>
+  </si>
+  <si>
+    <t>Prefix Sum</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/running-sum-of-1d-array/</t>
+  </si>
+  <si>
+    <t>Find Pivot Index</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/find-pivot-index/</t>
   </si>
   <si>
     <t>Missing Number</t>
   </si>
   <si>
+    <t>Gauss Formula or XOR</t>
+  </si>
+  <si>
     <t>https://leetcode.com/problems/missing-number/</t>
   </si>
   <si>
-    <t>Math/Loops</t>
-  </si>
-  <si>
-    <t>Palindrome Number</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/palindrome-number/</t>
-  </si>
-  <si>
-    <t>Reverse a Number</t>
-  </si>
-  <si>
-    <t>Reverse Integer</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/reverse-integer/</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>Count Primes</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/count-primes/</t>
-  </si>
-  <si>
-    <t>Prime Numbers</t>
-  </si>
-  <si>
-    <t>Number System</t>
-  </si>
-  <si>
-    <t>Base Conversion</t>
-  </si>
-  <si>
-    <t>Base 7</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/base-7/</t>
-  </si>
-  <si>
-    <t>Decimal to Any Base</t>
-  </si>
-  <si>
-    <t>Addition</t>
-  </si>
-  <si>
-    <t>Add Binary</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/add-binary/</t>
-  </si>
-  <si>
-    <t>Any Base Addition</t>
-  </si>
-  <si>
     <t>Add to Array-Form of Integer</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/add-to-array-form-of-integer/</t>
   </si>
   <si>
-    <t>Sum of two arrays</t>
-  </si>
-  <si>
-    <t>Arrays</t>
-  </si>
-  <si>
-    <t>Search/Math</t>
+    <t>Best Time to Buy and Sell Stock</t>
+  </si>
+  <si>
+    <t>Track Min Value</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock/</t>
+  </si>
+  <si>
+    <t>Arrays - Two Pointers</t>
+  </si>
+  <si>
+    <t>Two Pointers Technique</t>
+  </si>
+  <si>
+    <t>Reverse String</t>
+  </si>
+  <si>
+    <t>Two Pointers (Left/Right)</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/reverse-string/</t>
+  </si>
+  <si>
+    <t>Remove Element</t>
+  </si>
+  <si>
+    <t>Two Pointers (Slow/Fast)</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/remove-element/</t>
+  </si>
+  <si>
+    <t>Move Zeroes</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/move-zeroes/</t>
+  </si>
+  <si>
+    <t>27-07-2026</t>
+  </si>
+  <si>
+    <t>Squares of a Sorted Array</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/squares-of-a-sorted-array/</t>
+  </si>
+  <si>
+    <t>28-07-2026</t>
+  </si>
+  <si>
+    <t>Binary Search &amp; Sort</t>
+  </si>
+  <si>
+    <t>Binary Search</t>
+  </si>
+  <si>
+    <t>Find Target Indices After Sorting Array</t>
+  </si>
+  <si>
+    <t>Sorting</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/find-target-indices-after-sorting-array/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/binary-search/</t>
+  </si>
+  <si>
+    <t>Search Insert Position</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/search-insert-position/</t>
+  </si>
+  <si>
+    <t>First Bad Version</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/first-bad-version/</t>
+  </si>
+  <si>
+    <t>Hashing</t>
+  </si>
+  <si>
+    <t>HashMaps &amp; HashSets</t>
+  </si>
+  <si>
+    <t>Jewels and Stones</t>
+  </si>
+  <si>
+    <t>HashSet</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/jewels-and-stones/</t>
+  </si>
+  <si>
+    <t>Contains Duplicate</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/contains-duplicate/</t>
+  </si>
+  <si>
+    <t>Valid Anagram</t>
+  </si>
+  <si>
+    <t>HashMap / Frequency Array</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/valid-anagram/</t>
   </si>
   <si>
     <t>Two Sum</t>
   </si>
   <si>
+    <t>HashMap</t>
+  </si>
+  <si>
     <t>https://leetcode.com/problems/two-sum/</t>
   </si>
   <si>
-    <t>Find Element in Array</t>
-  </si>
-  <si>
-    <t>Find Target Indices After Sorting Array</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/find-target-indices-after-sorting-array/</t>
-  </si>
-  <si>
-    <t>Two Pointers</t>
-  </si>
-  <si>
-    <t>Move Zeroes</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/move-zeroes/</t>
-  </si>
-  <si>
-    <t>Array Manipulation</t>
-  </si>
-  <si>
-    <t>Squares of a Sorted Array</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/squares-of-a-sorted-array/</t>
-  </si>
-  <si>
-    <t>Counting</t>
-  </si>
-  <si>
     <t>Majority Element</t>
   </si>
   <si>
+    <t>Moore's Voting Algorithm</t>
+  </si>
+  <si>
     <t>https://leetcode.com/problems/majority-element/</t>
   </si>
   <si>
-    <t>Subarrays</t>
-  </si>
-  <si>
-    <t>Best Time to Buy and Sell Stock</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock/</t>
+    <t>Stacks</t>
+  </si>
+  <si>
+    <t>Stack Data Structure</t>
+  </si>
+  <si>
+    <t>Valid Parentheses</t>
   </si>
   <si>
     <t>Stack</t>
   </si>
   <si>
-    <t>Basic Stack</t>
-  </si>
-  <si>
-    <t>Valid Parentheses</t>
-  </si>
-  <si>
     <t>https://leetcode.com/problems/valid-parentheses/</t>
   </si>
   <si>
-    <t>Balanced Brackets</t>
-  </si>
-  <si>
     <t>Remove Outermost Parentheses</t>
   </si>
   <si>
+    <t>Stack or Counter</t>
+  </si>
+  <si>
     <t>https://leetcode.com/problems/remove-outermost-parentheses/</t>
   </si>
   <si>
-    <t>Duplicate Brackets</t>
-  </si>
-  <si>
     <t>Remove All Adjacent Duplicates In String</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/remove-all-adjacent-duplicates-in-string/</t>
   </si>
   <si>
-    <t>Stack Basics</t>
-  </si>
-  <si>
-    <t>Design</t>
-  </si>
-  <si>
     <t>Min Stack</t>
   </si>
   <si>
+    <t>Two Stacks</t>
+  </si>
+  <si>
     <t>https://leetcode.com/problems/min-stack/</t>
   </si>
   <si>
-    <t>Minimum Stack - 1</t>
-  </si>
-  <si>
-    <t>Evaluation</t>
-  </si>
-  <si>
     <t>Evaluate Reverse Polish Notation</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/evaluate-reverse-polish-notation/</t>
   </si>
   <si>
-    <t>Postfix Evaluations</t>
+    <t>Next Greater Element I</t>
   </si>
   <si>
     <t>Monotonic Stack</t>
   </si>
   <si>
-    <t>Next Greater Element I</t>
-  </si>
-  <si>
     <t>https://leetcode.com/problems/next-greater-element-i/</t>
   </si>
   <si>
-    <t>Next Greater Element on the Right</t>
-  </si>
-  <si>
     <t>Daily Temperatures</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/daily-temperatures/</t>
-  </si>
-  <si>
-    <t>YES</t>
-  </si>
-  <si>
-    <t>NO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -336,21 +450,6 @@
       <sz val="11"/>
       <color rgb="FFE36C09"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -397,11 +496,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -442,12 +540,8 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -748,19 +842,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="5" width="45" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="35" customWidth="1"/>
-    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="2" max="2" width="18.44140625" customWidth="1"/>
+    <col min="3" max="3" width="25.77734375" customWidth="1"/>
+    <col min="4" max="4" width="45" customWidth="1"/>
+    <col min="5" max="5" width="29.21875" customWidth="1"/>
+    <col min="6" max="6" width="45" customWidth="1"/>
+    <col min="7" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
     <col min="10" max="10" width="15" customWidth="1"/>
-    <col min="11" max="13" width="18" customWidth="1"/>
+    <col min="11" max="14" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
@@ -817,27 +911,25 @@
       <c r="D2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>90</v>
+      <c r="G2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>27</v>
       </c>
       <c r="I2" s="2">
         <v>5</v>
       </c>
       <c r="J2" s="12">
-        <v>46225</v>
-      </c>
-      <c r="K2" s="12">
-        <v>46226</v>
-      </c>
+        <v>46231</v>
+      </c>
+      <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
     </row>
@@ -854,27 +946,25 @@
       <c r="D3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>90</v>
+      <c r="G3" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>43</v>
       </c>
       <c r="I3" s="6">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="J3" s="13">
-        <v>46225</v>
-      </c>
-      <c r="K3" s="13">
-        <v>46226</v>
-      </c>
+        <v>46231</v>
+      </c>
+      <c r="K3" s="6"/>
       <c r="L3" s="6"/>
       <c r="M3" s="6"/>
     </row>
@@ -886,32 +976,24 @@
         <v>13</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="I4" s="2">
-        <v>10</v>
-      </c>
-      <c r="J4" s="12">
-        <v>46226</v>
-      </c>
-      <c r="K4" s="12">
-        <v>46227</v>
-      </c>
+      <c r="G4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H4" s="3"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
     </row>
@@ -923,31 +1005,31 @@
         <v>13</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="D5" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="F5" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="H5" s="6" t="s">
-        <v>90</v>
-      </c>
       <c r="I5" s="6">
-        <v>10</v>
-      </c>
-      <c r="J5" s="13">
-        <v>46226</v>
-      </c>
-      <c r="K5" s="13">
-        <v>46227</v>
+        <v>5</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>29</v>
       </c>
       <c r="L5" s="6"/>
       <c r="M5" s="6"/>
@@ -960,31 +1042,31 @@
         <v>13</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="D6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I6" s="2">
+        <v>5</v>
+      </c>
+      <c r="J6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="K6" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="I6" s="2">
-        <v>10</v>
-      </c>
-      <c r="J6" s="12">
-        <v>46226</v>
-      </c>
-      <c r="K6" s="12">
-        <v>46227</v>
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
@@ -997,31 +1079,31 @@
         <v>13</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="F7" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="G7" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="H7" s="6" t="s">
-        <v>91</v>
+      <c r="E7" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>27</v>
       </c>
       <c r="I7" s="6">
-        <v>30</v>
-      </c>
-      <c r="J7" s="13">
-        <v>46227</v>
-      </c>
-      <c r="K7" s="13">
-        <v>46228</v>
+        <v>10</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>36</v>
       </c>
       <c r="L7" s="6"/>
       <c r="M7" s="6"/>
@@ -1031,34 +1113,34 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" s="3" t="s">
+      <c r="F8" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I8" s="2">
+        <v>10</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K8" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="I8" s="2">
-        <v>30</v>
-      </c>
-      <c r="J8" s="12">
-        <v>46227</v>
-      </c>
-      <c r="K8" s="12">
-        <v>46228</v>
       </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
@@ -1068,34 +1150,34 @@
         <v>8</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="F9" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="G9" s="7" t="s">
+      <c r="F9" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="H9" s="6" t="s">
-        <v>91</v>
+      <c r="G9" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>43</v>
       </c>
       <c r="I9" s="6">
-        <v>10</v>
-      </c>
-      <c r="J9" s="13">
-        <v>46228</v>
-      </c>
-      <c r="K9" s="13">
-        <v>46229</v>
+        <v>30</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>44</v>
       </c>
       <c r="L9" s="6"/>
       <c r="M9" s="6"/>
@@ -1105,27 +1187,35 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="E10" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I10" s="2">
+        <v>30</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K10" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
     </row>
@@ -1134,34 +1224,34 @@
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="F11" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="I11" s="6">
+        <v>10</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="K11" s="6" t="s">
         <v>50</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="I11" s="6">
-        <v>20</v>
-      </c>
-      <c r="J11" s="13">
-        <v>46228</v>
-      </c>
-      <c r="K11" s="13">
-        <v>46229</v>
       </c>
       <c r="L11" s="6"/>
       <c r="M11" s="6"/>
@@ -1171,24 +1261,24 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="H12" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H12" s="3"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
@@ -1200,32 +1290,26 @@
         <v>12</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="E13" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="F13" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="G13" s="7" t="s">
+      <c r="E13" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="H13" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="I13" s="6">
-        <v>30</v>
-      </c>
-      <c r="J13" s="13">
-        <v>46229</v>
-      </c>
+      <c r="G13" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H13" s="7"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
       <c r="K13" s="6"/>
       <c r="L13" s="6"/>
       <c r="M13" s="6"/>
@@ -1235,24 +1319,24 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="F14" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H14" s="2"/>
+      <c r="F14" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H14" s="3"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
@@ -1264,24 +1348,24 @@
         <v>14</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="F15" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="F15" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="H15" s="6"/>
+      <c r="G15" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H15" s="7"/>
       <c r="I15" s="6"/>
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
@@ -1293,27 +1377,35 @@
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C16" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="E16" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="F16" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="F16" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
+      <c r="G16" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I16" s="2">
+        <v>10</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>36</v>
+      </c>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
     </row>
@@ -1322,24 +1414,24 @@
         <v>16</v>
       </c>
       <c r="B17" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D17" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="E17" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F17" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="D17" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="F17" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H17" s="6"/>
+      <c r="G17" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H17" s="7"/>
       <c r="I17" s="6"/>
       <c r="J17" s="6"/>
       <c r="K17" s="6"/>
@@ -1351,24 +1443,24 @@
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="H18" s="2"/>
+        <v>67</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H18" s="3"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
@@ -1380,24 +1472,24 @@
         <v>18</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="D19" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E19" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="F19" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="F19" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="G19" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="H19" s="6"/>
+      <c r="G19" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H19" s="7"/>
       <c r="I19" s="6"/>
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
@@ -1409,24 +1501,24 @@
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C20" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="E20" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="F20" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="E20" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="F20" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="H20" s="2"/>
+      <c r="G20" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H20" s="3"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
@@ -1438,27 +1530,35 @@
         <v>20</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C21" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="I21" s="6">
+        <v>5</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K21" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="D21" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="F21" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="G21" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
-      <c r="J21" s="6"/>
-      <c r="K21" s="6"/>
       <c r="L21" s="6"/>
       <c r="M21" s="6"/>
     </row>
@@ -1467,27 +1567,35 @@
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
+        <v>81</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I22" s="2">
+        <v>10</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>83</v>
+      </c>
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
     </row>
@@ -1496,57 +1604,522 @@
         <v>22</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D23" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F23" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="E23" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="F23" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="G23" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="H23" s="6"/>
+      <c r="G23" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H23" s="7"/>
       <c r="I23" s="6"/>
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
       <c r="L23" s="6"/>
       <c r="M23" s="6"/>
     </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A24" s="2">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H24" s="3"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="2"/>
+      <c r="M24" s="2"/>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A25" s="6">
+        <v>24</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H25" s="7"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="6"/>
+      <c r="K25" s="6"/>
+      <c r="L25" s="6"/>
+      <c r="M25" s="6"/>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A26" s="2">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="G26" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H26" s="3"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
+      <c r="L26" s="2"/>
+      <c r="M26" s="2"/>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A27" s="6">
+        <v>26</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="G27" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H27" s="7"/>
+      <c r="I27" s="6"/>
+      <c r="J27" s="6"/>
+      <c r="K27" s="6"/>
+      <c r="L27" s="6"/>
+      <c r="M27" s="6"/>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A28" s="2">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="G28" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H28" s="3"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="2"/>
+      <c r="K28" s="2"/>
+      <c r="L28" s="2"/>
+      <c r="M28" s="2"/>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A29" s="6">
+        <v>28</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="G29" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H29" s="7"/>
+      <c r="I29" s="6"/>
+      <c r="J29" s="6"/>
+      <c r="K29" s="6"/>
+      <c r="L29" s="6"/>
+      <c r="M29" s="6"/>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A30" s="2">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I30" s="2">
+        <v>20</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="L30" s="2"/>
+      <c r="M30" s="2"/>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A31" s="6">
+        <v>30</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="I31" s="6">
+        <v>40</v>
+      </c>
+      <c r="J31" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="K31" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="L31" s="6"/>
+      <c r="M31" s="6"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A32" s="2">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H32" s="3"/>
+      <c r="I32" s="2"/>
+      <c r="J32" s="2"/>
+      <c r="K32" s="2"/>
+      <c r="L32" s="2"/>
+      <c r="M32" s="2"/>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A33" s="6">
+        <v>32</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="G33" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H33" s="7"/>
+      <c r="I33" s="6"/>
+      <c r="J33" s="6"/>
+      <c r="K33" s="6"/>
+      <c r="L33" s="6"/>
+      <c r="M33" s="6"/>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A34" s="2">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H34" s="3"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="2"/>
+      <c r="K34" s="2"/>
+      <c r="L34" s="2"/>
+      <c r="M34" s="2"/>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A35" s="6">
+        <v>34</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="G35" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="H35" s="7"/>
+      <c r="I35" s="6"/>
+      <c r="J35" s="6"/>
+      <c r="K35" s="6"/>
+      <c r="L35" s="6"/>
+      <c r="M35" s="6"/>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A36" s="2">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="G36" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="H36" s="3"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="2"/>
+      <c r="K36" s="2"/>
+      <c r="L36" s="2"/>
+      <c r="M36" s="2"/>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A37" s="6">
+        <v>36</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="G37" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H37" s="7"/>
+      <c r="I37" s="6"/>
+      <c r="J37" s="6"/>
+      <c r="K37" s="6"/>
+      <c r="L37" s="6"/>
+      <c r="M37" s="6"/>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A38" s="2">
+        <v>37</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="G38" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="H38" s="3"/>
+      <c r="I38" s="2"/>
+      <c r="J38" s="2"/>
+      <c r="K38" s="2"/>
+      <c r="L38" s="2"/>
+      <c r="M38" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M23" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:M38" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="E3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="E4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="E5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="E6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="E7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="E8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="E9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="E10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="E11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="E12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="E13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="E14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="E15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="E16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="E17" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="E18" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="E19" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="E20" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="E21" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="E22" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="E23" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="F4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="F5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="F6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="F7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="F8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="F9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="F10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="F11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="F12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="F13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="F14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="F15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="F16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="F17" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="F18" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="F19" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="F20" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="F21" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="F22" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="F23" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="F24" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="F25" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="F26" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="F27" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="F28" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="F29" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="F30" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="F31" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="F32" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="F33" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="F34" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="F35" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="F36" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="F37" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="F38" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId23"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed class name issue
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C22EB971-0C7F-42C5-8ACD-FCD9A09E5E17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9505E845-FC4F-41AF-937D-0C8B1A5512FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="130">
   <si>
     <t>No.</t>
   </si>
@@ -990,9 +990,15 @@
       <c r="G4" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="3"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
+      <c r="H4" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I4" s="2">
+        <v>5</v>
+      </c>
+      <c r="J4" s="12">
+        <v>46231</v>
+      </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>

</xml_diff>

<commit_message>
Add solution for LeetCode 121 - Best Time to Buy and Sell Stock
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9505E845-FC4F-41AF-937D-0C8B1A5512FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B31E4C69-19FA-4325-AB3A-1890569EB1E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="130">
   <si>
     <t>No.</t>
   </si>
@@ -849,7 +849,7 @@
     <col min="2" max="2" width="18.44140625" customWidth="1"/>
     <col min="3" max="3" width="25.77734375" customWidth="1"/>
     <col min="4" max="4" width="45" customWidth="1"/>
-    <col min="5" max="5" width="29.21875" customWidth="1"/>
+    <col min="5" max="5" width="30.44140625" customWidth="1"/>
     <col min="6" max="6" width="45" customWidth="1"/>
     <col min="7" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
@@ -929,7 +929,9 @@
       <c r="J2" s="12">
         <v>46231</v>
       </c>
-      <c r="K2" s="2"/>
+      <c r="K2" s="12">
+        <v>46232</v>
+      </c>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
     </row>
@@ -959,12 +961,14 @@
         <v>43</v>
       </c>
       <c r="I3" s="6">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="J3" s="13">
         <v>46231</v>
       </c>
-      <c r="K3" s="6"/>
+      <c r="K3" s="13">
+        <v>46232</v>
+      </c>
       <c r="L3" s="6"/>
       <c r="M3" s="6"/>
     </row>
@@ -991,7 +995,7 @@
         <v>18</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="I4" s="2">
         <v>5</v>
@@ -999,7 +1003,9 @@
       <c r="J4" s="12">
         <v>46231</v>
       </c>
-      <c r="K4" s="2"/>
+      <c r="K4" s="12">
+        <v>46232</v>
+      </c>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
     </row>
@@ -1037,7 +1043,9 @@
       <c r="K5" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="L5" s="6"/>
+      <c r="L5" s="13">
+        <v>46232</v>
+      </c>
       <c r="M5" s="6"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
@@ -1074,7 +1082,9 @@
       <c r="K6" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="L6" s="2"/>
+      <c r="L6" s="12">
+        <v>46232</v>
+      </c>
       <c r="M6" s="2"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
@@ -1466,9 +1476,15 @@
       <c r="G18" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H18" s="3"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
+      <c r="H18" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I18" s="2">
+        <v>20</v>
+      </c>
+      <c r="J18" s="12">
+        <v>46232</v>
+      </c>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>

</xml_diff>

<commit_message>
Fix the class name issue
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B31E4C69-19FA-4325-AB3A-1890569EB1E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92443A3A-A4B9-4AC3-892B-F37A8A0CD935}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -842,6 +842,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:M38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -898,7 +899,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -935,7 +936,7 @@
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -972,7 +973,7 @@
       <c r="L3" s="6"/>
       <c r="M3" s="6"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1009,7 +1010,7 @@
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -1048,7 +1049,7 @@
       </c>
       <c r="M5" s="6"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1121,7 +1122,9 @@
       <c r="K7" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="L7" s="6"/>
+      <c r="L7" s="13">
+        <v>46233</v>
+      </c>
       <c r="M7" s="6"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
@@ -1161,7 +1164,7 @@
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -1198,7 +1201,7 @@
       <c r="L9" s="6"/>
       <c r="M9" s="6"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1235,7 +1238,7 @@
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -1272,7 +1275,7 @@
       <c r="L11" s="6"/>
       <c r="M11" s="6"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1301,7 +1304,7 @@
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -1330,7 +1333,7 @@
       <c r="L13" s="6"/>
       <c r="M13" s="6"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1359,7 +1362,7 @@
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -1425,7 +1428,7 @@
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -1454,7 +1457,7 @@
       <c r="L17" s="6"/>
       <c r="M17" s="6"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1489,7 +1492,7 @@
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -1518,7 +1521,7 @@
       <c r="L19" s="6"/>
       <c r="M19" s="6"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1547,7 +1550,7 @@
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -1584,7 +1587,7 @@
       <c r="L21" s="6"/>
       <c r="M21" s="6"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1621,7 +1624,7 @@
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -1650,7 +1653,7 @@
       <c r="L23" s="6"/>
       <c r="M23" s="6"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1679,7 +1682,7 @@
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -1708,7 +1711,7 @@
       <c r="L25" s="6"/>
       <c r="M25" s="6"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -1737,7 +1740,7 @@
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -1766,7 +1769,7 @@
       <c r="L27" s="6"/>
       <c r="M27" s="6"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -1795,7 +1798,7 @@
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -1824,7 +1827,7 @@
       <c r="L29" s="6"/>
       <c r="M29" s="6"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -1861,7 +1864,7 @@
       <c r="L30" s="2"/>
       <c r="M30" s="2"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="6">
         <v>30</v>
       </c>
@@ -1898,7 +1901,7 @@
       <c r="L31" s="6"/>
       <c r="M31" s="6"/>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -1927,7 +1930,7 @@
       <c r="L32" s="2"/>
       <c r="M32" s="2"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="6">
         <v>32</v>
       </c>
@@ -1956,7 +1959,7 @@
       <c r="L33" s="6"/>
       <c r="M33" s="6"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -1985,7 +1988,7 @@
       <c r="L34" s="2"/>
       <c r="M34" s="2"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="6">
         <v>34</v>
       </c>
@@ -2014,7 +2017,7 @@
       <c r="L35" s="6"/>
       <c r="M35" s="6"/>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -2043,7 +2046,7 @@
       <c r="L36" s="2"/>
       <c r="M36" s="2"/>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="6">
         <v>36</v>
       </c>
@@ -2072,7 +2075,7 @@
       <c r="L37" s="6"/>
       <c r="M37" s="6"/>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -2102,7 +2105,13 @@
       <c r="M38" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M38" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:M38" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="9">
+      <filters>
+        <filter val="23-07-2026"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="F3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>

</xml_diff>

<commit_message>
Solve LeetCode 1929: Concatenation of Array
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92443A3A-A4B9-4AC3-892B-F37A8A0CD935}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84BBD3D8-1675-4EB1-BB24-D15FEACAB99E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -842,7 +842,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:M38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -899,7 +898,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -936,7 +935,7 @@
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
     </row>
-    <row r="3" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -973,7 +972,7 @@
       <c r="L3" s="6"/>
       <c r="M3" s="6"/>
     </row>
-    <row r="4" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1010,7 +1009,7 @@
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
     </row>
-    <row r="5" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -1049,7 +1048,7 @@
       </c>
       <c r="M5" s="6"/>
     </row>
-    <row r="6" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1161,10 +1160,12 @@
       <c r="K8" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="L8" s="2"/>
+      <c r="L8" s="12">
+        <v>46233</v>
+      </c>
       <c r="M8" s="2"/>
     </row>
-    <row r="9" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -1198,10 +1199,12 @@
       <c r="K9" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="L9" s="6"/>
+      <c r="L9" s="13">
+        <v>46233</v>
+      </c>
       <c r="M9" s="6"/>
     </row>
-    <row r="10" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1238,7 +1241,7 @@
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
     </row>
-    <row r="11" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -1275,7 +1278,7 @@
       <c r="L11" s="6"/>
       <c r="M11" s="6"/>
     </row>
-    <row r="12" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1304,7 +1307,7 @@
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
     </row>
-    <row r="13" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -1333,7 +1336,7 @@
       <c r="L13" s="6"/>
       <c r="M13" s="6"/>
     </row>
-    <row r="14" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1362,7 +1365,7 @@
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
     </row>
-    <row r="15" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -1425,10 +1428,12 @@
       <c r="K16" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="L16" s="2"/>
+      <c r="L16" s="12">
+        <v>46233</v>
+      </c>
       <c r="M16" s="2"/>
     </row>
-    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -1457,7 +1462,7 @@
       <c r="L17" s="6"/>
       <c r="M17" s="6"/>
     </row>
-    <row r="18" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1492,7 +1497,7 @@
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
     </row>
-    <row r="19" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -1521,7 +1526,7 @@
       <c r="L19" s="6"/>
       <c r="M19" s="6"/>
     </row>
-    <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1550,7 +1555,7 @@
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
     </row>
-    <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -1587,7 +1592,7 @@
       <c r="L21" s="6"/>
       <c r="M21" s="6"/>
     </row>
-    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1624,7 +1629,7 @@
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
     </row>
-    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -1653,7 +1658,7 @@
       <c r="L23" s="6"/>
       <c r="M23" s="6"/>
     </row>
-    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1682,7 +1687,7 @@
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
     </row>
-    <row r="25" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -1711,7 +1716,7 @@
       <c r="L25" s="6"/>
       <c r="M25" s="6"/>
     </row>
-    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -1740,7 +1745,7 @@
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
     </row>
-    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -1769,7 +1774,7 @@
       <c r="L27" s="6"/>
       <c r="M27" s="6"/>
     </row>
-    <row r="28" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -1798,7 +1803,7 @@
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
     </row>
-    <row r="29" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -1827,7 +1832,7 @@
       <c r="L29" s="6"/>
       <c r="M29" s="6"/>
     </row>
-    <row r="30" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -1864,7 +1869,7 @@
       <c r="L30" s="2"/>
       <c r="M30" s="2"/>
     </row>
-    <row r="31" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" s="6">
         <v>30</v>
       </c>
@@ -1901,7 +1906,7 @@
       <c r="L31" s="6"/>
       <c r="M31" s="6"/>
     </row>
-    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -1930,7 +1935,7 @@
       <c r="L32" s="2"/>
       <c r="M32" s="2"/>
     </row>
-    <row r="33" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" s="6">
         <v>32</v>
       </c>
@@ -1959,7 +1964,7 @@
       <c r="L33" s="6"/>
       <c r="M33" s="6"/>
     </row>
-    <row r="34" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -1988,7 +1993,7 @@
       <c r="L34" s="2"/>
       <c r="M34" s="2"/>
     </row>
-    <row r="35" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" s="6">
         <v>34</v>
       </c>
@@ -2017,7 +2022,7 @@
       <c r="L35" s="6"/>
       <c r="M35" s="6"/>
     </row>
-    <row r="36" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -2046,7 +2051,7 @@
       <c r="L36" s="2"/>
       <c r="M36" s="2"/>
     </row>
-    <row r="37" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A37" s="6">
         <v>36</v>
       </c>
@@ -2075,7 +2080,7 @@
       <c r="L37" s="6"/>
       <c r="M37" s="6"/>
     </row>
-    <row r="38" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -2105,13 +2110,7 @@
       <c r="M38" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M38" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <filterColumn colId="9">
-      <filters>
-        <filter val="23-07-2026"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:M38" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="F3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>

</xml_diff>

<commit_message>
Solve LeetCode 2235: Add Two Integers solution
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84BBD3D8-1675-4EB1-BB24-D15FEACAB99E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_2B59E58F1BF641346044C83044E160314FECB551" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="DSA Tracker" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DSA Tracker'!$A$1:$M$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DSA Tracker'!$A$1:$M$48</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="163">
   <si>
     <t>No.</t>
   </si>
@@ -64,6 +64,42 @@
     <t>Revision 3</t>
   </si>
   <si>
+    <t>Absolute Basics</t>
+  </si>
+  <si>
+    <t>Writing a return statement</t>
+  </si>
+  <si>
+    <t>Add Two Integers</t>
+  </si>
+  <si>
+    <t>Math</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/add-two-integers/</t>
+  </si>
+  <si>
+    <t>Easy</t>
+  </si>
+  <si>
+    <t>Basic Math Formulas</t>
+  </si>
+  <si>
+    <t>Convert the Temperature</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/convert-the-temperature/</t>
+  </si>
+  <si>
+    <t>If/Else Statements</t>
+  </si>
+  <si>
+    <t>Smallest Even Multiple</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/smallest-even-multiple/</t>
+  </si>
+  <si>
     <t>Math &amp; Basics</t>
   </si>
   <si>
@@ -79,9 +115,6 @@
     <t>https://leetcode.com/problems/subtract-the-product-and-sum-of-digits-of-an-integer/</t>
   </si>
   <si>
-    <t>Easy</t>
-  </si>
-  <si>
     <t>Number of Steps to Reduce a Number to Zero</t>
   </si>
   <si>
@@ -178,6 +211,36 @@
     <t>26-07-2026</t>
   </si>
   <si>
+    <t>Strings</t>
+  </si>
+  <si>
+    <t>String Manipulation</t>
+  </si>
+  <si>
+    <t>Score of a String</t>
+  </si>
+  <si>
+    <t>ASCII Values</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/score-of-a-string/</t>
+  </si>
+  <si>
+    <t>Defanging an IP Address</t>
+  </si>
+  <si>
+    <t>String Replace</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/defanging-an-ip-address/</t>
+  </si>
+  <si>
+    <t>Goal Parser Interpretation</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/goal-parser-interpretation/</t>
+  </si>
+  <si>
     <t>Arrays</t>
   </si>
   <si>
@@ -196,6 +259,33 @@
     <t>https://leetcode.com/problems/concatenation-of-array/</t>
   </si>
   <si>
+    <t>Shuffle the Array</t>
+  </si>
+  <si>
+    <t>Array Indexing</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/shuffle-the-array/</t>
+  </si>
+  <si>
+    <t>Kids With the Greatest Number of Candies</t>
+  </si>
+  <si>
+    <t>Find Max &amp; Loop</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/kids-with-the-greatest-number-of-candies/</t>
+  </si>
+  <si>
+    <t>Richest Customer Wealth</t>
+  </si>
+  <si>
+    <t>2D Array Traversal</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/richest-customer-wealth/</t>
+  </si>
+  <si>
     <t>Running Sum of 1d Array</t>
   </si>
   <si>
@@ -320,6 +410,15 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/jewels-and-stones/</t>
+  </si>
+  <si>
+    <t>How Many Numbers Are Smaller Than the Current Number</t>
+  </si>
+  <si>
+    <t>Frequency Array</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/how-many-numbers-are-smaller-than-the-current-number/</t>
   </si>
   <si>
     <t>Contains Duplicate</t>
@@ -499,7 +598,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -528,16 +627,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -842,14 +935,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:M48"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="18.44140625" customWidth="1"/>
-    <col min="3" max="3" width="25.77734375" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="45" customWidth="1"/>
-    <col min="5" max="5" width="30.44140625" customWidth="1"/>
+    <col min="5" max="5" width="25" customWidth="1"/>
     <col min="6" max="6" width="45" customWidth="1"/>
     <col min="7" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
@@ -920,18 +1013,10 @@
       <c r="G2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I2" s="2">
-        <v>5</v>
-      </c>
-      <c r="J2" s="12">
-        <v>46231</v>
-      </c>
-      <c r="K2" s="12">
-        <v>46232</v>
-      </c>
+      <c r="H2" s="3"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
     </row>
@@ -943,32 +1028,24 @@
         <v>13</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E3" s="7" t="s">
         <v>16</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G3" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="I3" s="6">
-        <v>5</v>
-      </c>
-      <c r="J3" s="13">
-        <v>46231</v>
-      </c>
-      <c r="K3" s="13">
-        <v>46232</v>
-      </c>
+      <c r="H3" s="7"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
       <c r="L3" s="6"/>
       <c r="M3" s="6"/>
     </row>
@@ -980,32 +1057,24 @@
         <v>13</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I4" s="2">
-        <v>5</v>
-      </c>
-      <c r="J4" s="12">
-        <v>46231</v>
-      </c>
-      <c r="K4" s="12">
-        <v>46232</v>
-      </c>
+      <c r="H4" s="3"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
     </row>
@@ -1014,38 +1083,28 @@
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I5" s="6">
-        <v>5</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="K5" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="L5" s="13">
-        <v>46232</v>
-      </c>
+      <c r="H5" s="7"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
       <c r="M5" s="6"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
@@ -1053,38 +1112,28 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>30</v>
       </c>
       <c r="E6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F6" s="4" t="s">
-        <v>32</v>
-      </c>
       <c r="G6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I6" s="2">
-        <v>5</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="L6" s="12">
-        <v>46232</v>
-      </c>
+      <c r="H6" s="3"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
       <c r="M6" s="2"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
@@ -1092,38 +1141,28 @@
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="D7" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="F7" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="F7" s="8" t="s">
-        <v>35</v>
-      </c>
       <c r="G7" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I7" s="6">
-        <v>10</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="K7" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="L7" s="13">
-        <v>46233</v>
-      </c>
+      <c r="H7" s="7"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
       <c r="M7" s="6"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
@@ -1131,38 +1170,36 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="D8" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F8" s="4" t="s">
+      <c r="G8" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H8" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="I8" s="2">
+        <v>5</v>
+      </c>
+      <c r="J8" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="H8" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I8" s="2">
-        <v>10</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="K8" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="L8" s="12">
-        <v>46233</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="L8" s="2"/>
       <c r="M8" s="2"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
@@ -1170,38 +1207,36 @@
         <v>8</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="D9" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="I9" s="6">
+        <v>5</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="K9" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="G9" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="I9" s="6">
-        <v>30</v>
-      </c>
-      <c r="J9" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="K9" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="L9" s="13">
-        <v>46233</v>
-      </c>
+      <c r="L9" s="6"/>
       <c r="M9" s="6"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
@@ -1209,34 +1244,34 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="D10" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="F10" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="G10" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I10" s="2">
+        <v>10</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K10" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I10" s="2">
-        <v>30</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>44</v>
       </c>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
@@ -1246,34 +1281,34 @@
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>48</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="G11" s="9" t="s">
-        <v>18</v>
+      <c r="G11" s="10" t="s">
+        <v>50</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="I11" s="6">
         <v>10</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="L11" s="6"/>
       <c r="M11" s="6"/>
@@ -1283,27 +1318,35 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="E12" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="F12" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="E12" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F12" s="4" t="s">
+      <c r="G12" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="H12" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="G12" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="H12" s="3"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
+      <c r="I12" s="2">
+        <v>30</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>55</v>
+      </c>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
     </row>
@@ -1312,27 +1355,35 @@
         <v>12</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="D13" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="I13" s="6">
+        <v>30</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="K13" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="E13" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="G13" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="H13" s="7"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
       <c r="L13" s="6"/>
       <c r="M13" s="6"/>
     </row>
@@ -1341,27 +1392,35 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>58</v>
+        <v>28</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G14" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H14" s="3"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
+      <c r="H14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="I14" s="2">
+        <v>10</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>61</v>
+      </c>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
     </row>
@@ -1370,19 +1429,19 @@
         <v>14</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="G15" s="9" t="s">
         <v>18</v>
@@ -1399,38 +1458,28 @@
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H16" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I16" s="2">
-        <v>10</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="L16" s="12">
-        <v>46233</v>
-      </c>
+      <c r="H16" s="3"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
       <c r="M16" s="2"/>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
@@ -1438,19 +1487,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>16</v>
+        <v>68</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="G17" s="9" t="s">
         <v>18</v>
@@ -1467,32 +1516,26 @@
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>51</v>
+        <v>72</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>68</v>
+        <v>28</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="G18" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H18" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I18" s="2">
-        <v>20</v>
-      </c>
-      <c r="J18" s="12">
-        <v>46232</v>
-      </c>
+      <c r="H18" s="3"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
@@ -1502,19 +1545,19 @@
         <v>18</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>73</v>
+        <v>28</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="G19" s="9" t="s">
         <v>18</v>
@@ -1531,19 +1574,19 @@
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G20" s="5" t="s">
         <v>18</v>
@@ -1560,35 +1603,27 @@
         <v>20</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G21" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="H21" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I21" s="6">
-        <v>5</v>
-      </c>
-      <c r="J21" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="K21" s="6" t="s">
-        <v>80</v>
-      </c>
+      <c r="H21" s="7"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="6"/>
+      <c r="K21" s="6"/>
       <c r="L21" s="6"/>
       <c r="M21" s="6"/>
     </row>
@@ -1597,35 +1632,27 @@
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G22" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H22" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I22" s="2">
-        <v>10</v>
-      </c>
-      <c r="J22" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="K22" s="2" t="s">
-        <v>83</v>
-      </c>
+      <c r="H22" s="3"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
     </row>
@@ -1634,19 +1661,19 @@
         <v>22</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G23" s="9" t="s">
         <v>18</v>
@@ -1663,19 +1690,19 @@
         <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G24" s="5" t="s">
         <v>18</v>
@@ -1692,27 +1719,35 @@
         <v>24</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G25" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="H25" s="7"/>
-      <c r="I25" s="6"/>
-      <c r="J25" s="6"/>
-      <c r="K25" s="6"/>
+      <c r="H25" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="I25" s="6">
+        <v>10</v>
+      </c>
+      <c r="J25" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>47</v>
+      </c>
       <c r="L25" s="6"/>
       <c r="M25" s="6"/>
     </row>
@@ -1721,19 +1756,19 @@
         <v>25</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>85</v>
+        <v>28</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G26" s="5" t="s">
         <v>18</v>
@@ -1750,19 +1785,19 @@
         <v>26</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>94</v>
+        <v>72</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>95</v>
+        <v>73</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G27" s="9" t="s">
         <v>18</v>
@@ -1779,19 +1814,19 @@
         <v>27</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="G28" s="5" t="s">
         <v>18</v>
@@ -1808,19 +1843,19 @@
         <v>28</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="G29" s="9" t="s">
         <v>18</v>
@@ -1837,34 +1872,34 @@
         <v>29</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="G30" s="5" t="s">
         <v>18</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="I30" s="2">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>50</v>
+        <v>110</v>
       </c>
       <c r="L30" s="2"/>
       <c r="M30" s="2"/>
@@ -1874,34 +1909,34 @@
         <v>30</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="G31" s="9" t="s">
         <v>18</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="I31" s="6">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="J31" s="6" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="K31" s="6" t="s">
-        <v>83</v>
+        <v>113</v>
       </c>
       <c r="L31" s="6"/>
       <c r="M31" s="6"/>
@@ -1911,19 +1946,19 @@
         <v>31</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="G32" s="5" t="s">
         <v>18</v>
@@ -1940,19 +1975,19 @@
         <v>32</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D33" s="7" t="s">
         <v>115</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="G33" s="9" t="s">
         <v>18</v>
@@ -1969,19 +2004,19 @@
         <v>33</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="G34" s="5" t="s">
         <v>18</v>
@@ -1998,22 +2033,22 @@
         <v>34</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="G35" s="11" t="s">
-        <v>39</v>
+        <v>123</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>18</v>
       </c>
       <c r="H35" s="7"/>
       <c r="I35" s="6"/>
@@ -2027,22 +2062,22 @@
         <v>35</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="G36" s="10" t="s">
-        <v>39</v>
+        <v>128</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="H36" s="3"/>
       <c r="I36" s="2"/>
@@ -2056,19 +2091,19 @@
         <v>36</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="G37" s="9" t="s">
         <v>18</v>
@@ -2085,22 +2120,22 @@
         <v>37</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="G38" s="10" t="s">
-        <v>39</v>
+        <v>133</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="H38" s="3"/>
       <c r="I38" s="2"/>
@@ -2109,8 +2144,314 @@
       <c r="L38" s="2"/>
       <c r="M38" s="2"/>
     </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A39" s="6">
+        <v>38</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="F39" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="G39" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H39" s="7"/>
+      <c r="I39" s="6"/>
+      <c r="J39" s="6"/>
+      <c r="K39" s="6"/>
+      <c r="L39" s="6"/>
+      <c r="M39" s="6"/>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A40" s="2">
+        <v>39</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="G40" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I40" s="2">
+        <v>20</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="L40" s="2"/>
+      <c r="M40" s="2"/>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A41" s="6">
+        <v>40</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="G41" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H41" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="I41" s="6">
+        <v>40</v>
+      </c>
+      <c r="J41" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="K41" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="L41" s="6"/>
+      <c r="M41" s="6"/>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A42" s="2">
+        <v>41</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="G42" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H42" s="3"/>
+      <c r="I42" s="2"/>
+      <c r="J42" s="2"/>
+      <c r="K42" s="2"/>
+      <c r="L42" s="2"/>
+      <c r="M42" s="2"/>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A43" s="6">
+        <v>42</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="F43" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="G43" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H43" s="7"/>
+      <c r="I43" s="6"/>
+      <c r="J43" s="6"/>
+      <c r="K43" s="6"/>
+      <c r="L43" s="6"/>
+      <c r="M43" s="6"/>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A44" s="2">
+        <v>43</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H44" s="3"/>
+      <c r="I44" s="2"/>
+      <c r="J44" s="2"/>
+      <c r="K44" s="2"/>
+      <c r="L44" s="2"/>
+      <c r="M44" s="2"/>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A45" s="6">
+        <v>44</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="F45" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="G45" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="H45" s="7"/>
+      <c r="I45" s="6"/>
+      <c r="J45" s="6"/>
+      <c r="K45" s="6"/>
+      <c r="L45" s="6"/>
+      <c r="M45" s="6"/>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A46" s="2">
+        <v>45</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="G46" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="H46" s="3"/>
+      <c r="I46" s="2"/>
+      <c r="J46" s="2"/>
+      <c r="K46" s="2"/>
+      <c r="L46" s="2"/>
+      <c r="M46" s="2"/>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A47" s="6">
+        <v>46</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="F47" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="G47" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H47" s="7"/>
+      <c r="I47" s="6"/>
+      <c r="J47" s="6"/>
+      <c r="K47" s="6"/>
+      <c r="L47" s="6"/>
+      <c r="M47" s="6"/>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A48" s="2">
+        <v>47</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="G48" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="H48" s="3"/>
+      <c r="I48" s="2"/>
+      <c r="J48" s="2"/>
+      <c r="K48" s="2"/>
+      <c r="L48" s="2"/>
+      <c r="M48" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M38" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:M48" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="F3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
@@ -2149,6 +2490,16 @@
     <hyperlink ref="F36" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
     <hyperlink ref="F37" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
     <hyperlink ref="F38" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="F39" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="F40" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="F41" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="F42" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="F43" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="F44" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="F45" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="F46" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="F47" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="F48" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Solve LeetCode 2469: Convert the Temperature in Java
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_2B59E58F1BF641346044C83044E160314FECB551" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49ABCD62-9AB0-4139-B14B-76926B7BB018}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="DSA Tracker" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DSA Tracker'!$A$1:$M$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DSA Tracker'!$A$1:$L$48</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="165">
   <si>
     <t>No.</t>
   </si>
@@ -49,9 +49,6 @@
     <t>Solved Alone?</t>
   </si>
   <si>
-    <t>Time Taken (mins)</t>
-  </si>
-  <si>
     <t>Date Solved</t>
   </si>
   <si>
@@ -82,6 +79,15 @@
     <t>Easy</t>
   </si>
   <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>31-07-2026</t>
+  </si>
+  <si>
+    <t>01-08-2026</t>
+  </si>
+  <si>
     <t>Basic Math Formulas</t>
   </si>
   <si>
@@ -115,6 +121,12 @@
     <t>https://leetcode.com/problems/subtract-the-product-and-sum-of-digits-of-an-integer/</t>
   </si>
   <si>
+    <t>28-07-2026</t>
+  </si>
+  <si>
+    <t>29-07-2026</t>
+  </si>
+  <si>
     <t>Number of Steps to Reduce a Number to Zero</t>
   </si>
   <si>
@@ -139,9 +151,6 @@
     <t>https://leetcode.com/problems/fibonacci-number/</t>
   </si>
   <si>
-    <t>YES</t>
-  </si>
-  <si>
     <t>22-07-2026</t>
   </si>
   <si>
@@ -169,6 +178,9 @@
     <t>24-07-2026</t>
   </si>
   <si>
+    <t>30-07-2026</t>
+  </si>
+  <si>
     <t>Reverse Integer</t>
   </si>
   <si>
@@ -187,184 +199,178 @@
     <t>https://leetcode.com/problems/count-primes/</t>
   </si>
   <si>
-    <t>NO</t>
+    <t>Base 7</t>
+  </si>
+  <si>
+    <t>Base Conversion</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/base-7/</t>
   </si>
   <si>
     <t>25-07-2026</t>
   </si>
   <si>
-    <t>Base 7</t>
-  </si>
-  <si>
-    <t>Base Conversion</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/base-7/</t>
-  </si>
-  <si>
     <t>Add Binary</t>
   </si>
   <si>
     <t>https://leetcode.com/problems/add-binary/</t>
   </si>
   <si>
+    <t>Strings</t>
+  </si>
+  <si>
+    <t>String Manipulation</t>
+  </si>
+  <si>
+    <t>Score of a String</t>
+  </si>
+  <si>
+    <t>ASCII Values</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/score-of-a-string/</t>
+  </si>
+  <si>
+    <t>Defanging an IP Address</t>
+  </si>
+  <si>
+    <t>String Replace</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/defanging-an-ip-address/</t>
+  </si>
+  <si>
+    <t>Goal Parser Interpretation</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/goal-parser-interpretation/</t>
+  </si>
+  <si>
+    <t>Arrays</t>
+  </si>
+  <si>
+    <t>Basic Array Traversal</t>
+  </si>
+  <si>
+    <t>Build Array from Permutation</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/build-array-from-permutation/</t>
+  </si>
+  <si>
+    <t>Concatenation of Array</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/concatenation-of-array/</t>
+  </si>
+  <si>
+    <t>Shuffle the Array</t>
+  </si>
+  <si>
+    <t>Array Indexing</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/shuffle-the-array/</t>
+  </si>
+  <si>
+    <t>Kids With the Greatest Number of Candies</t>
+  </si>
+  <si>
+    <t>Find Max &amp; Loop</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/kids-with-the-greatest-number-of-candies/</t>
+  </si>
+  <si>
+    <t>Richest Customer Wealth</t>
+  </si>
+  <si>
+    <t>2D Array Traversal</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/richest-customer-wealth/</t>
+  </si>
+  <si>
+    <t>Running Sum of 1d Array</t>
+  </si>
+  <si>
+    <t>Prefix Sum</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/running-sum-of-1d-array/</t>
+  </si>
+  <si>
+    <t>Find Pivot Index</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/find-pivot-index/</t>
+  </si>
+  <si>
+    <t>Missing Number</t>
+  </si>
+  <si>
+    <t>Gauss Formula or XOR</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/missing-number/</t>
+  </si>
+  <si>
+    <t>Add to Array-Form of Integer</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/add-to-array-form-of-integer/</t>
+  </si>
+  <si>
+    <t>Best Time to Buy and Sell Stock</t>
+  </si>
+  <si>
+    <t>Track Min Value</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock/</t>
+  </si>
+  <si>
+    <t>Arrays - Two Pointers</t>
+  </si>
+  <si>
+    <t>Two Pointers Technique</t>
+  </si>
+  <si>
+    <t>Reverse String</t>
+  </si>
+  <si>
+    <t>Two Pointers (Left/Right)</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/reverse-string/</t>
+  </si>
+  <si>
+    <t>Remove Element</t>
+  </si>
+  <si>
+    <t>Two Pointers (Slow/Fast)</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/remove-element/</t>
+  </si>
+  <si>
+    <t>Move Zeroes</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/move-zeroes/</t>
+  </si>
+  <si>
     <t>26-07-2026</t>
   </si>
   <si>
-    <t>Strings</t>
-  </si>
-  <si>
-    <t>String Manipulation</t>
-  </si>
-  <si>
-    <t>Score of a String</t>
-  </si>
-  <si>
-    <t>ASCII Values</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/score-of-a-string/</t>
-  </si>
-  <si>
-    <t>Defanging an IP Address</t>
-  </si>
-  <si>
-    <t>String Replace</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/defanging-an-ip-address/</t>
-  </si>
-  <si>
-    <t>Goal Parser Interpretation</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/goal-parser-interpretation/</t>
-  </si>
-  <si>
-    <t>Arrays</t>
-  </si>
-  <si>
-    <t>Basic Array Traversal</t>
-  </si>
-  <si>
-    <t>Build Array from Permutation</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/build-array-from-permutation/</t>
-  </si>
-  <si>
-    <t>Concatenation of Array</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/concatenation-of-array/</t>
-  </si>
-  <si>
-    <t>Shuffle the Array</t>
-  </si>
-  <si>
-    <t>Array Indexing</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/shuffle-the-array/</t>
-  </si>
-  <si>
-    <t>Kids With the Greatest Number of Candies</t>
-  </si>
-  <si>
-    <t>Find Max &amp; Loop</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/kids-with-the-greatest-number-of-candies/</t>
-  </si>
-  <si>
-    <t>Richest Customer Wealth</t>
-  </si>
-  <si>
-    <t>2D Array Traversal</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/richest-customer-wealth/</t>
-  </si>
-  <si>
-    <t>Running Sum of 1d Array</t>
-  </si>
-  <si>
-    <t>Prefix Sum</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/running-sum-of-1d-array/</t>
-  </si>
-  <si>
-    <t>Find Pivot Index</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/find-pivot-index/</t>
-  </si>
-  <si>
-    <t>Missing Number</t>
-  </si>
-  <si>
-    <t>Gauss Formula or XOR</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/missing-number/</t>
-  </si>
-  <si>
-    <t>Add to Array-Form of Integer</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/add-to-array-form-of-integer/</t>
-  </si>
-  <si>
-    <t>Best Time to Buy and Sell Stock</t>
-  </si>
-  <si>
-    <t>Track Min Value</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock/</t>
-  </si>
-  <si>
-    <t>Arrays - Two Pointers</t>
-  </si>
-  <si>
-    <t>Two Pointers Technique</t>
-  </si>
-  <si>
-    <t>Reverse String</t>
-  </si>
-  <si>
-    <t>Two Pointers (Left/Right)</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/reverse-string/</t>
-  </si>
-  <si>
-    <t>Remove Element</t>
-  </si>
-  <si>
-    <t>Two Pointers (Slow/Fast)</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/remove-element/</t>
-  </si>
-  <si>
-    <t>Move Zeroes</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/move-zeroes/</t>
+    <t>Squares of a Sorted Array</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/squares-of-a-sorted-array/</t>
   </si>
   <si>
     <t>27-07-2026</t>
-  </si>
-  <si>
-    <t>Squares of a Sorted Array</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/squares-of-a-sorted-array/</t>
-  </si>
-  <si>
-    <t>28-07-2026</t>
   </si>
   <si>
     <t>Binary Search &amp; Sort</t>
@@ -598,7 +604,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -631,6 +637,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -935,7 +944,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M48"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -944,13 +954,11 @@
     <col min="4" max="4" width="45" customWidth="1"/>
     <col min="5" max="5" width="25" customWidth="1"/>
     <col min="6" max="6" width="45" customWidth="1"/>
-    <col min="7" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="15" customWidth="1"/>
-    <col min="11" max="14" width="18" customWidth="1"/>
+    <col min="7" max="9" width="15" customWidth="1"/>
+    <col min="10" max="13" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -987,1471 +995,1461 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="4" t="s">
-        <v>17</v>
-      </c>
       <c r="G2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="3"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
+      <c r="I2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>20</v>
+      </c>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6">
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H3" s="7"/>
       <c r="I3" s="6"/>
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
       <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H4" s="3"/>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="6">
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G5" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="7"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
+      <c r="I5" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>33</v>
+      </c>
       <c r="K5" s="6"/>
       <c r="L5" s="6"/>
-      <c r="M5" s="6"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>28</v>
-      </c>
       <c r="F6" s="4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="G6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="3"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
+      <c r="I6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6">
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D7" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I7" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="J7" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="H7" s="7"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="I8" s="2">
-        <v>5</v>
+      <c r="I8" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="6">
         <v>8</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E9" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I9" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="J9" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="G9" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="I9" s="6">
-        <v>5</v>
-      </c>
-      <c r="J9" s="6" t="s">
-        <v>39</v>
-      </c>
       <c r="K9" s="6" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="G10" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="H10" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="I10" s="2">
-        <v>10</v>
+      <c r="I10" s="2" t="s">
+        <v>43</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="6">
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D11" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="7" t="s">
-        <v>45</v>
-      </c>
       <c r="F11" s="8" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G11" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="J11" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="H11" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="I11" s="6">
-        <v>10</v>
-      </c>
-      <c r="J11" s="6" t="s">
-        <v>40</v>
-      </c>
       <c r="K11" s="6" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D12" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="K12" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E12" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="G12" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="I12" s="2">
-        <v>30</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>55</v>
-      </c>
       <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="6">
         <v>12</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G13" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H13" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="H13" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="I13" s="6">
-        <v>30</v>
+      <c r="I13" s="6" t="s">
+        <v>50</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G14" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="H14" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="I14" s="2">
-        <v>10</v>
+      <c r="I14" s="2" t="s">
+        <v>50</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="6">
         <v>14</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H15" s="7"/>
       <c r="I15" s="6"/>
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
       <c r="L15" s="6"/>
-      <c r="M15" s="6"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H16" s="3"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="6">
         <v>16</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D17" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E17" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="E17" s="7" t="s">
-        <v>68</v>
-      </c>
       <c r="F17" s="8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H17" s="7"/>
       <c r="I17" s="6"/>
       <c r="J17" s="6"/>
       <c r="K17" s="6"/>
       <c r="L17" s="6"/>
-      <c r="M17" s="6"/>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H18" s="3"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
-      <c r="M18" s="2"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
         <v>18</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G19" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H19" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="H19" s="7"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="6"/>
+      <c r="I19" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>19</v>
+      </c>
       <c r="K19" s="6"/>
       <c r="L19" s="6"/>
-      <c r="M19" s="6"/>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H20" s="3"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
-      <c r="M20" s="2"/>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6">
         <v>20</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H21" s="7"/>
       <c r="I21" s="6"/>
       <c r="J21" s="6"/>
       <c r="K21" s="6"/>
       <c r="L21" s="6"/>
-      <c r="M21" s="6"/>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H22" s="3"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="6">
         <v>22</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H23" s="7"/>
       <c r="I23" s="6"/>
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
       <c r="L23" s="6"/>
-      <c r="M23" s="6"/>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D24" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="E24" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="E24" s="3" t="s">
-        <v>88</v>
-      </c>
       <c r="F24" s="4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H24" s="3"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6">
         <v>24</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G25" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H25" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="H25" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="I25" s="6">
-        <v>10</v>
+      <c r="I25" s="6" t="s">
+        <v>42</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="L25" s="6"/>
-      <c r="M25" s="6"/>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>25</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H26" s="3"/>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
-      <c r="M26" s="2"/>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="6">
         <v>26</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G27" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H27" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="H27" s="7"/>
-      <c r="I27" s="6"/>
-      <c r="J27" s="6"/>
+      <c r="I27" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J27" s="6" t="s">
+        <v>51</v>
+      </c>
       <c r="K27" s="6"/>
       <c r="L27" s="6"/>
-      <c r="M27" s="6"/>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="28" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>27</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H28" s="3"/>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
-      <c r="M28" s="2"/>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="29" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="6">
         <v>28</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H29" s="7"/>
       <c r="I29" s="6"/>
       <c r="J29" s="6"/>
       <c r="K29" s="6"/>
       <c r="L29" s="6"/>
-      <c r="M29" s="6"/>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="30" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>29</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D30" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E30" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="E30" s="3" t="s">
-        <v>106</v>
-      </c>
       <c r="F30" s="4" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="G30" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H30" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="H30" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="I30" s="2">
-        <v>5</v>
+      <c r="I30" s="2" t="s">
+        <v>61</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>61</v>
+        <v>112</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>110</v>
+        <v>20</v>
       </c>
       <c r="L30" s="2"/>
-      <c r="M30" s="2"/>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" s="6">
         <v>30</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F31" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I31" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="G31" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="H31" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="I31" s="6">
-        <v>10</v>
-      </c>
       <c r="J31" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="K31" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
+      </c>
+      <c r="K31" s="12">
+        <v>46236</v>
       </c>
       <c r="L31" s="6"/>
-      <c r="M31" s="6"/>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="32" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
         <v>31</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H32" s="3"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
-      <c r="M32" s="2"/>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="33" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="6">
         <v>32</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H33" s="7"/>
       <c r="I33" s="6"/>
       <c r="J33" s="6"/>
       <c r="K33" s="6"/>
       <c r="L33" s="6"/>
-      <c r="M33" s="6"/>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="34" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
         <v>33</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H34" s="3"/>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
       <c r="L34" s="2"/>
-      <c r="M34" s="2"/>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="35" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="6">
         <v>34</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H35" s="7"/>
       <c r="I35" s="6"/>
       <c r="J35" s="6"/>
       <c r="K35" s="6"/>
       <c r="L35" s="6"/>
-      <c r="M35" s="6"/>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="36" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
         <v>35</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H36" s="3"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
-      <c r="M36" s="2"/>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="37" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="6">
         <v>36</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="G37" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H37" s="7"/>
       <c r="I37" s="6"/>
       <c r="J37" s="6"/>
       <c r="K37" s="6"/>
       <c r="L37" s="6"/>
-      <c r="M37" s="6"/>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="38" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
         <v>37</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H38" s="3"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
       <c r="L38" s="2"/>
-      <c r="M38" s="2"/>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="39" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="6">
         <v>38</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G39" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H39" s="7"/>
       <c r="I39" s="6"/>
       <c r="J39" s="6"/>
       <c r="K39" s="6"/>
       <c r="L39" s="6"/>
-      <c r="M39" s="6"/>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="40" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
         <v>39</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G40" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H40" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="H40" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="I40" s="2">
+      <c r="I40" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="K40" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="J40" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="K40" s="2" t="s">
-        <v>61</v>
-      </c>
       <c r="L40" s="2"/>
-      <c r="M40" s="2"/>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="41" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="6">
         <v>40</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G41" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H41" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="H41" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="I41" s="6">
-        <v>40</v>
+      <c r="I41" s="6" t="s">
+        <v>115</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="K41" s="6" t="s">
-        <v>113</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="K41" s="6"/>
       <c r="L41" s="6"/>
-      <c r="M41" s="6"/>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="42" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
         <v>41</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H42" s="3"/>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
       <c r="L42" s="2"/>
-      <c r="M42" s="2"/>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="43" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="6">
         <v>42</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G43" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H43" s="7"/>
       <c r="I43" s="6"/>
       <c r="J43" s="6"/>
       <c r="K43" s="6"/>
       <c r="L43" s="6"/>
-      <c r="M43" s="6"/>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="44" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
         <v>43</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H44" s="3"/>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
-      <c r="M44" s="2"/>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="45" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="6">
         <v>44</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="G45" s="10" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="H45" s="7"/>
       <c r="I45" s="6"/>
       <c r="J45" s="6"/>
       <c r="K45" s="6"/>
       <c r="L45" s="6"/>
-      <c r="M45" s="6"/>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="46" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
         <v>45</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="G46" s="11" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="H46" s="3"/>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
       <c r="L46" s="2"/>
-      <c r="M46" s="2"/>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="47" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="6">
         <v>46</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F47" s="8" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H47" s="7"/>
       <c r="I47" s="6"/>
       <c r="J47" s="6"/>
       <c r="K47" s="6"/>
       <c r="L47" s="6"/>
-      <c r="M47" s="6"/>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+    </row>
+    <row r="48" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
         <v>47</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D48" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E48" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="E48" s="3" t="s">
-        <v>159</v>
-      </c>
       <c r="F48" s="4" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="G48" s="11" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="H48" s="3"/>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
       <c r="L48" s="2"/>
-      <c r="M48" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M48" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:L48" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="8">
+      <filters>
+        <filter val="26-07-2026"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="F3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>

</xml_diff>

<commit_message>
Solve LeetCode 2413: Smallest Even Multiple in Java
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49ABCD62-9AB0-4139-B14B-76926B7BB018}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F48E159F-041A-4259-9AD1-E4216ACF7C58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="166">
   <si>
     <t>No.</t>
   </si>
@@ -518,6 +518,9 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/daily-temperatures/</t>
+  </si>
+  <si>
+    <t>NA</t>
   </si>
 </sst>
 </file>
@@ -944,7 +947,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:L48"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -996,7 +998,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1025,12 +1027,16 @@
         <v>19</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-    </row>
-    <row r="3" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+        <v>165</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -1052,13 +1058,23 @@
       <c r="G3" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="7"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-    </row>
-    <row r="4" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H3" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="12">
+        <v>46235</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1086,7 +1102,7 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -1120,7 +1136,7 @@
       <c r="K5" s="6"/>
       <c r="L5" s="6"/>
     </row>
-    <row r="6" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1154,7 +1170,7 @@
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
     </row>
-    <row r="7" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="6">
         <v>6</v>
       </c>
@@ -1188,7 +1204,7 @@
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
     </row>
-    <row r="8" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1224,7 +1240,7 @@
       </c>
       <c r="L8" s="2"/>
     </row>
-    <row r="9" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -1260,7 +1276,7 @@
       </c>
       <c r="L9" s="6"/>
     </row>
-    <row r="10" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1296,7 +1312,7 @@
       </c>
       <c r="L10" s="2"/>
     </row>
-    <row r="11" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -1332,7 +1348,7 @@
       </c>
       <c r="L11" s="6"/>
     </row>
-    <row r="12" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1368,7 +1384,7 @@
       </c>
       <c r="L12" s="2"/>
     </row>
-    <row r="13" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -1404,7 +1420,7 @@
       </c>
       <c r="L13" s="6"/>
     </row>
-    <row r="14" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1440,7 +1456,7 @@
       </c>
       <c r="L14" s="2"/>
     </row>
-    <row r="15" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -1468,7 +1484,7 @@
       <c r="K15" s="6"/>
       <c r="L15" s="6"/>
     </row>
-    <row r="16" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1496,7 +1512,7 @@
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
     </row>
-    <row r="17" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -1524,7 +1540,7 @@
       <c r="K17" s="6"/>
       <c r="L17" s="6"/>
     </row>
-    <row r="18" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1552,7 +1568,7 @@
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
     </row>
-    <row r="19" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -1586,7 +1602,7 @@
       <c r="K19" s="6"/>
       <c r="L19" s="6"/>
     </row>
-    <row r="20" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1614,7 +1630,7 @@
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
     </row>
-    <row r="21" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -1642,7 +1658,7 @@
       <c r="K21" s="6"/>
       <c r="L21" s="6"/>
     </row>
-    <row r="22" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1670,7 +1686,7 @@
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
     </row>
-    <row r="23" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -1698,7 +1714,7 @@
       <c r="K23" s="6"/>
       <c r="L23" s="6"/>
     </row>
-    <row r="24" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1726,7 +1742,7 @@
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
     </row>
-    <row r="25" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -1762,7 +1778,7 @@
       </c>
       <c r="L25" s="6"/>
     </row>
-    <row r="26" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -1790,7 +1806,7 @@
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
     </row>
-    <row r="27" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -1824,7 +1840,7 @@
       <c r="K27" s="6"/>
       <c r="L27" s="6"/>
     </row>
-    <row r="28" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -1852,7 +1868,7 @@
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
     </row>
-    <row r="29" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -1880,7 +1896,7 @@
       <c r="K29" s="6"/>
       <c r="L29" s="6"/>
     </row>
-    <row r="30" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -1952,7 +1968,7 @@
       </c>
       <c r="L31" s="6"/>
     </row>
-    <row r="32" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -1980,7 +1996,7 @@
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
     </row>
-    <row r="33" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33" s="6">
         <v>32</v>
       </c>
@@ -2008,7 +2024,7 @@
       <c r="K33" s="6"/>
       <c r="L33" s="6"/>
     </row>
-    <row r="34" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -2036,7 +2052,7 @@
       <c r="K34" s="2"/>
       <c r="L34" s="2"/>
     </row>
-    <row r="35" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" s="6">
         <v>34</v>
       </c>
@@ -2064,7 +2080,7 @@
       <c r="K35" s="6"/>
       <c r="L35" s="6"/>
     </row>
-    <row r="36" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -2092,7 +2108,7 @@
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
     </row>
-    <row r="37" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37" s="6">
         <v>36</v>
       </c>
@@ -2120,7 +2136,7 @@
       <c r="K37" s="6"/>
       <c r="L37" s="6"/>
     </row>
-    <row r="38" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -2148,7 +2164,7 @@
       <c r="K38" s="2"/>
       <c r="L38" s="2"/>
     </row>
-    <row r="39" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39" s="6">
         <v>38</v>
       </c>
@@ -2176,7 +2192,7 @@
       <c r="K39" s="6"/>
       <c r="L39" s="6"/>
     </row>
-    <row r="40" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -2212,7 +2228,7 @@
       </c>
       <c r="L40" s="2"/>
     </row>
-    <row r="41" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A41" s="6">
         <v>40</v>
       </c>
@@ -2246,7 +2262,7 @@
       <c r="K41" s="6"/>
       <c r="L41" s="6"/>
     </row>
-    <row r="42" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -2274,7 +2290,7 @@
       <c r="K42" s="2"/>
       <c r="L42" s="2"/>
     </row>
-    <row r="43" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A43" s="6">
         <v>42</v>
       </c>
@@ -2302,7 +2318,7 @@
       <c r="K43" s="6"/>
       <c r="L43" s="6"/>
     </row>
-    <row r="44" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -2330,7 +2346,7 @@
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
     </row>
-    <row r="45" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A45" s="6">
         <v>44</v>
       </c>
@@ -2358,7 +2374,7 @@
       <c r="K45" s="6"/>
       <c r="L45" s="6"/>
     </row>
-    <row r="46" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -2386,7 +2402,7 @@
       <c r="K46" s="2"/>
       <c r="L46" s="2"/>
     </row>
-    <row r="47" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A47" s="6">
         <v>46</v>
       </c>
@@ -2414,7 +2430,7 @@
       <c r="K47" s="6"/>
       <c r="L47" s="6"/>
     </row>
-    <row r="48" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -2443,13 +2459,7 @@
       <c r="L48" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L48" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <filterColumn colId="8">
-      <filters>
-        <filter val="26-07-2026"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:L48" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="F3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>

</xml_diff>

<commit_message>
Solve LeetCode 1920: Build Array from Permutation in Java
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F48E159F-041A-4259-9AD1-E4216ACF7C58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51522A20-84A9-442B-A951-699356C4349D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="166">
   <si>
     <t>No.</t>
   </si>
@@ -607,7 +607,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -643,6 +643,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1096,11 +1099,21 @@
       <c r="G4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H4" s="3"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
+      <c r="H4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="13">
+        <v>46235</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="6">

</xml_diff>

<commit_message>
Solve LeetCode 1470: Shuffle the Array using alternate indexing
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51522A20-84A9-442B-A951-699356C4349D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AA6BA56-8A6F-46A8-AC9E-C49AEFA179A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="166">
   <si>
     <t>No.</t>
   </si>
@@ -1575,11 +1575,21 @@
       <c r="G18" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H18" s="3"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
-      <c r="L18" s="2"/>
+      <c r="H18" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I18" s="13">
+        <v>46235</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="6">

</xml_diff>

<commit_message>
Solve LeetCode 1672: Richest Customer Wealth
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AA6BA56-8A6F-46A8-AC9E-C49AEFA179A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9674B1FB-9501-47C4-8456-0B98A90245A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="167">
   <si>
     <t>No.</t>
   </si>
@@ -521,6 +521,9 @@
   </si>
   <si>
     <t>NA</t>
+  </si>
+  <si>
+    <t>NO</t>
   </si>
 </sst>
 </file>
@@ -1647,8 +1650,12 @@
       <c r="G20" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H20" s="3"/>
-      <c r="I20" s="2"/>
+      <c r="H20" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="I20" s="13">
+        <v>46235</v>
+      </c>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>

</xml_diff>

<commit_message>
Solve LeetCode 1480: Running Sum of 1d Array
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9674B1FB-9501-47C4-8456-0B98A90245A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D922DCEB-291D-4019-9A72-E73E2E44BF0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="167">
   <si>
     <t>No.</t>
   </si>
@@ -1710,8 +1710,12 @@
       <c r="G22" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H22" s="3"/>
-      <c r="I22" s="2"/>
+      <c r="H22" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="I22" s="13">
+        <v>46236</v>
+      </c>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>

</xml_diff>

<commit_message>
Solve LeetCode 724: Find Pivot Index using prefix sum
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D922DCEB-291D-4019-9A72-E73E2E44BF0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49FB62BB-2058-4345-A8F1-7BF923D4BF4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4116" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DSA Tracker" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="168">
   <si>
     <t>No.</t>
   </si>
@@ -524,6 +524,9 @@
   </si>
   <si>
     <t>NO</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> .</t>
   </si>
 </sst>
 </file>
@@ -953,7 +956,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -1149,7 +1152,9 @@
       <c r="J5" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="K5" s="6"/>
+      <c r="K5" s="12">
+        <v>46206</v>
+      </c>
       <c r="L5" s="6"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
@@ -1183,7 +1188,9 @@
       <c r="J6" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K6" s="2"/>
+      <c r="K6" s="13">
+        <v>46206</v>
+      </c>
       <c r="L6" s="2"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -1217,7 +1224,9 @@
       <c r="J7" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="K7" s="6"/>
+      <c r="K7" s="12">
+        <v>46206</v>
+      </c>
       <c r="L7" s="6"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
@@ -1742,8 +1751,12 @@
       <c r="G23" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H23" s="7"/>
-      <c r="I23" s="6"/>
+      <c r="H23" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="I23" s="12">
+        <v>46236</v>
+      </c>
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
       <c r="L23" s="6"/>
@@ -2293,7 +2306,9 @@
       <c r="J41" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="K41" s="6"/>
+      <c r="K41" s="12">
+        <v>46237</v>
+      </c>
       <c r="L41" s="6"/>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.3">
@@ -2491,6 +2506,11 @@
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
       <c r="L48" s="2"/>
+    </row>
+    <row r="51" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K51" t="s">
+        <v>167</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L48" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>

<commit_message>
Solve LeetCode 1108: Defanging an IP Address
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49FB62BB-2058-4345-A8F1-7BF923D4BF4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2182B624-1BE9-4F6E-B644-D3F86CDF0B0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4116" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DSA Tracker" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="168">
   <si>
     <t>No.</t>
   </si>
@@ -1783,8 +1783,12 @@
       <c r="G24" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H24" s="3"/>
-      <c r="I24" s="2"/>
+      <c r="H24" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="I24" s="13">
+        <v>46237</v>
+      </c>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>

</xml_diff>

<commit_message>
Solve LeetCode 3110: Score of a String using adjacent ASCII differences
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2182B624-1BE9-4F6E-B644-D3F86CDF0B0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C764F63D-A63A-4D69-A0B5-FF4C4AB65F96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="168">
   <si>
     <t>No.</t>
   </si>
@@ -1531,8 +1531,12 @@
       <c r="G16" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H16" s="3"/>
-      <c r="I16" s="2"/>
+      <c r="H16" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I16" s="13">
+        <v>46238</v>
+      </c>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>

</xml_diff>

<commit_message>
Solve LeetCode 1678 Goal Parser Interpretation using StringBuilder
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C764F63D-A63A-4D69-A0B5-FF4C4AB65F96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4DF0ED4-3E9D-4F45-A0A9-AE053D874A5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="168">
   <si>
     <t>No.</t>
   </si>
@@ -1503,8 +1503,12 @@
       <c r="G15" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H15" s="7"/>
-      <c r="I15" s="6"/>
+      <c r="H15" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I15" s="12">
+        <v>46238</v>
+      </c>
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
       <c r="L15" s="6"/>
@@ -1563,8 +1567,12 @@
       <c r="G17" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H17" s="7"/>
-      <c r="I17" s="6"/>
+      <c r="H17" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I17" s="12">
+        <v>46238</v>
+      </c>
       <c r="J17" s="6"/>
       <c r="K17" s="6"/>
       <c r="L17" s="6"/>

</xml_diff>

<commit_message>
Solve LeetCode 35: Search Insert Position using binary search
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4DF0ED4-3E9D-4F45-A0A9-AE053D874A5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A70EDE4C-8035-4204-A0CF-714BCA39FB27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="168">
   <si>
     <t>No.</t>
   </si>
@@ -960,7 +960,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="2" max="2" width="20.21875" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="45" customWidth="1"/>
     <col min="5" max="5" width="25" customWidth="1"/>
@@ -2081,8 +2081,12 @@
       <c r="G33" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H33" s="7"/>
-      <c r="I33" s="6"/>
+      <c r="H33" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I33" s="12">
+        <v>46238</v>
+      </c>
       <c r="J33" s="6"/>
       <c r="K33" s="6"/>
       <c r="L33" s="6"/>

</xml_diff>

<commit_message>
Solve LeetCode 20: Valid Parentheses using stack
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A70EDE4C-8035-4204-A0CF-714BCA39FB27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4BB441B-683A-4753-98A4-B5B46081328E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="168">
   <si>
     <t>No.</t>
   </si>
@@ -2113,8 +2113,12 @@
       <c r="G34" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H34" s="3"/>
-      <c r="I34" s="2"/>
+      <c r="H34" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I34" s="13">
+        <v>46238</v>
+      </c>
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
       <c r="L34" s="2"/>

</xml_diff>

<commit_message>
Solve LeetCode 26: Remove Duplicates from Sorted Array using two pointers
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4BB441B-683A-4753-98A4-B5B46081328E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37F6DCD4-3681-47C3-93C0-4431C5D669D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="225">
   <si>
     <t>No.</t>
   </si>
@@ -64,48 +64,51 @@
     <t>Absolute Basics</t>
   </si>
   <si>
+    <t>Basic Math Formulas</t>
+  </si>
+  <si>
+    <t>Convert the Temperature</t>
+  </si>
+  <si>
+    <t>Math</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/convert-the-temperature/</t>
+  </si>
+  <si>
+    <t>Easy</t>
+  </si>
+  <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>01-08-2026</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>If/Else Statements</t>
+  </si>
+  <si>
+    <t>Smallest Even Multiple</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/smallest-even-multiple/</t>
+  </si>
+  <si>
     <t>Writing a return statement</t>
   </si>
   <si>
     <t>Add Two Integers</t>
   </si>
   <si>
-    <t>Math</t>
-  </si>
-  <si>
     <t>https://leetcode.com/problems/add-two-integers/</t>
   </si>
   <si>
-    <t>Easy</t>
-  </si>
-  <si>
-    <t>YES</t>
-  </si>
-  <si>
     <t>31-07-2026</t>
   </si>
   <si>
-    <t>01-08-2026</t>
-  </si>
-  <si>
-    <t>Basic Math Formulas</t>
-  </si>
-  <si>
-    <t>Convert the Temperature</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/convert-the-temperature/</t>
-  </si>
-  <si>
-    <t>If/Else Statements</t>
-  </si>
-  <si>
-    <t>Smallest Even Multiple</t>
-  </si>
-  <si>
-    <t>https://leetcode.com/problems/smallest-even-multiple/</t>
-  </si>
-  <si>
     <t>Math &amp; Basics</t>
   </si>
   <si>
@@ -127,6 +130,9 @@
     <t>29-07-2026</t>
   </si>
   <si>
+    <t>03-07-2026</t>
+  </si>
+  <si>
     <t>Number of Steps to Reduce a Number to Zero</t>
   </si>
   <si>
@@ -232,6 +238,9 @@
     <t>https://leetcode.com/problems/score-of-a-string/</t>
   </si>
   <si>
+    <t>04-08-2026</t>
+  </si>
+  <si>
     <t>Defanging an IP Address</t>
   </si>
   <si>
@@ -274,6 +283,9 @@
     <t>https://leetcode.com/problems/shuffle-the-array/</t>
   </si>
   <si>
+    <t>NO</t>
+  </si>
+  <si>
     <t>Kids With the Greatest Number of Candies</t>
   </si>
   <si>
@@ -292,6 +304,9 @@
     <t>https://leetcode.com/problems/richest-customer-wealth/</t>
   </si>
   <si>
+    <t>02-08-2026</t>
+  </si>
+  <si>
     <t>Running Sum of 1d Array</t>
   </si>
   <si>
@@ -307,6 +322,9 @@
     <t>https://leetcode.com/problems/find-pivot-index/</t>
   </si>
   <si>
+    <t>03-08-2026</t>
+  </si>
+  <si>
     <t>Missing Number</t>
   </si>
   <si>
@@ -331,6 +349,51 @@
     <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock/</t>
   </si>
   <si>
+    <t>Logic/Math</t>
+  </si>
+  <si>
+    <t>Find All Numbers Disappeared in an Array</t>
+  </si>
+  <si>
+    <t>Array Iteration</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/find-all-numbers-disappeared-in-an-array/</t>
+  </si>
+  <si>
+    <t>Span of Array</t>
+  </si>
+  <si>
+    <t>Find Minimum in Rotated Sorted Array</t>
+  </si>
+  <si>
+    <t>Binary Search</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/find-minimum-in-rotated-sorted-array/</t>
+  </si>
+  <si>
+    <t>Subarray</t>
+  </si>
+  <si>
+    <t>Maximum Subarray</t>
+  </si>
+  <si>
+    <t>Kadanes Algorithm</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/maximum-subarray/</t>
+  </si>
+  <si>
+    <t>Two Pointers</t>
+  </si>
+  <si>
+    <t>Remove Duplicates from Sorted Array</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/remove-duplicates-from-sorted-array/</t>
+  </si>
+  <si>
     <t>Arrays - Two Pointers</t>
   </si>
   <si>
@@ -376,9 +439,6 @@
     <t>Binary Search &amp; Sort</t>
   </si>
   <si>
-    <t>Binary Search</t>
-  </si>
-  <si>
     <t>Find Target Indices After Sorting Array</t>
   </si>
   <si>
@@ -460,9 +520,99 @@
     <t>https://leetcode.com/problems/majority-element/</t>
   </si>
   <si>
+    <t>Linked Lists</t>
+  </si>
+  <si>
+    <t>Merging</t>
+  </si>
+  <si>
+    <t>Merge Two Sorted Lists</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/merge-two-sorted-lists/</t>
+  </si>
+  <si>
+    <t>Modification</t>
+  </si>
+  <si>
+    <t>Remove Linked List Elements</t>
+  </si>
+  <si>
+    <t>Iteration</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/remove-linked-list-elements/</t>
+  </si>
+  <si>
+    <t>Remove Duplicates from Sorted List</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/remove-duplicates-from-sorted-list/</t>
+  </si>
+  <si>
+    <t>Reversal</t>
+  </si>
+  <si>
+    <t>Reverse Linked List</t>
+  </si>
+  <si>
+    <t>Iterative/Recursive</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/reverse-linked-list/</t>
+  </si>
+  <si>
+    <t>Slow/Fast Ptr</t>
+  </si>
+  <si>
+    <t>Linked List Cycle</t>
+  </si>
+  <si>
+    <t>Tortoise &amp; Hare</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/linked-list-cycle/</t>
+  </si>
+  <si>
+    <t>Middle of the Linked List</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/middle-of-the-linked-list/</t>
+  </si>
+  <si>
+    <t>Palindrome Linked List</t>
+  </si>
+  <si>
+    <t>Reversal &amp; Pointers</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/palindrome-linked-list/</t>
+  </si>
+  <si>
     <t>Stacks</t>
   </si>
   <si>
+    <t>Implementation</t>
+  </si>
+  <si>
+    <t>Implement Queue using Stacks</t>
+  </si>
+  <si>
+    <t>Two Stacks</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/implement-queue-using-stacks/</t>
+  </si>
+  <si>
+    <t>Implement Stack using Queues</t>
+  </si>
+  <si>
+    <t>Two Queues</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/implement-stack-using-queues/</t>
+  </si>
+  <si>
     <t>Stack Data Structure</t>
   </si>
   <si>
@@ -493,9 +643,6 @@
     <t>Min Stack</t>
   </si>
   <si>
-    <t>Two Stacks</t>
-  </si>
-  <si>
     <t>https://leetcode.com/problems/min-stack/</t>
   </si>
   <si>
@@ -520,20 +667,47 @@
     <t>https://leetcode.com/problems/daily-temperatures/</t>
   </si>
   <si>
-    <t>NA</t>
-  </si>
-  <si>
-    <t>NO</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> .</t>
+    <t>String Ops</t>
+  </si>
+  <si>
+    <t>Backspace String Compare</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/backspace-string-compare/</t>
+  </si>
+  <si>
+    <t>Recursion</t>
+  </si>
+  <si>
+    <t>Power of Three</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/power-of-three/</t>
+  </si>
+  <si>
+    <t>Power of Four</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/power-of-four/</t>
+  </si>
+  <si>
+    <t>Power</t>
+  </si>
+  <si>
+    <t>Pow(x, n)</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/powx-n/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
+  </numFmts>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -565,8 +739,15 @@
       <color rgb="FFE36C09"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="9" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -585,8 +766,14 @@
         <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -609,49 +796,67 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -956,7 +1161,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -1032,17 +1237,17 @@
       <c r="H2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="11" t="s">
         <v>19</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>165</v>
+        <v>20</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>165</v>
+        <v>20</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>165</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
@@ -1070,17 +1275,17 @@
       <c r="H3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="12">
-        <v>46235</v>
+      <c r="I3" s="12" t="s">
+        <v>19</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>165</v>
+        <v>20</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>165</v>
+        <v>20</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>165</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
@@ -1108,17 +1313,17 @@
       <c r="H4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I4" s="13">
-        <v>46235</v>
+      <c r="I4" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>165</v>
+        <v>20</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>165</v>
+        <v>20</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>165</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
@@ -1126,19 +1331,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>17</v>
@@ -1147,13 +1352,13 @@
         <v>18</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="K5" s="12">
-        <v>46206</v>
+        <v>34</v>
+      </c>
+      <c r="K5" s="12" t="s">
+        <v>35</v>
       </c>
       <c r="L5" s="6"/>
     </row>
@@ -1162,19 +1367,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>17</v>
@@ -1183,13 +1388,13 @@
         <v>18</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="K6" s="13">
-        <v>46206</v>
+        <v>34</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>35</v>
       </c>
       <c r="L6" s="2"/>
     </row>
@@ -1198,19 +1403,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>17</v>
@@ -1219,13 +1424,13 @@
         <v>18</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="K7" s="12">
-        <v>46206</v>
+        <v>34</v>
+      </c>
+      <c r="K7" s="12" t="s">
+        <v>35</v>
       </c>
       <c r="L7" s="6"/>
     </row>
@@ -1234,19 +1439,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>17</v>
@@ -1255,13 +1460,13 @@
         <v>18</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="L8" s="2"/>
     </row>
@@ -1270,19 +1475,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G9" s="9" t="s">
         <v>17</v>
@@ -1291,13 +1496,13 @@
         <v>18</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="L9" s="6"/>
     </row>
@@ -1306,19 +1511,19 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>17</v>
@@ -1327,13 +1532,13 @@
         <v>18</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="L10" s="2"/>
     </row>
@@ -1342,34 +1547,34 @@
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
+      </c>
+      <c r="G11" s="13" t="s">
+        <v>56</v>
       </c>
       <c r="H11" s="7" t="s">
         <v>18</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="L11" s="6"/>
     </row>
@@ -1378,34 +1583,34 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E12" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G12" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="G12" s="11" t="s">
-        <v>54</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>18</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="L12" s="2"/>
     </row>
@@ -1414,19 +1619,19 @@
         <v>12</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G13" s="9" t="s">
         <v>17</v>
@@ -1435,13 +1640,13 @@
         <v>18</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="L13" s="6"/>
     </row>
@@ -1450,19 +1655,19 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G14" s="5" t="s">
         <v>17</v>
@@ -1471,13 +1676,13 @@
         <v>18</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="L14" s="2"/>
     </row>
@@ -1486,19 +1691,19 @@
         <v>14</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G15" s="9" t="s">
         <v>17</v>
@@ -1506,8 +1711,8 @@
       <c r="H15" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I15" s="12">
-        <v>46238</v>
+      <c r="I15" s="12" t="s">
+        <v>71</v>
       </c>
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
@@ -1518,19 +1723,19 @@
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>17</v>
@@ -1538,8 +1743,8 @@
       <c r="H16" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I16" s="13">
-        <v>46238</v>
+      <c r="I16" s="11" t="s">
+        <v>71</v>
       </c>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
@@ -1550,19 +1755,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="G17" s="9" t="s">
         <v>17</v>
@@ -1570,8 +1775,8 @@
       <c r="H17" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I17" s="12">
-        <v>46238</v>
+      <c r="I17" s="12" t="s">
+        <v>71</v>
       </c>
       <c r="J17" s="6"/>
       <c r="K17" s="6"/>
@@ -1582,19 +1787,19 @@
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G18" s="5" t="s">
         <v>17</v>
@@ -1602,17 +1807,17 @@
       <c r="H18" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="13">
-        <v>46235</v>
+      <c r="I18" s="11" t="s">
+        <v>19</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>165</v>
+        <v>20</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>165</v>
+        <v>20</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>165</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.3">
@@ -1620,19 +1825,19 @@
         <v>18</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="G19" s="9" t="s">
         <v>17</v>
@@ -1641,10 +1846,10 @@
         <v>18</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="K19" s="6"/>
       <c r="L19" s="6"/>
@@ -1654,28 +1859,28 @@
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="G20" s="5" t="s">
         <v>17</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="I20" s="13">
-        <v>46235</v>
+        <v>86</v>
+      </c>
+      <c r="I20" s="11" t="s">
+        <v>19</v>
       </c>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
@@ -1686,19 +1891,19 @@
         <v>20</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G21" s="9" t="s">
         <v>17</v>
@@ -1714,28 +1919,28 @@
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D22" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H22" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="E22" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="G22" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="H22" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="I22" s="13">
-        <v>46236</v>
+      <c r="I22" s="11" t="s">
+        <v>93</v>
       </c>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
@@ -1746,28 +1951,28 @@
         <v>22</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="G23" s="9" t="s">
         <v>17</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="I23" s="12">
-        <v>46236</v>
+        <v>86</v>
+      </c>
+      <c r="I23" s="12" t="s">
+        <v>93</v>
       </c>
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
@@ -1778,28 +1983,28 @@
         <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="G24" s="5" t="s">
         <v>17</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="I24" s="13">
-        <v>46237</v>
+        <v>86</v>
+      </c>
+      <c r="I24" s="11" t="s">
+        <v>99</v>
       </c>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
@@ -1810,19 +2015,19 @@
         <v>24</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="G25" s="9" t="s">
         <v>17</v>
@@ -1831,13 +2036,13 @@
         <v>18</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="L25" s="6"/>
     </row>
@@ -1846,19 +2051,19 @@
         <v>25</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="G26" s="5" t="s">
         <v>17</v>
@@ -1874,19 +2079,19 @@
         <v>26</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="G27" s="9" t="s">
         <v>17</v>
@@ -1895,10 +2100,10 @@
         <v>18</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="K27" s="6"/>
       <c r="L27" s="6"/>
@@ -1908,19 +2113,19 @@
         <v>27</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>102</v>
+        <v>77</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="G28" s="5" t="s">
         <v>17</v>
@@ -1936,22 +2141,22 @@
         <v>28</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>102</v>
+        <v>77</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="G29" s="9" t="s">
-        <v>17</v>
+        <v>115</v>
+      </c>
+      <c r="G29" s="14" t="s">
+        <v>56</v>
       </c>
       <c r="H29" s="7"/>
       <c r="I29" s="6"/>
@@ -1964,35 +2169,27 @@
         <v>29</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>102</v>
+        <v>77</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="H30" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I30" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="J30" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="K30" s="2" t="s">
-        <v>20</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="G30" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H30" s="3"/>
+      <c r="I30" s="2"/>
+      <c r="J30" s="2"/>
+      <c r="K30" s="2"/>
       <c r="L30" s="2"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.3">
@@ -2000,35 +2197,27 @@
         <v>30</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>102</v>
+        <v>77</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="G31" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H31" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I31" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="J31" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="K31" s="12">
-        <v>46236</v>
-      </c>
+      <c r="H31" s="7"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="6"/>
+      <c r="K31" s="6"/>
       <c r="L31" s="6"/>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.3">
@@ -2036,19 +2225,19 @@
         <v>31</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="G32" s="5" t="s">
         <v>17</v>
@@ -2064,29 +2253,25 @@
         <v>32</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="G33" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H33" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I33" s="12">
-        <v>46238</v>
-      </c>
+      <c r="H33" s="7"/>
+      <c r="I33" s="6"/>
       <c r="J33" s="6"/>
       <c r="K33" s="6"/>
       <c r="L33" s="6"/>
@@ -2096,19 +2281,19 @@
         <v>33</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="G34" s="5" t="s">
         <v>17</v>
@@ -2116,11 +2301,15 @@
       <c r="H34" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I34" s="13">
-        <v>46238</v>
-      </c>
-      <c r="J34" s="2"/>
-      <c r="K34" s="2"/>
+      <c r="I34" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="L34" s="2"/>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.3">
@@ -2128,27 +2317,35 @@
         <v>34</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="G35" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H35" s="7"/>
-      <c r="I35" s="6"/>
-      <c r="J35" s="6"/>
-      <c r="K35" s="6"/>
+      <c r="H35" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="K35" s="12" t="s">
+        <v>93</v>
+      </c>
       <c r="L35" s="6"/>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.3">
@@ -2156,19 +2353,19 @@
         <v>35</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="G36" s="5" t="s">
         <v>17</v>
@@ -2184,25 +2381,29 @@
         <v>36</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>131</v>
+        <v>114</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="G37" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H37" s="7"/>
-      <c r="I37" s="6"/>
+      <c r="H37" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I37" s="12" t="s">
+        <v>71</v>
+      </c>
       <c r="J37" s="6"/>
       <c r="K37" s="6"/>
       <c r="L37" s="6"/>
@@ -2212,25 +2413,29 @@
         <v>37</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>129</v>
+        <v>114</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="G38" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H38" s="3"/>
-      <c r="I38" s="2"/>
+      <c r="H38" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I38" s="11" t="s">
+        <v>71</v>
+      </c>
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
       <c r="L38" s="2"/>
@@ -2240,19 +2445,19 @@
         <v>38</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>137</v>
+        <v>114</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="G39" s="9" t="s">
         <v>17</v>
@@ -2268,35 +2473,27 @@
         <v>39</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>126</v>
+        <v>146</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>127</v>
+        <v>147</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="G40" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H40" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I40" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="J40" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="K40" s="2" t="s">
-        <v>20</v>
-      </c>
+      <c r="H40" s="3"/>
+      <c r="I40" s="2"/>
+      <c r="J40" s="2"/>
+      <c r="K40" s="2"/>
       <c r="L40" s="2"/>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.3">
@@ -2304,35 +2501,27 @@
         <v>40</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>126</v>
+        <v>146</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>127</v>
+        <v>147</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="G41" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H41" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I41" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="J41" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="K41" s="12">
-        <v>46237</v>
-      </c>
+      <c r="H41" s="7"/>
+      <c r="I41" s="6"/>
+      <c r="J41" s="6"/>
+      <c r="K41" s="6"/>
       <c r="L41" s="6"/>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.3">
@@ -2340,19 +2529,19 @@
         <v>41</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="G42" s="5" t="s">
         <v>17</v>
@@ -2368,19 +2557,19 @@
         <v>42</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="G43" s="9" t="s">
         <v>17</v>
@@ -2396,27 +2585,35 @@
         <v>43</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="G44" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H44" s="3"/>
-      <c r="I44" s="2"/>
-      <c r="J44" s="2"/>
-      <c r="K44" s="2"/>
+      <c r="H44" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="L44" s="2"/>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.3">
@@ -2424,27 +2621,35 @@
         <v>44</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="G45" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="H45" s="7"/>
-      <c r="I45" s="6"/>
-      <c r="J45" s="6"/>
-      <c r="K45" s="6"/>
+        <v>164</v>
+      </c>
+      <c r="G45" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H45" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I45" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="J45" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="K45" s="12" t="s">
+        <v>99</v>
+      </c>
       <c r="L45" s="6"/>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.3">
@@ -2452,22 +2657,22 @@
         <v>45</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>145</v>
+        <v>165</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>146</v>
+        <v>166</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>148</v>
+        <v>120</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="G46" s="11" t="s">
-        <v>54</v>
+        <v>168</v>
+      </c>
+      <c r="G46" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="H46" s="3"/>
       <c r="I46" s="2"/>
@@ -2480,19 +2685,19 @@
         <v>46</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>145</v>
+        <v>165</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>146</v>
+        <v>169</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="F47" s="8" t="s">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="G47" s="9" t="s">
         <v>17</v>
@@ -2508,22 +2713,22 @@
         <v>47</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>145</v>
+        <v>165</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>146</v>
+        <v>169</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="G48" s="11" t="s">
-        <v>54</v>
+        <v>174</v>
+      </c>
+      <c r="G48" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="H48" s="3"/>
       <c r="I48" s="2"/>
@@ -2531,10 +2736,485 @@
       <c r="K48" s="2"/>
       <c r="L48" s="2"/>
     </row>
-    <row r="51" spans="11:11" x14ac:dyDescent="0.3">
-      <c r="K51" t="s">
-        <v>167</v>
-      </c>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A49" s="6">
+        <v>48</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="E49" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="F49" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="G49" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H49" s="7"/>
+      <c r="I49" s="6"/>
+      <c r="J49" s="6"/>
+      <c r="K49" s="6"/>
+      <c r="L49" s="6"/>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A50" s="2">
+        <v>49</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="G50" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H50" s="3"/>
+      <c r="I50" s="2"/>
+      <c r="J50" s="2"/>
+      <c r="K50" s="2"/>
+      <c r="L50" s="2"/>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A51" s="6">
+        <v>50</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="E51" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="F51" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="G51" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H51" s="7"/>
+      <c r="I51" s="6"/>
+      <c r="J51" s="6"/>
+      <c r="K51" s="6"/>
+      <c r="L51" s="6"/>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A52" s="2">
+        <v>51</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="G52" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H52" s="3"/>
+      <c r="I52" s="2"/>
+      <c r="J52" s="2"/>
+      <c r="K52" s="2"/>
+      <c r="L52" s="2"/>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A53" s="6">
+        <v>52</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="E53" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="F53" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="G53" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H53" s="7"/>
+      <c r="I53" s="6"/>
+      <c r="J53" s="6"/>
+      <c r="K53" s="6"/>
+      <c r="L53" s="6"/>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A54" s="2">
+        <v>53</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="G54" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H54" s="3"/>
+      <c r="I54" s="2"/>
+      <c r="J54" s="2"/>
+      <c r="K54" s="2"/>
+      <c r="L54" s="2"/>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A55" s="6">
+        <v>54</v>
+      </c>
+      <c r="B55" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="D55" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="E55" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="F55" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="G55" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H55" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I55" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="J55" s="6"/>
+      <c r="K55" s="6"/>
+      <c r="L55" s="6"/>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A56" s="2">
+        <v>55</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="G56" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H56" s="3"/>
+      <c r="I56" s="2"/>
+      <c r="J56" s="2"/>
+      <c r="K56" s="2"/>
+      <c r="L56" s="2"/>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A57" s="6">
+        <v>56</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="E57" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="F57" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="G57" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H57" s="7"/>
+      <c r="I57" s="6"/>
+      <c r="J57" s="6"/>
+      <c r="K57" s="6"/>
+      <c r="L57" s="6"/>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A58" s="2">
+        <v>57</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="G58" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H58" s="3"/>
+      <c r="I58" s="2"/>
+      <c r="J58" s="2"/>
+      <c r="K58" s="2"/>
+      <c r="L58" s="2"/>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A59" s="6">
+        <v>58</v>
+      </c>
+      <c r="B59" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="C59" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="D59" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="E59" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="F59" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="G59" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="H59" s="7"/>
+      <c r="I59" s="6"/>
+      <c r="J59" s="6"/>
+      <c r="K59" s="6"/>
+      <c r="L59" s="6"/>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A60" s="2">
+        <v>59</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="F60" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="G60" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H60" s="3"/>
+      <c r="I60" s="2"/>
+      <c r="J60" s="2"/>
+      <c r="K60" s="2"/>
+      <c r="L60" s="2"/>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A61" s="6">
+        <v>60</v>
+      </c>
+      <c r="B61" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="C61" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="D61" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="E61" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="F61" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="G61" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="H61" s="7"/>
+      <c r="I61" s="6"/>
+      <c r="J61" s="6"/>
+      <c r="K61" s="6"/>
+      <c r="L61" s="6"/>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A62" s="2">
+        <v>61</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="F62" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="G62" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H62" s="3"/>
+      <c r="I62" s="2"/>
+      <c r="J62" s="2"/>
+      <c r="K62" s="2"/>
+      <c r="L62" s="2"/>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A63" s="6">
+        <v>62</v>
+      </c>
+      <c r="B63" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="C63" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="D63" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="E63" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="F63" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="G63" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H63" s="7"/>
+      <c r="I63" s="6"/>
+      <c r="J63" s="6"/>
+      <c r="K63" s="6"/>
+      <c r="L63" s="6"/>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A64" s="2">
+        <v>63</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="E64" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="F64" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="G64" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H64" s="3"/>
+      <c r="I64" s="2"/>
+      <c r="J64" s="2"/>
+      <c r="K64" s="2"/>
+      <c r="L64" s="2"/>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A65" s="6">
+        <v>64</v>
+      </c>
+      <c r="B65" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="C65" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="D65" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="E65" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="F65" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="G65" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="H65" s="7"/>
+      <c r="I65" s="6"/>
+      <c r="J65" s="6"/>
+      <c r="K65" s="6"/>
+      <c r="L65" s="6"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L48" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
@@ -2586,6 +3266,23 @@
     <hyperlink ref="F46" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
     <hyperlink ref="F47" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
     <hyperlink ref="F48" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="F49" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="F50" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="F51" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="F52" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="F53" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="F54" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="F55" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="F56" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="F57" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="F58" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="F59" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="F60" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="F61" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="F62" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="F63" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
+    <hyperlink ref="F64" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="F65" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Made a program to find the roots of a quadratic equation
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37F6DCD4-3681-47C3-93C0-4431C5D669D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81722816-CFE4-4C81-B040-DEE4BFC333C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="225">
   <si>
     <t>No.</t>
   </si>
@@ -815,7 +815,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -857,6 +857,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2214,8 +2217,12 @@
       <c r="G31" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H31" s="7"/>
-      <c r="I31" s="6"/>
+      <c r="H31" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I31" s="15">
+        <v>46239</v>
+      </c>
       <c r="J31" s="6"/>
       <c r="K31" s="6"/>
       <c r="L31" s="6"/>

</xml_diff>

<commit_message>
Solve LeetCode 125 Valid Palindrome
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vaibhav\DSA-Java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81722816-CFE4-4C81-B040-DEE4BFC333C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA7C3A54-9014-4399-A46B-1F43884F6307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="DSA Tracker" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DSA Tracker'!$A$1:$L$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DSA Tracker'!$A$1:$L$69</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="240">
   <si>
     <t>No.</t>
   </si>
@@ -256,6 +256,30 @@
     <t>https://leetcode.com/problems/goal-parser-interpretation/</t>
   </si>
   <si>
+    <t>Length of Last Word</t>
+  </si>
+  <si>
+    <t>Iteration</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/length-of-last-word/</t>
+  </si>
+  <si>
+    <t>10-08-2026</t>
+  </si>
+  <si>
+    <t>Roman to Integer</t>
+  </si>
+  <si>
+    <t>HashMap</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/roman-to-integer/</t>
+  </si>
+  <si>
+    <t>08-08-2026</t>
+  </si>
+  <si>
     <t>Arrays</t>
   </si>
   <si>
@@ -394,6 +418,9 @@
     <t>https://leetcode.com/problems/remove-duplicates-from-sorted-array/</t>
   </si>
   <si>
+    <t>06-08-2026</t>
+  </si>
+  <si>
     <t>Arrays - Two Pointers</t>
   </si>
   <si>
@@ -409,6 +436,9 @@
     <t>https://leetcode.com/problems/reverse-string/</t>
   </si>
   <si>
+    <t>11-08-2026</t>
+  </si>
+  <si>
     <t>Remove Element</t>
   </si>
   <si>
@@ -436,6 +466,18 @@
     <t>27-07-2026</t>
   </si>
   <si>
+    <t>Trapping Rain Water</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/trapping-rain-water/</t>
+  </si>
+  <si>
+    <t>Hard</t>
+  </si>
+  <si>
+    <t>12-08-2026</t>
+  </si>
+  <si>
     <t>Binary Search &amp; Sort</t>
   </si>
   <si>
@@ -463,6 +505,12 @@
     <t>https://leetcode.com/problems/first-bad-version/</t>
   </si>
   <si>
+    <t>Sqrt(x)</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/sqrtx/</t>
+  </si>
+  <si>
     <t>Hashing</t>
   </si>
   <si>
@@ -505,9 +553,6 @@
     <t>Two Sum</t>
   </si>
   <si>
-    <t>HashMap</t>
-  </si>
-  <si>
     <t>https://leetcode.com/problems/two-sum/</t>
   </si>
   <si>
@@ -538,9 +583,6 @@
     <t>Remove Linked List Elements</t>
   </si>
   <si>
-    <t>Iteration</t>
-  </si>
-  <si>
     <t>https://leetcode.com/problems/remove-linked-list-elements/</t>
   </si>
   <si>
@@ -638,6 +680,9 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/remove-all-adjacent-duplicates-in-string/</t>
+  </si>
+  <si>
+    <t>09-08-2026</t>
   </si>
   <si>
     <t>Min Stack</t>
@@ -704,9 +749,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
-  </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -742,12 +784,11 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="9" tint="-0.249977111117893"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -764,12 +805,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
         <bgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -815,7 +850,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -844,22 +879,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1164,7 +1190,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -1240,7 +1266,7 @@
       <c r="H2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="I2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="J2" s="2" t="s">
@@ -1278,7 +1304,7 @@
       <c r="H3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="I3" s="6" t="s">
         <v>19</v>
       </c>
       <c r="J3" s="6" t="s">
@@ -1360,7 +1386,7 @@
       <c r="J5" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="K5" s="12" t="s">
+      <c r="K5" s="6" t="s">
         <v>35</v>
       </c>
       <c r="L5" s="6"/>
@@ -1396,7 +1422,7 @@
       <c r="J6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="K6" s="11" t="s">
+      <c r="K6" s="2" t="s">
         <v>35</v>
       </c>
       <c r="L6" s="2"/>
@@ -1432,7 +1458,7 @@
       <c r="J7" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="K7" s="12" t="s">
+      <c r="K7" s="6" t="s">
         <v>35</v>
       </c>
       <c r="L7" s="6"/>
@@ -1564,7 +1590,7 @@
       <c r="F11" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="G11" s="13" t="s">
+      <c r="G11" s="10" t="s">
         <v>56</v>
       </c>
       <c r="H11" s="7" t="s">
@@ -1600,7 +1626,7 @@
       <c r="F12" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="G12" s="11" t="s">
         <v>56</v>
       </c>
       <c r="H12" s="3" t="s">
@@ -1714,7 +1740,7 @@
       <c r="H15" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I15" s="12" t="s">
+      <c r="I15" s="6" t="s">
         <v>71</v>
       </c>
       <c r="J15" s="6"/>
@@ -1746,7 +1772,7 @@
       <c r="H16" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I16" s="11" t="s">
+      <c r="I16" s="2" t="s">
         <v>71</v>
       </c>
       <c r="J16" s="2"/>
@@ -1778,7 +1804,7 @@
       <c r="H17" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I17" s="12" t="s">
+      <c r="I17" s="6" t="s">
         <v>71</v>
       </c>
       <c r="J17" s="6"/>
@@ -1790,19 +1816,19 @@
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="E18" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="F18" s="4" t="s">
         <v>79</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>80</v>
       </c>
       <c r="G18" s="5" t="s">
         <v>17</v>
@@ -1810,37 +1836,31 @@
       <c r="H18" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="L18" s="2" t="s">
-        <v>20</v>
-      </c>
+      <c r="I18" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
+      <c r="L18" s="2"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
         <v>18</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>81</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>31</v>
+        <v>82</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G19" s="9" t="s">
         <v>17</v>
@@ -1849,11 +1869,9 @@
         <v>18</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="J19" s="6" t="s">
-        <v>27</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="J19" s="6"/>
       <c r="K19" s="6"/>
       <c r="L19" s="6"/>
     </row>
@@ -1862,58 +1880,70 @@
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>84</v>
+        <v>31</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="G20" s="5" t="s">
         <v>17</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="I20" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="I20" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
-      <c r="L20" s="2"/>
+      <c r="J20" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="6">
         <v>20</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>88</v>
+        <v>31</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G21" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H21" s="7"/>
-      <c r="I21" s="6"/>
-      <c r="J21" s="6"/>
+      <c r="H21" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>27</v>
+      </c>
       <c r="K21" s="6"/>
       <c r="L21" s="6"/>
     </row>
@@ -1922,28 +1952,28 @@
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G22" s="5" t="s">
         <v>17</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="I22" s="11" t="s">
-        <v>93</v>
+        <v>94</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
@@ -1954,29 +1984,25 @@
         <v>22</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G23" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H23" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="I23" s="12" t="s">
-        <v>93</v>
-      </c>
+      <c r="H23" s="7"/>
+      <c r="I23" s="6"/>
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
       <c r="L23" s="6"/>
@@ -1986,28 +2012,28 @@
         <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G24" s="5" t="s">
         <v>17</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="I24" s="11" t="s">
-        <v>99</v>
+        <v>94</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>101</v>
       </c>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
@@ -2018,35 +2044,31 @@
         <v>24</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E25" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="I25" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="F25" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="G25" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="H25" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I25" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="J25" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="K25" s="6" t="s">
-        <v>34</v>
-      </c>
+      <c r="J25" s="6"/>
+      <c r="K25" s="6"/>
       <c r="L25" s="6"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.3">
@@ -2054,25 +2076,29 @@
         <v>25</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="D26" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="E26" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="E26" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="F26" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G26" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H26" s="3"/>
-      <c r="I26" s="2"/>
+      <c r="H26" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>107</v>
+      </c>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
@@ -2082,19 +2108,19 @@
         <v>26</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="G27" s="9" t="s">
         <v>17</v>
@@ -2103,12 +2129,14 @@
         <v>18</v>
       </c>
       <c r="I27" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J27" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K27" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="J27" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="K27" s="6"/>
       <c r="L27" s="6"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.3">
@@ -2116,19 +2144,19 @@
         <v>27</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>110</v>
+        <v>31</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G28" s="5" t="s">
         <v>17</v>
@@ -2144,10 +2172,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>112</v>
+        <v>86</v>
       </c>
       <c r="D29" s="7" t="s">
         <v>113</v>
@@ -2158,12 +2186,18 @@
       <c r="F29" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="G29" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="H29" s="7"/>
-      <c r="I29" s="6"/>
-      <c r="J29" s="6"/>
+      <c r="G29" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="J29" s="6" t="s">
+        <v>53</v>
+      </c>
       <c r="K29" s="6"/>
       <c r="L29" s="6"/>
     </row>
@@ -2172,7 +2206,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>116</v>
@@ -2186,8 +2220,8 @@
       <c r="F30" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="G30" s="10" t="s">
-        <v>56</v>
+      <c r="G30" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="H30" s="3"/>
       <c r="I30" s="2"/>
@@ -2200,7 +2234,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C31" s="7" t="s">
         <v>120</v>
@@ -2209,20 +2243,16 @@
         <v>121</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="G31" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="H31" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="I31" s="15">
-        <v>46239</v>
-      </c>
+        <v>123</v>
+      </c>
+      <c r="G31" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H31" s="7"/>
+      <c r="I31" s="6"/>
       <c r="J31" s="6"/>
       <c r="K31" s="6"/>
       <c r="L31" s="6"/>
@@ -2232,7 +2262,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>123</v>
+        <v>85</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>124</v>
@@ -2246,8 +2276,8 @@
       <c r="F32" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="G32" s="5" t="s">
-        <v>17</v>
+      <c r="G32" s="11" t="s">
+        <v>56</v>
       </c>
       <c r="H32" s="3"/>
       <c r="I32" s="2"/>
@@ -2260,16 +2290,16 @@
         <v>32</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>123</v>
+        <v>85</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="D33" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="E33" s="7" t="s">
         <v>128</v>
-      </c>
-      <c r="E33" s="7" t="s">
-        <v>129</v>
       </c>
       <c r="F33" s="8" t="s">
         <v>130</v>
@@ -2277,8 +2307,12 @@
       <c r="G33" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H33" s="7"/>
-      <c r="I33" s="6"/>
+      <c r="H33" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I33" s="6" t="s">
+        <v>131</v>
+      </c>
       <c r="J33" s="6"/>
       <c r="K33" s="6"/>
       <c r="L33" s="6"/>
@@ -2288,19 +2322,19 @@
         <v>33</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="G34" s="5" t="s">
         <v>17</v>
@@ -2309,14 +2343,10 @@
         <v>18</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="J34" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="K34" s="2" t="s">
-        <v>19</v>
-      </c>
+        <v>137</v>
+      </c>
+      <c r="J34" s="2"/>
+      <c r="K34" s="2"/>
       <c r="L34" s="2"/>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.3">
@@ -2324,35 +2354,27 @@
         <v>34</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="G35" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H35" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I35" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="J35" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="K35" s="12" t="s">
-        <v>93</v>
-      </c>
+      <c r="H35" s="7"/>
+      <c r="I35" s="6"/>
+      <c r="J35" s="6"/>
+      <c r="K35" s="6"/>
       <c r="L35" s="6"/>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.3">
@@ -2360,27 +2382,35 @@
         <v>35</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>139</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="G36" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H36" s="3"/>
-      <c r="I36" s="2"/>
-      <c r="J36" s="2"/>
-      <c r="K36" s="2"/>
+      <c r="H36" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="L36" s="2"/>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.3">
@@ -2388,19 +2418,19 @@
         <v>36</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>114</v>
+        <v>144</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="G37" s="9" t="s">
         <v>17</v>
@@ -2408,11 +2438,15 @@
       <c r="H37" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I37" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="J37" s="6"/>
-      <c r="K37" s="6"/>
+      <c r="I37" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="J37" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>101</v>
+      </c>
       <c r="L37" s="6"/>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.3">
@@ -2420,28 +2454,28 @@
         <v>37</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="G38" s="5" t="s">
-        <v>17</v>
+        <v>148</v>
+      </c>
+      <c r="G38" s="12" t="s">
+        <v>149</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I38" s="11" t="s">
-        <v>71</v>
+        <v>94</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>150</v>
       </c>
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
@@ -2452,19 +2486,19 @@
         <v>38</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>114</v>
+        <v>153</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="G39" s="9" t="s">
         <v>17</v>
@@ -2480,25 +2514,29 @@
         <v>39</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>147</v>
+        <v>122</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>148</v>
+        <v>122</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>149</v>
+        <v>122</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="G40" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H40" s="3"/>
-      <c r="I40" s="2"/>
+      <c r="H40" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>71</v>
+      </c>
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
       <c r="L40" s="2"/>
@@ -2508,25 +2546,29 @@
         <v>40</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>147</v>
+        <v>122</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>152</v>
+        <v>122</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G41" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H41" s="7"/>
-      <c r="I41" s="6"/>
+      <c r="H41" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I41" s="6" t="s">
+        <v>71</v>
+      </c>
       <c r="J41" s="6"/>
       <c r="K41" s="6"/>
       <c r="L41" s="6"/>
@@ -2536,25 +2578,29 @@
         <v>41</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>147</v>
+        <v>122</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>149</v>
+        <v>122</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="G42" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H42" s="3"/>
-      <c r="I42" s="2"/>
+      <c r="H42" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>131</v>
+      </c>
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
       <c r="L42" s="2"/>
@@ -2564,25 +2610,29 @@
         <v>42</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>147</v>
+        <v>122</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>157</v>
+        <v>122</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="G43" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H43" s="7"/>
-      <c r="I43" s="6"/>
+      <c r="H43" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I43" s="6" t="s">
+        <v>150</v>
+      </c>
       <c r="J43" s="6"/>
       <c r="K43" s="6"/>
       <c r="L43" s="6"/>
@@ -2592,35 +2642,27 @@
         <v>43</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>146</v>
+        <v>162</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="G44" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H44" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I44" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="J44" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="K44" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="H44" s="3"/>
+      <c r="I44" s="2"/>
+      <c r="J44" s="2"/>
+      <c r="K44" s="2"/>
       <c r="L44" s="2"/>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.3">
@@ -2628,35 +2670,27 @@
         <v>44</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>146</v>
+        <v>162</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="G45" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H45" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I45" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="J45" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="K45" s="12" t="s">
-        <v>99</v>
-      </c>
+      <c r="H45" s="7"/>
+      <c r="I45" s="6"/>
+      <c r="J45" s="6"/>
+      <c r="K45" s="6"/>
       <c r="L45" s="6"/>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.3">
@@ -2664,19 +2698,19 @@
         <v>45</v>
       </c>
       <c r="B46" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="E46" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="C46" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="E46" s="3" t="s">
-        <v>120</v>
-      </c>
       <c r="F46" s="4" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="G46" s="5" t="s">
         <v>17</v>
@@ -2692,19 +2726,19 @@
         <v>46</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="F47" s="8" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="G47" s="9" t="s">
         <v>17</v>
@@ -2720,27 +2754,35 @@
         <v>47</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>171</v>
+        <v>82</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G48" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H48" s="3"/>
-      <c r="I48" s="2"/>
-      <c r="J48" s="2"/>
-      <c r="K48" s="2"/>
+      <c r="H48" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="J48" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="L48" s="2"/>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.3">
@@ -2748,27 +2790,35 @@
         <v>48</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E49" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F49" s="8" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G49" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H49" s="7"/>
-      <c r="I49" s="6"/>
-      <c r="J49" s="6"/>
-      <c r="K49" s="6"/>
+      <c r="H49" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I49" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="J49" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="K49" s="6" t="s">
+        <v>107</v>
+      </c>
       <c r="L49" s="6"/>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.3">
@@ -2776,19 +2826,19 @@
         <v>49</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>165</v>
+        <v>180</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>181</v>
+        <v>128</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G50" s="5" t="s">
         <v>17</v>
@@ -2804,19 +2854,19 @@
         <v>50</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>165</v>
+        <v>180</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="E51" s="7" t="s">
-        <v>181</v>
+        <v>78</v>
       </c>
       <c r="F51" s="8" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="G51" s="9" t="s">
         <v>17</v>
@@ -2832,19 +2882,19 @@
         <v>51</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>165</v>
+        <v>180</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>186</v>
+        <v>78</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G52" s="5" t="s">
         <v>17</v>
@@ -2860,7 +2910,7 @@
         <v>52</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="C53" s="7" t="s">
         <v>189</v>
@@ -2888,19 +2938,19 @@
         <v>53</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G54" s="5" t="s">
         <v>17</v>
@@ -2916,29 +2966,25 @@
         <v>54</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="D55" s="7" t="s">
         <v>197</v>
       </c>
       <c r="E55" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="F55" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="F55" s="8" t="s">
-        <v>199</v>
-      </c>
       <c r="G55" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H55" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="I55" s="12" t="s">
-        <v>71</v>
-      </c>
+      <c r="H55" s="7"/>
+      <c r="I55" s="6"/>
       <c r="J55" s="6"/>
       <c r="K55" s="6"/>
       <c r="L55" s="6"/>
@@ -2948,19 +2994,19 @@
         <v>55</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="D56" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="E56" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="E56" s="3" t="s">
+      <c r="F56" s="4" t="s">
         <v>201</v>
-      </c>
-      <c r="F56" s="4" t="s">
-        <v>202</v>
       </c>
       <c r="G56" s="5" t="s">
         <v>17</v>
@@ -2976,19 +3022,19 @@
         <v>56</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>188</v>
+        <v>202</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="D57" s="7" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E57" s="7" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="F57" s="8" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="G57" s="9" t="s">
         <v>17</v>
@@ -3004,22 +3050,22 @@
         <v>57</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>188</v>
+        <v>202</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>191</v>
+        <v>208</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="G58" s="10" t="s">
-        <v>56</v>
+        <v>209</v>
+      </c>
+      <c r="G58" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="H58" s="3"/>
       <c r="I58" s="2"/>
@@ -3032,25 +3078,29 @@
         <v>58</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>188</v>
+        <v>202</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>196</v>
+        <v>210</v>
       </c>
       <c r="D59" s="7" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E59" s="7" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
       <c r="F59" s="8" t="s">
-        <v>208</v>
-      </c>
-      <c r="G59" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="H59" s="7"/>
-      <c r="I59" s="6"/>
+        <v>213</v>
+      </c>
+      <c r="G59" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H59" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I59" s="6" t="s">
+        <v>71</v>
+      </c>
       <c r="J59" s="6"/>
       <c r="K59" s="6"/>
       <c r="L59" s="6"/>
@@ -3060,19 +3110,19 @@
         <v>59</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>188</v>
+        <v>202</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>196</v>
+        <v>210</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="G60" s="5" t="s">
         <v>17</v>
@@ -3088,25 +3138,29 @@
         <v>60</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>188</v>
+        <v>202</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>196</v>
+        <v>210</v>
       </c>
       <c r="D61" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="E61" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="E61" s="7" t="s">
-        <v>210</v>
-      </c>
       <c r="F61" s="8" t="s">
-        <v>213</v>
-      </c>
-      <c r="G61" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="H61" s="7"/>
-      <c r="I61" s="6"/>
+        <v>218</v>
+      </c>
+      <c r="G61" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H61" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I61" s="6" t="s">
+        <v>219</v>
+      </c>
       <c r="J61" s="6"/>
       <c r="K61" s="6"/>
       <c r="L61" s="6"/>
@@ -3116,22 +3170,22 @@
         <v>61</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>188</v>
+        <v>202</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="G62" s="5" t="s">
-        <v>17</v>
+        <v>221</v>
+      </c>
+      <c r="G62" s="11" t="s">
+        <v>56</v>
       </c>
       <c r="H62" s="3"/>
       <c r="I62" s="2"/>
@@ -3144,22 +3198,22 @@
         <v>62</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>217</v>
+        <v>202</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>108</v>
+        <v>210</v>
       </c>
       <c r="D63" s="7" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E63" s="7" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="F63" s="8" t="s">
-        <v>219</v>
-      </c>
-      <c r="G63" s="9" t="s">
-        <v>17</v>
+        <v>223</v>
+      </c>
+      <c r="G63" s="10" t="s">
+        <v>56</v>
       </c>
       <c r="H63" s="7"/>
       <c r="I63" s="6"/>
@@ -3172,19 +3226,19 @@
         <v>63</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>217</v>
+        <v>202</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>108</v>
+        <v>210</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="G64" s="5" t="s">
         <v>17</v>
@@ -3200,21 +3254,21 @@
         <v>64</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>217</v>
+        <v>202</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="E65" s="7" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="F65" s="8" t="s">
-        <v>224</v>
-      </c>
-      <c r="G65" s="13" t="s">
+        <v>228</v>
+      </c>
+      <c r="G65" s="10" t="s">
         <v>56</v>
       </c>
       <c r="H65" s="7"/>
@@ -3223,8 +3277,120 @@
       <c r="K65" s="6"/>
       <c r="L65" s="6"/>
     </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A66" s="2">
+        <v>65</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="E66" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="F66" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="G66" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H66" s="3"/>
+      <c r="I66" s="2"/>
+      <c r="J66" s="2"/>
+      <c r="K66" s="2"/>
+      <c r="L66" s="2"/>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A67" s="6">
+        <v>66</v>
+      </c>
+      <c r="B67" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="C67" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="D67" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="E67" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="F67" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="G67" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H67" s="7"/>
+      <c r="I67" s="6"/>
+      <c r="J67" s="6"/>
+      <c r="K67" s="6"/>
+      <c r="L67" s="6"/>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A68" s="2">
+        <v>67</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="E68" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="G68" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H68" s="3"/>
+      <c r="I68" s="2"/>
+      <c r="J68" s="2"/>
+      <c r="K68" s="2"/>
+      <c r="L68" s="2"/>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A69" s="6">
+        <v>68</v>
+      </c>
+      <c r="B69" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="C69" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="D69" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="E69" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="F69" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="G69" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H69" s="7"/>
+      <c r="I69" s="6"/>
+      <c r="J69" s="6"/>
+      <c r="K69" s="6"/>
+      <c r="L69" s="6"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L48" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:L69" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="F3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
@@ -3290,6 +3456,10 @@
     <hyperlink ref="F63" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
     <hyperlink ref="F64" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
     <hyperlink ref="F65" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="F66" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="F67" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="F68" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="F69" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add a local hosted website to track dsa revison
</commit_message>
<xml_diff>
--- a/LeetCode_DSA_Tracker.xlsx
+++ b/LeetCode_DSA_Tracker.xlsx
@@ -9,7 +9,7 @@
     <sheet name="DSA Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DSA Tracker'!$A$1:$L$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DSA Tracker'!$A$1:$L$99</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -594,17 +594,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L86"/>
+  <dimension ref="A1:L99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="20.21875" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="9"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="13"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -710,7 +714,7 @@
       </c>
       <c r="I2" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="J2" s="13" t="inlineStr">
@@ -770,7 +774,7 @@
       </c>
       <c r="I3" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="J3" s="17" t="inlineStr">
@@ -830,7 +834,7 @@
       </c>
       <c r="I4" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
+          <t>31-07-2026</t>
         </is>
       </c>
       <c r="J4" s="13" t="inlineStr">
@@ -865,17 +869,17 @@
       </c>
       <c r="D5" s="18" t="inlineStr">
         <is>
-          <t>Smallest Missing Multiple of K</t>
+          <t>Add Digits</t>
         </is>
       </c>
       <c r="E5" s="18" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F5" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/smallest-missing-multiple-of-k/</t>
+          <t>https://leetcode.com/problems/add-digits/</t>
         </is>
       </c>
       <c r="G5" s="20" t="inlineStr">
@@ -890,12 +894,12 @@
       </c>
       <c r="I5" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J5" s="17" t="n"/>
-      <c r="K5" s="17" t="n"/>
-      <c r="L5" s="17" t="n"/>
+          <t>19-08-2026</t>
+        </is>
+      </c>
+      <c r="J5" s="17" t="inlineStr"/>
+      <c r="K5" s="17" t="inlineStr"/>
+      <c r="L5" s="17" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="13" t="n">
@@ -913,17 +917,17 @@
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>Add Digits</t>
+          <t>Smallest Missing Multiple of K</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/add-digits/</t>
+          <t>https://leetcode.com/problems/smallest-missing-multiple-of-k/</t>
         </is>
       </c>
       <c r="G6" s="16" t="inlineStr">
@@ -938,7 +942,7 @@
       </c>
       <c r="I6" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
+          <t>25-08-2026</t>
         </is>
       </c>
       <c r="J6" s="13" t="inlineStr"/>
@@ -961,7 +965,7 @@
       </c>
       <c r="D7" s="18" t="inlineStr">
         <is>
-          <t>Subtract the Product and Sum of Digits of an Integer</t>
+          <t>Add Binary</t>
         </is>
       </c>
       <c r="E7" s="18" t="inlineStr">
@@ -971,7 +975,7 @@
       </c>
       <c r="F7" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/subtract-the-product-and-sum-of-digits-of-an-integer/</t>
+          <t>https://leetcode.com/problems/add-binary/</t>
         </is>
       </c>
       <c r="G7" s="20" t="inlineStr">
@@ -986,20 +990,20 @@
       </c>
       <c r="I7" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="J7" s="17" t="inlineStr">
         <is>
-          <t>29-07-2026</t>
+          <t>25-07-2026</t>
         </is>
       </c>
       <c r="K7" s="17" t="inlineStr">
         <is>
-          <t>03-07-2026</t>
-        </is>
-      </c>
-      <c r="L7" s="17" t="n"/>
+          <t>31-07-2026</t>
+        </is>
+      </c>
+      <c r="L7" s="17" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="13" t="n">
@@ -1017,17 +1021,17 @@
       </c>
       <c r="D8" s="14" t="inlineStr">
         <is>
-          <t>Number of Steps to Reduce a Number to Zero</t>
+          <t>Base 7</t>
         </is>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Base Conversion</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/number-of-steps-to-reduce-a-number-to-zero/</t>
+          <t>https://leetcode.com/problems/base-7/</t>
         </is>
       </c>
       <c r="G8" s="16" t="inlineStr">
@@ -1042,20 +1046,20 @@
       </c>
       <c r="I8" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="J8" s="13" t="inlineStr">
         <is>
-          <t>29-07-2026</t>
+          <t>25-07-2026</t>
         </is>
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>03-07-2026</t>
-        </is>
-      </c>
-      <c r="L8" s="13" t="n"/>
+          <t>31-07-2026</t>
+        </is>
+      </c>
+      <c r="L8" s="13" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="17" t="n">
@@ -1073,17 +1077,17 @@
       </c>
       <c r="D9" s="18" t="inlineStr">
         <is>
-          <t>Power of Two</t>
+          <t>Climbing Stairs</t>
         </is>
       </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>Bitwise or Repeated Division</t>
+          <t>Fibonacci Sequence</t>
         </is>
       </c>
       <c r="F9" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/power-of-two/</t>
+          <t>https://leetcode.com/problems/climbing-stairs/</t>
         </is>
       </c>
       <c r="G9" s="20" t="inlineStr">
@@ -1098,20 +1102,20 @@
       </c>
       <c r="I9" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
+          <t>22-07-2026</t>
         </is>
       </c>
       <c r="J9" s="17" t="inlineStr">
         <is>
+          <t>23-07-2026</t>
+        </is>
+      </c>
+      <c r="K9" s="17" t="inlineStr">
+        <is>
           <t>29-07-2026</t>
         </is>
       </c>
-      <c r="K9" s="17" t="inlineStr">
-        <is>
-          <t>03-07-2026</t>
-        </is>
-      </c>
-      <c r="L9" s="17" t="n"/>
+      <c r="L9" s="17" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="13" t="n">
@@ -1129,22 +1133,22 @@
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>Fibonacci Number</t>
+          <t>Count Primes</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Recursion or DP</t>
+          <t>Sieve of Eratosthenes</t>
         </is>
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/fibonacci-number/</t>
-        </is>
-      </c>
-      <c r="G10" s="16" t="inlineStr">
-        <is>
-          <t>Easy</t>
+          <t>https://leetcode.com/problems/count-primes/</t>
+        </is>
+      </c>
+      <c r="G10" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H10" s="14" t="inlineStr">
@@ -1154,20 +1158,20 @@
       </c>
       <c r="I10" s="13" t="inlineStr">
         <is>
-          <t>22-07-2026</t>
+          <t>23-07-2026</t>
         </is>
       </c>
       <c r="J10" s="13" t="inlineStr">
         <is>
-          <t>23-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
-          <t>29-07-2026</t>
-        </is>
-      </c>
-      <c r="L10" s="13" t="n"/>
+          <t>30-07-2026</t>
+        </is>
+      </c>
+      <c r="L10" s="13" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="17" t="n">
@@ -1185,17 +1189,17 @@
       </c>
       <c r="D11" s="18" t="inlineStr">
         <is>
-          <t>Climbing Stairs</t>
+          <t>Fibonacci Number</t>
         </is>
       </c>
       <c r="E11" s="18" t="inlineStr">
         <is>
-          <t>Fibonacci Sequence</t>
+          <t>Recursion or DP</t>
         </is>
       </c>
       <c r="F11" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/climbing-stairs/</t>
+          <t>https://leetcode.com/problems/fibonacci-number/</t>
         </is>
       </c>
       <c r="G11" s="20" t="inlineStr">
@@ -1223,7 +1227,7 @@
           <t>29-07-2026</t>
         </is>
       </c>
-      <c r="L11" s="17" t="n"/>
+      <c r="L11" s="17" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="13" t="n">
@@ -1241,17 +1245,17 @@
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>Palindrome Number</t>
+          <t>Find Greatest Common Divisor of Array</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>Digit Extraction</t>
+          <t>Euclidean GCD</t>
         </is>
       </c>
       <c r="F12" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/palindrome-number/</t>
+          <t>https://leetcode.com/problems/find-greatest-common-divisor-of-array/</t>
         </is>
       </c>
       <c r="G12" s="16" t="inlineStr">
@@ -1266,20 +1270,12 @@
       </c>
       <c r="I12" s="13" t="inlineStr">
         <is>
-          <t>23-07-2026</t>
-        </is>
-      </c>
-      <c r="J12" s="13" t="inlineStr">
-        <is>
-          <t>24-07-2026</t>
-        </is>
-      </c>
-      <c r="K12" s="13" t="inlineStr">
-        <is>
-          <t>30-07-2026</t>
-        </is>
-      </c>
-      <c r="L12" s="13" t="n"/>
+          <t>10-09-2026</t>
+        </is>
+      </c>
+      <c r="J12" s="13" t="inlineStr"/>
+      <c r="K12" s="13" t="inlineStr"/>
+      <c r="L12" s="13" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="17" t="n">
@@ -1297,22 +1293,22 @@
       </c>
       <c r="D13" s="18" t="inlineStr">
         <is>
-          <t>Reverse Integer</t>
+          <t>Maximum 69 Number</t>
         </is>
       </c>
       <c r="E13" s="18" t="inlineStr">
         <is>
-          <t>Digit Extraction</t>
+          <t>Greedy / String Replace</t>
         </is>
       </c>
       <c r="F13" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/reverse-integer/</t>
-        </is>
-      </c>
-      <c r="G13" s="22" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>https://leetcode.com/problems/maximum-69-number/</t>
+        </is>
+      </c>
+      <c r="G13" s="20" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="H13" s="18" t="inlineStr">
@@ -1322,20 +1318,12 @@
       </c>
       <c r="I13" s="17" t="inlineStr">
         <is>
-          <t>23-07-2026</t>
-        </is>
-      </c>
-      <c r="J13" s="17" t="inlineStr">
-        <is>
-          <t>24-07-2026</t>
-        </is>
-      </c>
-      <c r="K13" s="17" t="inlineStr">
-        <is>
-          <t>30-07-2026</t>
-        </is>
-      </c>
-      <c r="L13" s="17" t="n"/>
+          <t>31-08-2026</t>
+        </is>
+      </c>
+      <c r="J13" s="17" t="inlineStr"/>
+      <c r="K13" s="17" t="inlineStr"/>
+      <c r="L13" s="17" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="13" t="n">
@@ -1353,22 +1341,22 @@
       </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
-          <t>Count Primes</t>
+          <t>Number of Steps to Reduce a Number to Zero</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Sieve of Eratosthenes</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F14" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/count-primes/</t>
-        </is>
-      </c>
-      <c r="G14" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>https://leetcode.com/problems/number-of-steps-to-reduce-a-number-to-zero/</t>
+        </is>
+      </c>
+      <c r="G14" s="16" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="H14" s="14" t="inlineStr">
@@ -1378,20 +1366,20 @@
       </c>
       <c r="I14" s="13" t="inlineStr">
         <is>
-          <t>23-07-2026</t>
+          <t>28-07-2026</t>
         </is>
       </c>
       <c r="J14" s="13" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="K14" s="13" t="inlineStr">
         <is>
-          <t>30-07-2026</t>
-        </is>
-      </c>
-      <c r="L14" s="13" t="n"/>
+          <t>03-07-2026</t>
+        </is>
+      </c>
+      <c r="L14" s="13" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="17" t="n">
@@ -1409,17 +1397,17 @@
       </c>
       <c r="D15" s="18" t="inlineStr">
         <is>
-          <t>Base 7</t>
+          <t>Palindrome Number</t>
         </is>
       </c>
       <c r="E15" s="18" t="inlineStr">
         <is>
-          <t>Base Conversion</t>
+          <t>Digit Extraction</t>
         </is>
       </c>
       <c r="F15" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/base-7/</t>
+          <t>https://leetcode.com/problems/palindrome-number/</t>
         </is>
       </c>
       <c r="G15" s="20" t="inlineStr">
@@ -1434,20 +1422,20 @@
       </c>
       <c r="I15" s="17" t="inlineStr">
         <is>
+          <t>23-07-2026</t>
+        </is>
+      </c>
+      <c r="J15" s="17" t="inlineStr">
+        <is>
           <t>24-07-2026</t>
         </is>
       </c>
-      <c r="J15" s="17" t="inlineStr">
-        <is>
-          <t>25-07-2026</t>
-        </is>
-      </c>
       <c r="K15" s="17" t="inlineStr">
         <is>
-          <t>31-07-2026</t>
-        </is>
-      </c>
-      <c r="L15" s="17" t="n"/>
+          <t>30-07-2026</t>
+        </is>
+      </c>
+      <c r="L15" s="17" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="13" t="n">
@@ -1465,17 +1453,17 @@
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
-          <t>Add Binary</t>
+          <t>Power of Two</t>
         </is>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Bitwise or Repeated Division</t>
         </is>
       </c>
       <c r="F16" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/add-binary/</t>
+          <t>https://leetcode.com/problems/power-of-two/</t>
         </is>
       </c>
       <c r="G16" s="16" t="inlineStr">
@@ -1490,20 +1478,20 @@
       </c>
       <c r="I16" s="13" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>28-07-2026</t>
         </is>
       </c>
       <c r="J16" s="13" t="inlineStr">
         <is>
-          <t>25-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="K16" s="13" t="inlineStr">
         <is>
-          <t>31-07-2026</t>
-        </is>
-      </c>
-      <c r="L16" s="13" t="n"/>
+          <t>03-07-2026</t>
+        </is>
+      </c>
+      <c r="L16" s="13" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="17" t="n">
@@ -1516,27 +1504,27 @@
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>Brainteaser</t>
+          <t>Basic Math &amp; Loops</t>
         </is>
       </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>Nim Game</t>
+          <t>Reverse Integer</t>
         </is>
       </c>
       <c r="E17" s="18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Digit Extraction</t>
         </is>
       </c>
       <c r="F17" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/nim-game/</t>
-        </is>
-      </c>
-      <c r="G17" s="20" t="inlineStr">
-        <is>
-          <t>Easy</t>
+          <t>https://leetcode.com/problems/reverse-integer/</t>
+        </is>
+      </c>
+      <c r="G17" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H17" s="18" t="inlineStr">
@@ -1546,11 +1534,19 @@
       </c>
       <c r="I17" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J17" s="17" t="inlineStr"/>
-      <c r="K17" s="17" t="inlineStr"/>
+          <t>23-07-2026</t>
+        </is>
+      </c>
+      <c r="J17" s="17" t="inlineStr">
+        <is>
+          <t>24-07-2026</t>
+        </is>
+      </c>
+      <c r="K17" s="17" t="inlineStr">
+        <is>
+          <t>30-07-2026</t>
+        </is>
+      </c>
       <c r="L17" s="17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1559,32 +1555,32 @@
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>Strings</t>
+          <t>Math &amp; Basics</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>Sliding Window</t>
+          <t>Basic Math &amp; Loops</t>
         </is>
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
-          <t>Shortest and Lexicographically Smallest Beautiful String</t>
+          <t>Subtract the Product and Sum of Digits of an Integer</t>
         </is>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Sliding Window</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F18" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/shortest-and-lexicographically-smallest-beautiful-string/</t>
-        </is>
-      </c>
-      <c r="G18" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>https://leetcode.com/problems/subtract-the-product-and-sum-of-digits-of-an-integer/</t>
+        </is>
+      </c>
+      <c r="G18" s="16" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="H18" s="14" t="inlineStr">
@@ -1594,12 +1590,20 @@
       </c>
       <c r="I18" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J18" s="13" t="n"/>
-      <c r="K18" s="13" t="n"/>
-      <c r="L18" s="13" t="n"/>
+          <t>28-07-2026</t>
+        </is>
+      </c>
+      <c r="J18" s="13" t="inlineStr">
+        <is>
+          <t>29-07-2026</t>
+        </is>
+      </c>
+      <c r="K18" s="13" t="inlineStr">
+        <is>
+          <t>03-07-2026</t>
+        </is>
+      </c>
+      <c r="L18" s="13" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="17" t="n">
@@ -1607,32 +1611,32 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>Strings</t>
+          <t>Math &amp; Basics</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>Sliding Window</t>
+          <t>Brainteaser</t>
         </is>
       </c>
       <c r="D19" s="18" t="inlineStr">
         <is>
-          <t>Longest Substring Without Repeating Characters</t>
+          <t>Nim Game</t>
         </is>
       </c>
       <c r="E19" s="18" t="inlineStr">
         <is>
-          <t>Sliding Window</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F19" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/longest-substring-without-repeating-characters/</t>
-        </is>
-      </c>
-      <c r="G19" s="22" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>https://leetcode.com/problems/nim-game/</t>
+        </is>
+      </c>
+      <c r="G19" s="20" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="H19" s="18" t="inlineStr">
@@ -1642,12 +1646,12 @@
       </c>
       <c r="I19" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J19" s="17" t="n"/>
-      <c r="K19" s="17" t="n"/>
-      <c r="L19" s="17" t="n"/>
+          <t>15-08-2026</t>
+        </is>
+      </c>
+      <c r="J19" s="17" t="inlineStr"/>
+      <c r="K19" s="17" t="inlineStr"/>
+      <c r="L19" s="17" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="13" t="n">
@@ -1655,27 +1659,27 @@
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>Strings</t>
+          <t>Math &amp; Basics</t>
         </is>
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>String Manipulation</t>
+          <t>Math &amp; Combinatorics</t>
         </is>
       </c>
       <c r="D20" s="14" t="inlineStr">
         <is>
-          <t>Score of a String</t>
+          <t>Count Commas in Range</t>
         </is>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>ASCII Values</t>
+          <t>Math / Range Counting</t>
         </is>
       </c>
       <c r="F20" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/score-of-a-string/</t>
+          <t>https://leetcode.com/problems/count-commas-in-range/</t>
         </is>
       </c>
       <c r="G20" s="16" t="inlineStr">
@@ -1690,12 +1694,12 @@
       </c>
       <c r="I20" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J20" s="13" t="n"/>
-      <c r="K20" s="13" t="n"/>
-      <c r="L20" s="13" t="n"/>
+          <t>08-09-2026</t>
+        </is>
+      </c>
+      <c r="J20" s="13" t="inlineStr"/>
+      <c r="K20" s="13" t="inlineStr"/>
+      <c r="L20" s="13" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="17" t="n">
@@ -1703,32 +1707,32 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>Strings</t>
+          <t>Math &amp; Basics</t>
         </is>
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>String Manipulation</t>
+          <t>Math &amp; Combinatorics</t>
         </is>
       </c>
       <c r="D21" s="18" t="inlineStr">
         <is>
-          <t>Defanging an IP Address</t>
+          <t>Count Commas in Range II</t>
         </is>
       </c>
       <c r="E21" s="18" t="inlineStr">
         <is>
-          <t>String Replace</t>
+          <t>Digit Math / Intervals</t>
         </is>
       </c>
       <c r="F21" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/defanging-an-ip-address/</t>
-        </is>
-      </c>
-      <c r="G21" s="20" t="inlineStr">
-        <is>
-          <t>Easy</t>
+          <t>https://leetcode.com/problems/count-commas-in-range-ii/</t>
+        </is>
+      </c>
+      <c r="G21" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H21" s="18" t="inlineStr">
@@ -1738,12 +1742,12 @@
       </c>
       <c r="I21" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J21" s="17" t="n"/>
-      <c r="K21" s="17" t="n"/>
-      <c r="L21" s="17" t="n"/>
+          <t>09-09-2026</t>
+        </is>
+      </c>
+      <c r="J21" s="17" t="inlineStr"/>
+      <c r="K21" s="17" t="inlineStr"/>
+      <c r="L21" s="17" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="13" t="n">
@@ -1756,27 +1760,27 @@
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>String Manipulation</t>
+          <t>Sliding Window</t>
         </is>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>Goal Parser Interpretation</t>
+          <t>Longest Substring Without Repeating Characters</t>
         </is>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>String Replace</t>
+          <t>Sliding Window</t>
         </is>
       </c>
       <c r="F22" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/goal-parser-interpretation/</t>
-        </is>
-      </c>
-      <c r="G22" s="16" t="inlineStr">
-        <is>
-          <t>Easy</t>
+          <t>https://leetcode.com/problems/longest-substring-without-repeating-characters/</t>
+        </is>
+      </c>
+      <c r="G22" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H22" s="14" t="inlineStr">
@@ -1786,12 +1790,12 @@
       </c>
       <c r="I22" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J22" s="13" t="n"/>
-      <c r="K22" s="13" t="n"/>
-      <c r="L22" s="13" t="n"/>
+          <t>23-08-2026</t>
+        </is>
+      </c>
+      <c r="J22" s="13" t="inlineStr"/>
+      <c r="K22" s="13" t="inlineStr"/>
+      <c r="L22" s="13" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="17" t="n">
@@ -1804,27 +1808,27 @@
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>String Manipulation</t>
+          <t>Sliding Window</t>
         </is>
       </c>
       <c r="D23" s="18" t="inlineStr">
         <is>
-          <t>Length of Last Word</t>
+          <t>Shortest and Lexicographically Smallest Beautiful String</t>
         </is>
       </c>
       <c r="E23" s="18" t="inlineStr">
         <is>
-          <t>Iteration</t>
+          <t>Sliding Window</t>
         </is>
       </c>
       <c r="F23" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/length-of-last-word/</t>
-        </is>
-      </c>
-      <c r="G23" s="20" t="inlineStr">
-        <is>
-          <t>Easy</t>
+          <t>https://leetcode.com/problems/shortest-and-lexicographically-smallest-beautiful-string/</t>
+        </is>
+      </c>
+      <c r="G23" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H23" s="18" t="inlineStr">
@@ -1834,12 +1838,12 @@
       </c>
       <c r="I23" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J23" s="17" t="n"/>
-      <c r="K23" s="17" t="n"/>
-      <c r="L23" s="17" t="n"/>
+          <t>26-08-2026</t>
+        </is>
+      </c>
+      <c r="J23" s="17" t="inlineStr"/>
+      <c r="K23" s="17" t="inlineStr"/>
+      <c r="L23" s="17" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="13" t="n">
@@ -1857,17 +1861,17 @@
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
-          <t>Roman to Integer</t>
+          <t>Defanging an IP Address</t>
         </is>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>HashMap</t>
+          <t>String Replace</t>
         </is>
       </c>
       <c r="F24" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/roman-to-integer/</t>
+          <t>https://leetcode.com/problems/defanging-an-ip-address/</t>
         </is>
       </c>
       <c r="G24" s="16" t="inlineStr">
@@ -1882,12 +1886,12 @@
       </c>
       <c r="I24" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J24" s="13" t="n"/>
-      <c r="K24" s="13" t="n"/>
-      <c r="L24" s="13" t="n"/>
+          <t>04-08-2026</t>
+        </is>
+      </c>
+      <c r="J24" s="13" t="inlineStr"/>
+      <c r="K24" s="13" t="inlineStr"/>
+      <c r="L24" s="13" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="17" t="n">
@@ -1905,7 +1909,7 @@
       </c>
       <c r="D25" s="18" t="inlineStr">
         <is>
-          <t>Longest Common Prefix</t>
+          <t>Final Value of Variable After Performing Operations</t>
         </is>
       </c>
       <c r="E25" s="18" t="inlineStr">
@@ -1915,7 +1919,7 @@
       </c>
       <c r="F25" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/longest-common-prefix/</t>
+          <t>https://leetcode.com/problems/final-value-of-variable-after-performing-operations/</t>
         </is>
       </c>
       <c r="G25" s="20" t="inlineStr">
@@ -1930,12 +1934,12 @@
       </c>
       <c r="I25" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J25" s="17" t="n"/>
-      <c r="K25" s="17" t="n"/>
-      <c r="L25" s="17" t="n"/>
+          <t>24-08-2026</t>
+        </is>
+      </c>
+      <c r="J25" s="17" t="inlineStr"/>
+      <c r="K25" s="17" t="inlineStr"/>
+      <c r="L25" s="17" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="13" t="n">
@@ -1953,17 +1957,17 @@
       </c>
       <c r="D26" s="14" t="inlineStr">
         <is>
-          <t>Final Value of Variable After Performing Operations</t>
+          <t>Goal Parser Interpretation</t>
         </is>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>Iteration</t>
+          <t>String Replace</t>
         </is>
       </c>
       <c r="F26" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/final-value-of-variable-after-performing-operations/</t>
+          <t>https://leetcode.com/problems/goal-parser-interpretation/</t>
         </is>
       </c>
       <c r="G26" s="16" t="inlineStr">
@@ -1978,12 +1982,12 @@
       </c>
       <c r="I26" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J26" s="13" t="n"/>
-      <c r="K26" s="13" t="n"/>
-      <c r="L26" s="13" t="n"/>
+          <t>04-08-2026</t>
+        </is>
+      </c>
+      <c r="J26" s="13" t="inlineStr"/>
+      <c r="K26" s="13" t="inlineStr"/>
+      <c r="L26" s="13" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="17" t="n">
@@ -2026,12 +2030,12 @@
       </c>
       <c r="I27" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J27" s="17" t="n"/>
-      <c r="K27" s="17" t="n"/>
-      <c r="L27" s="17" t="n"/>
+          <t>20-08-2026</t>
+        </is>
+      </c>
+      <c r="J27" s="17" t="inlineStr"/>
+      <c r="K27" s="17" t="inlineStr"/>
+      <c r="L27" s="17" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="13" t="n">
@@ -2044,22 +2048,22 @@
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>String Matching</t>
+          <t>String Manipulation</t>
         </is>
       </c>
       <c r="D28" s="14" t="inlineStr">
         <is>
-          <t>Find the Index of the First Occurrence in a String</t>
+          <t>Length of Last Word</t>
         </is>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Iteration</t>
         </is>
       </c>
       <c r="F28" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/find-the-index-of-the-first-occurrence-in-a-string/</t>
+          <t>https://leetcode.com/problems/length-of-last-word/</t>
         </is>
       </c>
       <c r="G28" s="16" t="inlineStr">
@@ -2074,7 +2078,7 @@
       </c>
       <c r="I28" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
+          <t>10-08-2026</t>
         </is>
       </c>
       <c r="J28" s="13" t="inlineStr"/>
@@ -2092,22 +2096,22 @@
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>Two Pointers</t>
+          <t>String Manipulation</t>
         </is>
       </c>
       <c r="D29" s="18" t="inlineStr">
         <is>
-          <t>Valid Palindrome</t>
+          <t>Longest Common Prefix</t>
         </is>
       </c>
       <c r="E29" s="18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Iteration</t>
         </is>
       </c>
       <c r="F29" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/valid-palindrome/</t>
+          <t>https://leetcode.com/problems/longest-common-prefix/</t>
         </is>
       </c>
       <c r="G29" s="20" t="inlineStr">
@@ -2135,27 +2139,27 @@
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>Arrays</t>
+          <t>Strings</t>
         </is>
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>Basic Array Traversal</t>
+          <t>String Manipulation</t>
         </is>
       </c>
       <c r="D30" s="14" t="inlineStr">
         <is>
-          <t>Build Array from Permutation</t>
+          <t>Roman to Integer</t>
         </is>
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>HashMap</t>
         </is>
       </c>
       <c r="F30" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/build-array-from-permutation/</t>
+          <t>https://leetcode.com/problems/roman-to-integer/</t>
         </is>
       </c>
       <c r="G30" s="16" t="inlineStr">
@@ -2170,24 +2174,12 @@
       </c>
       <c r="I30" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J30" s="13" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="K30" s="13" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="L30" s="13" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
+          <t>07-08-2026</t>
+        </is>
+      </c>
+      <c r="J30" s="13" t="inlineStr"/>
+      <c r="K30" s="13" t="inlineStr"/>
+      <c r="L30" s="13" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="17" t="n">
@@ -2195,27 +2187,27 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>Arrays</t>
+          <t>Strings</t>
         </is>
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>Basic Array Traversal</t>
+          <t>String Manipulation</t>
         </is>
       </c>
       <c r="D31" s="18" t="inlineStr">
         <is>
-          <t>Concatenation of Array</t>
+          <t>Score of a String</t>
         </is>
       </c>
       <c r="E31" s="18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ASCII Values</t>
         </is>
       </c>
       <c r="F31" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/concatenation-of-array/</t>
+          <t>https://leetcode.com/problems/score-of-a-string/</t>
         </is>
       </c>
       <c r="G31" s="20" t="inlineStr">
@@ -2230,16 +2222,12 @@
       </c>
       <c r="I31" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J31" s="17" t="inlineStr">
-        <is>
-          <t>31-07-2026</t>
-        </is>
-      </c>
-      <c r="K31" s="17" t="n"/>
-      <c r="L31" s="17" t="n"/>
+          <t>04-08-2026</t>
+        </is>
+      </c>
+      <c r="J31" s="17" t="inlineStr"/>
+      <c r="K31" s="17" t="inlineStr"/>
+      <c r="L31" s="17" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="13" t="n">
@@ -2247,27 +2235,27 @@
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>Arrays</t>
+          <t>Strings</t>
         </is>
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>Basic Array Traversal</t>
+          <t>String Matching</t>
         </is>
       </c>
       <c r="D32" s="14" t="inlineStr">
         <is>
-          <t>Shuffle the Array</t>
+          <t>Find the Index of the First Occurrence in a String</t>
         </is>
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
-          <t>Array Indexing</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F32" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/shuffle-the-array/</t>
+          <t>https://leetcode.com/problems/find-the-index-of-the-first-occurrence-in-a-string/</t>
         </is>
       </c>
       <c r="G32" s="16" t="inlineStr">
@@ -2282,12 +2270,12 @@
       </c>
       <c r="I32" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J32" s="13" t="n"/>
-      <c r="K32" s="13" t="n"/>
-      <c r="L32" s="13" t="n"/>
+          <t>18-08-2026</t>
+        </is>
+      </c>
+      <c r="J32" s="13" t="inlineStr"/>
+      <c r="K32" s="13" t="inlineStr"/>
+      <c r="L32" s="13" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="17" t="n">
@@ -2295,27 +2283,27 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>Arrays</t>
+          <t>Strings</t>
         </is>
       </c>
       <c r="C33" s="18" t="inlineStr">
         <is>
-          <t>Basic Array Traversal</t>
+          <t>Two Pointers</t>
         </is>
       </c>
       <c r="D33" s="18" t="inlineStr">
         <is>
-          <t>Kids With the Greatest Number of Candies</t>
+          <t>Valid Palindrome</t>
         </is>
       </c>
       <c r="E33" s="18" t="inlineStr">
         <is>
-          <t>Find Max &amp; Loop</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F33" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/kids-with-the-greatest-number-of-candies/</t>
+          <t>https://leetcode.com/problems/valid-palindrome/</t>
         </is>
       </c>
       <c r="G33" s="20" t="inlineStr">
@@ -2323,11 +2311,19 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H33" s="18" t="n"/>
-      <c r="I33" s="17" t="n"/>
-      <c r="J33" s="17" t="n"/>
-      <c r="K33" s="17" t="n"/>
-      <c r="L33" s="17" t="n"/>
+      <c r="H33" s="18" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I33" s="17" t="inlineStr">
+        <is>
+          <t>14-08-2026</t>
+        </is>
+      </c>
+      <c r="J33" s="17" t="inlineStr"/>
+      <c r="K33" s="17" t="inlineStr"/>
+      <c r="L33" s="17" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="13" t="n">
@@ -2345,17 +2341,17 @@
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>Richest Customer Wealth</t>
+          <t>Add to Array-Form of Integer</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>2D Array Traversal</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F34" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/richest-customer-wealth/</t>
+          <t>https://leetcode.com/problems/add-to-array-form-of-integer/</t>
         </is>
       </c>
       <c r="G34" s="16" t="inlineStr">
@@ -2363,19 +2359,11 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H34" s="14" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="I34" s="13" t="inlineStr">
-        <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J34" s="13" t="n"/>
-      <c r="K34" s="13" t="n"/>
-      <c r="L34" s="13" t="n"/>
+      <c r="H34" s="14" t="inlineStr"/>
+      <c r="I34" s="13" t="inlineStr"/>
+      <c r="J34" s="13" t="inlineStr"/>
+      <c r="K34" s="13" t="inlineStr"/>
+      <c r="L34" s="13" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="17" t="n">
@@ -2393,17 +2381,17 @@
       </c>
       <c r="D35" s="18" t="inlineStr">
         <is>
-          <t>Running Sum of 1d Array</t>
+          <t>Best Time to Buy and Sell Stock</t>
         </is>
       </c>
       <c r="E35" s="18" t="inlineStr">
         <is>
-          <t>Prefix Sum</t>
+          <t>Track Min Value</t>
         </is>
       </c>
       <c r="F35" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/running-sum-of-1d-array/</t>
+          <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock/</t>
         </is>
       </c>
       <c r="G35" s="20" t="inlineStr">
@@ -2418,12 +2406,16 @@
       </c>
       <c r="I35" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J35" s="17" t="n"/>
-      <c r="K35" s="17" t="n"/>
-      <c r="L35" s="17" t="n"/>
+          <t>29-07-2026</t>
+        </is>
+      </c>
+      <c r="J35" s="17" t="inlineStr">
+        <is>
+          <t>30-07-2026</t>
+        </is>
+      </c>
+      <c r="K35" s="17" t="inlineStr"/>
+      <c r="L35" s="17" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="13" t="n">
@@ -2441,17 +2433,17 @@
       </c>
       <c r="D36" s="14" t="inlineStr">
         <is>
-          <t>Find Pivot Index</t>
+          <t>Build Array from Permutation</t>
         </is>
       </c>
       <c r="E36" s="14" t="inlineStr">
         <is>
-          <t>Prefix Sum</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F36" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/find-pivot-index/</t>
+          <t>https://leetcode.com/problems/build-array-from-permutation/</t>
         </is>
       </c>
       <c r="G36" s="16" t="inlineStr">
@@ -2466,12 +2458,24 @@
       </c>
       <c r="I36" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J36" s="13" t="n"/>
-      <c r="K36" s="13" t="n"/>
-      <c r="L36" s="13" t="n"/>
+          <t>01-08-2026</t>
+        </is>
+      </c>
+      <c r="J36" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K36" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L36" s="13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="17" t="n">
@@ -2489,17 +2493,17 @@
       </c>
       <c r="D37" s="18" t="inlineStr">
         <is>
-          <t>Missing Number</t>
+          <t>Concatenation of Array</t>
         </is>
       </c>
       <c r="E37" s="18" t="inlineStr">
         <is>
-          <t>Gauss Formula or XOR</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F37" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/missing-number/</t>
+          <t>https://leetcode.com/problems/concatenation-of-array/</t>
         </is>
       </c>
       <c r="G37" s="20" t="inlineStr">
@@ -2514,20 +2518,16 @@
       </c>
       <c r="I37" s="17" t="inlineStr">
         <is>
-          <t>22-07-2026</t>
+          <t>20-08-2026</t>
         </is>
       </c>
       <c r="J37" s="17" t="inlineStr">
         <is>
-          <t>23-07-2026</t>
-        </is>
-      </c>
-      <c r="K37" s="17" t="inlineStr">
-        <is>
-          <t>29-07-2026</t>
-        </is>
-      </c>
-      <c r="L37" s="17" t="n"/>
+          <t>31-07-2026</t>
+        </is>
+      </c>
+      <c r="K37" s="17" t="inlineStr"/>
+      <c r="L37" s="17" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="13" t="n">
@@ -2545,17 +2545,17 @@
       </c>
       <c r="D38" s="14" t="inlineStr">
         <is>
-          <t>Add to Array-Form of Integer</t>
+          <t>Find Pivot Index</t>
         </is>
       </c>
       <c r="E38" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Prefix Sum</t>
         </is>
       </c>
       <c r="F38" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/add-to-array-form-of-integer/</t>
+          <t>https://leetcode.com/problems/find-pivot-index/</t>
         </is>
       </c>
       <c r="G38" s="16" t="inlineStr">
@@ -2563,11 +2563,19 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H38" s="14" t="n"/>
-      <c r="I38" s="13" t="n"/>
-      <c r="J38" s="13" t="n"/>
-      <c r="K38" s="13" t="n"/>
-      <c r="L38" s="13" t="n"/>
+      <c r="H38" s="14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I38" s="13" t="inlineStr">
+        <is>
+          <t>03-08-2026</t>
+        </is>
+      </c>
+      <c r="J38" s="13" t="inlineStr"/>
+      <c r="K38" s="13" t="inlineStr"/>
+      <c r="L38" s="13" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="17" t="n">
@@ -2585,17 +2593,17 @@
       </c>
       <c r="D39" s="18" t="inlineStr">
         <is>
-          <t>Best Time to Buy and Sell Stock</t>
+          <t>Kids With the Greatest Number of Candies</t>
         </is>
       </c>
       <c r="E39" s="18" t="inlineStr">
         <is>
-          <t>Track Min Value</t>
+          <t>Find Max &amp; Loop</t>
         </is>
       </c>
       <c r="F39" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock/</t>
+          <t>https://leetcode.com/problems/kids-with-the-greatest-number-of-candies/</t>
         </is>
       </c>
       <c r="G39" s="20" t="inlineStr">
@@ -2603,23 +2611,11 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H39" s="18" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="I39" s="17" t="inlineStr">
-        <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J39" s="17" t="inlineStr">
-        <is>
-          <t>30-07-2026</t>
-        </is>
-      </c>
-      <c r="K39" s="17" t="n"/>
-      <c r="L39" s="17" t="n"/>
+      <c r="H39" s="18" t="inlineStr"/>
+      <c r="I39" s="17" t="inlineStr"/>
+      <c r="J39" s="17" t="inlineStr"/>
+      <c r="K39" s="17" t="inlineStr"/>
+      <c r="L39" s="17" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="13" t="n">
@@ -2637,17 +2633,17 @@
       </c>
       <c r="D40" s="14" t="inlineStr">
         <is>
-          <t>Third Maximum Number</t>
+          <t>Missing Number</t>
         </is>
       </c>
       <c r="E40" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Gauss Formula or XOR</t>
         </is>
       </c>
       <c r="F40" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/third-maximum-number/</t>
+          <t>https://leetcode.com/problems/missing-number/</t>
         </is>
       </c>
       <c r="G40" s="16" t="inlineStr">
@@ -2662,11 +2658,19 @@
       </c>
       <c r="I40" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J40" s="13" t="inlineStr"/>
-      <c r="K40" s="13" t="inlineStr"/>
+          <t>22-07-2026</t>
+        </is>
+      </c>
+      <c r="J40" s="13" t="inlineStr">
+        <is>
+          <t>23-07-2026</t>
+        </is>
+      </c>
+      <c r="K40" s="13" t="inlineStr">
+        <is>
+          <t>29-07-2026</t>
+        </is>
+      </c>
       <c r="L40" s="13" t="inlineStr"/>
     </row>
     <row r="41">
@@ -2680,22 +2684,22 @@
       </c>
       <c r="C41" s="18" t="inlineStr">
         <is>
-          <t>Bit Manipulation</t>
+          <t>Basic Array Traversal</t>
         </is>
       </c>
       <c r="D41" s="18" t="inlineStr">
         <is>
-          <t>XOR Operation in an Array</t>
+          <t>Richest Customer Wealth</t>
         </is>
       </c>
       <c r="E41" s="18" t="inlineStr">
         <is>
-          <t>Bitwise</t>
+          <t>2D Array Traversal</t>
         </is>
       </c>
       <c r="F41" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/xor-operation-in-an-array/</t>
+          <t>https://leetcode.com/problems/richest-customer-wealth/</t>
         </is>
       </c>
       <c r="G41" s="20" t="inlineStr">
@@ -2710,12 +2714,12 @@
       </c>
       <c r="I41" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J41" s="17" t="n"/>
-      <c r="K41" s="17" t="n"/>
-      <c r="L41" s="17" t="n"/>
+          <t>02-08-2026</t>
+        </is>
+      </c>
+      <c r="J41" s="17" t="inlineStr"/>
+      <c r="K41" s="17" t="inlineStr"/>
+      <c r="L41" s="17" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="13" t="n">
@@ -2728,22 +2732,22 @@
       </c>
       <c r="C42" s="14" t="inlineStr">
         <is>
-          <t>Logic/Math</t>
+          <t>Basic Array Traversal</t>
         </is>
       </c>
       <c r="D42" s="14" t="inlineStr">
         <is>
-          <t>Find All Numbers Disappeared in an Array</t>
+          <t>Running Sum of 1d Array</t>
         </is>
       </c>
       <c r="E42" s="14" t="inlineStr">
         <is>
-          <t>Array Iteration</t>
+          <t>Prefix Sum</t>
         </is>
       </c>
       <c r="F42" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/find-all-numbers-disappeared-in-an-array/</t>
+          <t>https://leetcode.com/problems/running-sum-of-1d-array/</t>
         </is>
       </c>
       <c r="G42" s="16" t="inlineStr">
@@ -2751,11 +2755,19 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H42" s="14" t="n"/>
-      <c r="I42" s="13" t="n"/>
-      <c r="J42" s="13" t="n"/>
-      <c r="K42" s="13" t="n"/>
-      <c r="L42" s="13" t="n"/>
+      <c r="H42" s="14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I42" s="13" t="inlineStr">
+        <is>
+          <t>03-08-2026</t>
+        </is>
+      </c>
+      <c r="J42" s="13" t="inlineStr"/>
+      <c r="K42" s="13" t="inlineStr"/>
+      <c r="L42" s="13" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="17" t="n">
@@ -2768,27 +2780,27 @@
       </c>
       <c r="C43" s="18" t="inlineStr">
         <is>
-          <t>Prefix Sum</t>
+          <t>Basic Array Traversal</t>
         </is>
       </c>
       <c r="D43" s="18" t="inlineStr">
         <is>
-          <t>Minimum Operations to Make Array Sum Divisible by K</t>
+          <t>Shuffle the Array</t>
         </is>
       </c>
       <c r="E43" s="18" t="inlineStr">
         <is>
-          <t>HashMap</t>
+          <t>Array Indexing</t>
         </is>
       </c>
       <c r="F43" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/minimum-operations-to-make-array-sum-divisible-by-k/</t>
-        </is>
-      </c>
-      <c r="G43" s="22" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>https://leetcode.com/problems/shuffle-the-array/</t>
+        </is>
+      </c>
+      <c r="G43" s="20" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="H43" s="18" t="inlineStr">
@@ -2798,12 +2810,12 @@
       </c>
       <c r="I43" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J43" s="17" t="n"/>
-      <c r="K43" s="17" t="n"/>
-      <c r="L43" s="17" t="n"/>
+          <t>20-08-2026</t>
+        </is>
+      </c>
+      <c r="J43" s="17" t="inlineStr"/>
+      <c r="K43" s="17" t="inlineStr"/>
+      <c r="L43" s="17" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="13" t="n">
@@ -2816,34 +2828,42 @@
       </c>
       <c r="C44" s="14" t="inlineStr">
         <is>
-          <t>Span of Array</t>
+          <t>Basic Array Traversal</t>
         </is>
       </c>
       <c r="D44" s="14" t="inlineStr">
         <is>
-          <t>Find Minimum in Rotated Sorted Array</t>
+          <t>Smallest Stable Index I</t>
         </is>
       </c>
       <c r="E44" s="14" t="inlineStr">
         <is>
-          <t>Binary Search</t>
+          <t>Linear Scan / Brute Force</t>
         </is>
       </c>
       <c r="F44" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/find-minimum-in-rotated-sorted-array/</t>
-        </is>
-      </c>
-      <c r="G44" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H44" s="14" t="n"/>
-      <c r="I44" s="13" t="n"/>
-      <c r="J44" s="13" t="n"/>
-      <c r="K44" s="13" t="n"/>
-      <c r="L44" s="13" t="n"/>
+          <t>https://leetcode.com/problems/smallest-stable-index-i/</t>
+        </is>
+      </c>
+      <c r="G44" s="16" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H44" s="14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I44" s="13" t="inlineStr">
+        <is>
+          <t>04-09-2026</t>
+        </is>
+      </c>
+      <c r="J44" s="13" t="inlineStr"/>
+      <c r="K44" s="13" t="inlineStr"/>
+      <c r="L44" s="13" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="17" t="n">
@@ -2856,34 +2876,42 @@
       </c>
       <c r="C45" s="18" t="inlineStr">
         <is>
-          <t>Subarray</t>
+          <t>Basic Array Traversal</t>
         </is>
       </c>
       <c r="D45" s="18" t="inlineStr">
         <is>
-          <t>Maximum Subarray</t>
+          <t>Third Maximum Number</t>
         </is>
       </c>
       <c r="E45" s="18" t="inlineStr">
         <is>
-          <t>Kadanes Algorithm</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F45" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/maximum-subarray/</t>
-        </is>
-      </c>
-      <c r="G45" s="22" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H45" s="18" t="n"/>
-      <c r="I45" s="17" t="n"/>
-      <c r="J45" s="17" t="n"/>
-      <c r="K45" s="17" t="n"/>
-      <c r="L45" s="17" t="n"/>
+          <t>https://leetcode.com/problems/third-maximum-number/</t>
+        </is>
+      </c>
+      <c r="G45" s="20" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H45" s="18" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I45" s="17" t="inlineStr">
+        <is>
+          <t>16-08-2026</t>
+        </is>
+      </c>
+      <c r="J45" s="17" t="inlineStr"/>
+      <c r="K45" s="17" t="inlineStr"/>
+      <c r="L45" s="17" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="13" t="n">
@@ -2896,22 +2924,22 @@
       </c>
       <c r="C46" s="14" t="inlineStr">
         <is>
-          <t>Two Pointers</t>
+          <t>Basic Array Traversal</t>
         </is>
       </c>
       <c r="D46" s="14" t="inlineStr">
         <is>
-          <t>Remove Duplicates from Sorted Array</t>
+          <t>Unique 3-Digit Even Numbers</t>
         </is>
       </c>
       <c r="E46" s="14" t="inlineStr">
         <is>
-          <t>Two Pointers</t>
+          <t>Frequency Array / Counting</t>
         </is>
       </c>
       <c r="F46" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/remove-duplicates-from-sorted-array/</t>
+          <t>https://leetcode.com/problems/unique-3-digit-even-numbers/</t>
         </is>
       </c>
       <c r="G46" s="16" t="inlineStr">
@@ -2926,12 +2954,12 @@
       </c>
       <c r="I46" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J46" s="13" t="n"/>
-      <c r="K46" s="13" t="n"/>
-      <c r="L46" s="13" t="n"/>
+          <t>11-09-2026</t>
+        </is>
+      </c>
+      <c r="J46" s="13" t="inlineStr"/>
+      <c r="K46" s="13" t="inlineStr"/>
+      <c r="L46" s="13" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="17" t="n">
@@ -2944,22 +2972,22 @@
       </c>
       <c r="C47" s="18" t="inlineStr">
         <is>
-          <t>Two Pointers</t>
+          <t>Bit Manipulation</t>
         </is>
       </c>
       <c r="D47" s="18" t="inlineStr">
         <is>
-          <t>Max Consecutive Ones</t>
+          <t>XOR Operation in an Array</t>
         </is>
       </c>
       <c r="E47" s="18" t="inlineStr">
         <is>
-          <t>Two Pointers</t>
+          <t>Bitwise</t>
         </is>
       </c>
       <c r="F47" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/max-consecutive-ones/</t>
+          <t>https://leetcode.com/problems/xor-operation-in-an-array/</t>
         </is>
       </c>
       <c r="G47" s="20" t="inlineStr">
@@ -2974,12 +3002,12 @@
       </c>
       <c r="I47" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J47" s="17" t="n"/>
-      <c r="K47" s="17" t="n"/>
-      <c r="L47" s="17" t="n"/>
+          <t>22-08-2026</t>
+        </is>
+      </c>
+      <c r="J47" s="17" t="inlineStr"/>
+      <c r="K47" s="17" t="inlineStr"/>
+      <c r="L47" s="17" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="13" t="n">
@@ -2987,32 +3015,32 @@
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>Arrays - Two Pointers</t>
+          <t>Arrays</t>
         </is>
       </c>
       <c r="C48" s="14" t="inlineStr">
         <is>
-          <t>Two Pointers Technique</t>
+          <t>Grid / Matrix Traversal</t>
         </is>
       </c>
       <c r="D48" s="14" t="inlineStr">
         <is>
-          <t>Reverse String</t>
+          <t>Minimum Moves to Clean the Classroom</t>
         </is>
       </c>
       <c r="E48" s="14" t="inlineStr">
         <is>
-          <t>Two Pointers (Left/Right)</t>
+          <t>BFS / Simulation</t>
         </is>
       </c>
       <c r="F48" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/reverse-string/</t>
-        </is>
-      </c>
-      <c r="G48" s="16" t="inlineStr">
-        <is>
-          <t>Easy</t>
+          <t>https://leetcode.com/problems/minimum-moves-to-clean-the-classroom/</t>
+        </is>
+      </c>
+      <c r="G48" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H48" s="14" t="inlineStr">
@@ -3022,12 +3050,12 @@
       </c>
       <c r="I48" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J48" s="13" t="n"/>
-      <c r="K48" s="13" t="n"/>
-      <c r="L48" s="13" t="n"/>
+          <t>01-09-2026</t>
+        </is>
+      </c>
+      <c r="J48" s="13" t="inlineStr"/>
+      <c r="K48" s="13" t="inlineStr"/>
+      <c r="L48" s="13" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="17" t="n">
@@ -3035,27 +3063,27 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>Arrays - Two Pointers</t>
+          <t>Arrays</t>
         </is>
       </c>
       <c r="C49" s="18" t="inlineStr">
         <is>
-          <t>Two Pointers Technique</t>
+          <t>Logic/Math</t>
         </is>
       </c>
       <c r="D49" s="18" t="inlineStr">
         <is>
-          <t>Remove Element</t>
+          <t>Find All Numbers Disappeared in an Array</t>
         </is>
       </c>
       <c r="E49" s="18" t="inlineStr">
         <is>
-          <t>Two Pointers (Slow/Fast)</t>
+          <t>Array Iteration</t>
         </is>
       </c>
       <c r="F49" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/remove-element/</t>
+          <t>https://leetcode.com/problems/find-all-numbers-disappeared-in-an-array/</t>
         </is>
       </c>
       <c r="G49" s="20" t="inlineStr">
@@ -3063,11 +3091,11 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H49" s="18" t="n"/>
-      <c r="I49" s="17" t="n"/>
-      <c r="J49" s="17" t="n"/>
-      <c r="K49" s="17" t="n"/>
-      <c r="L49" s="17" t="n"/>
+      <c r="H49" s="18" t="inlineStr"/>
+      <c r="I49" s="17" t="inlineStr"/>
+      <c r="J49" s="17" t="inlineStr"/>
+      <c r="K49" s="17" t="inlineStr"/>
+      <c r="L49" s="17" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="13" t="n">
@@ -3075,27 +3103,27 @@
       </c>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>Arrays - Two Pointers</t>
+          <t>Arrays</t>
         </is>
       </c>
       <c r="C50" s="14" t="inlineStr">
         <is>
-          <t>Two Pointers Technique</t>
+          <t>Math &amp; Parity</t>
         </is>
       </c>
       <c r="D50" s="14" t="inlineStr">
         <is>
-          <t>Move Zeroes</t>
+          <t>Construct Uniform Parity Array I</t>
         </is>
       </c>
       <c r="E50" s="14" t="inlineStr">
         <is>
-          <t>Two Pointers (Slow/Fast)</t>
+          <t>Array Traversal</t>
         </is>
       </c>
       <c r="F50" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/move-zeroes/</t>
+          <t>https://leetcode.com/problems/construct-uniform-parity-array-i/</t>
         </is>
       </c>
       <c r="G50" s="16" t="inlineStr">
@@ -3110,20 +3138,12 @@
       </c>
       <c r="I50" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J50" s="13" t="inlineStr">
-        <is>
-          <t>26-07-2026</t>
-        </is>
-      </c>
-      <c r="K50" s="13" t="inlineStr">
-        <is>
-          <t>01-08-2026</t>
-        </is>
-      </c>
-      <c r="L50" s="13" t="n"/>
+          <t>02-09-2026</t>
+        </is>
+      </c>
+      <c r="J50" s="13" t="inlineStr"/>
+      <c r="K50" s="13" t="inlineStr"/>
+      <c r="L50" s="13" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="17" t="n">
@@ -3131,32 +3151,32 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>Arrays - Two Pointers</t>
+          <t>Arrays</t>
         </is>
       </c>
       <c r="C51" s="18" t="inlineStr">
         <is>
-          <t>Two Pointers Technique</t>
+          <t>Math &amp; Parity</t>
         </is>
       </c>
       <c r="D51" s="18" t="inlineStr">
         <is>
-          <t>Squares of a Sorted Array</t>
+          <t>Construct Uniform Parity Array II</t>
         </is>
       </c>
       <c r="E51" s="18" t="inlineStr">
         <is>
-          <t>Two Pointers (Left/Right)</t>
+          <t>Greedy / Parity Check</t>
         </is>
       </c>
       <c r="F51" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/squares-of-a-sorted-array/</t>
-        </is>
-      </c>
-      <c r="G51" s="20" t="inlineStr">
-        <is>
-          <t>Easy</t>
+          <t>https://leetcode.com/problems/construct-uniform-parity-array-ii/</t>
+        </is>
+      </c>
+      <c r="G51" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H51" s="18" t="inlineStr">
@@ -3166,20 +3186,12 @@
       </c>
       <c r="I51" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J51" s="17" t="inlineStr">
-        <is>
-          <t>27-07-2026</t>
-        </is>
-      </c>
-      <c r="K51" s="17" t="inlineStr">
-        <is>
-          <t>02-08-2026</t>
-        </is>
-      </c>
-      <c r="L51" s="17" t="n"/>
+          <t>03-09-2026</t>
+        </is>
+      </c>
+      <c r="J51" s="17" t="inlineStr"/>
+      <c r="K51" s="17" t="inlineStr"/>
+      <c r="L51" s="17" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="13" t="n">
@@ -3187,32 +3199,32 @@
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>Arrays - Two Pointers</t>
+          <t>Arrays</t>
         </is>
       </c>
       <c r="C52" s="14" t="inlineStr">
         <is>
-          <t>Two Pointers Technique</t>
+          <t>Prefix Sum</t>
         </is>
       </c>
       <c r="D52" s="14" t="inlineStr">
         <is>
-          <t>Trapping Rain Water</t>
+          <t>Minimum Operations to Make Array Sum Divisible by K</t>
         </is>
       </c>
       <c r="E52" s="14" t="inlineStr">
         <is>
-          <t>Two Pointers</t>
+          <t>HashMap</t>
         </is>
       </c>
       <c r="F52" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/trapping-rain-water/</t>
-        </is>
-      </c>
-      <c r="G52" s="24" t="inlineStr">
-        <is>
-          <t>Hard</t>
+          <t>https://leetcode.com/problems/minimum-operations-to-make-array-sum-divisible-by-k/</t>
+        </is>
+      </c>
+      <c r="G52" s="16" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="H52" s="14" t="inlineStr">
@@ -3222,12 +3234,12 @@
       </c>
       <c r="I52" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J52" s="13" t="n"/>
-      <c r="K52" s="13" t="n"/>
-      <c r="L52" s="13" t="n"/>
+          <t>28-08-2026</t>
+        </is>
+      </c>
+      <c r="J52" s="13" t="inlineStr"/>
+      <c r="K52" s="13" t="inlineStr"/>
+      <c r="L52" s="13" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="17" t="n">
@@ -3235,39 +3247,47 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>Binary Search &amp; Sort</t>
+          <t>Arrays</t>
         </is>
       </c>
       <c r="C53" s="18" t="inlineStr">
         <is>
-          <t>Binary Search</t>
+          <t>Prefix/Suffix Array</t>
         </is>
       </c>
       <c r="D53" s="18" t="inlineStr">
         <is>
-          <t>Find Target Indices After Sorting Array</t>
+          <t>Smallest Stable Index II</t>
         </is>
       </c>
       <c r="E53" s="18" t="inlineStr">
         <is>
-          <t>Sorting</t>
+          <t>Prefix &amp; Suffix Min/Max</t>
         </is>
       </c>
       <c r="F53" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/find-target-indices-after-sorting-array/</t>
-        </is>
-      </c>
-      <c r="G53" s="20" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="H53" s="18" t="n"/>
-      <c r="I53" s="17" t="n"/>
-      <c r="J53" s="17" t="n"/>
-      <c r="K53" s="17" t="n"/>
-      <c r="L53" s="17" t="n"/>
+          <t>https://leetcode.com/problems/smallest-stable-index-ii/</t>
+        </is>
+      </c>
+      <c r="G53" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H53" s="18" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I53" s="17" t="inlineStr">
+        <is>
+          <t>05-09-2026</t>
+        </is>
+      </c>
+      <c r="J53" s="17" t="inlineStr"/>
+      <c r="K53" s="17" t="inlineStr"/>
+      <c r="L53" s="17" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="13" t="n">
@@ -3275,47 +3295,39 @@
       </c>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>Binary Search &amp; Sort</t>
+          <t>Arrays</t>
         </is>
       </c>
       <c r="C54" s="14" t="inlineStr">
         <is>
+          <t>Span of Array</t>
+        </is>
+      </c>
+      <c r="D54" s="14" t="inlineStr">
+        <is>
+          <t>Find Minimum in Rotated Sorted Array</t>
+        </is>
+      </c>
+      <c r="E54" s="14" t="inlineStr">
+        <is>
           <t>Binary Search</t>
         </is>
       </c>
-      <c r="D54" s="14" t="inlineStr">
-        <is>
-          <t>Binary Search</t>
-        </is>
-      </c>
-      <c r="E54" s="14" t="inlineStr">
-        <is>
-          <t>Binary Search</t>
-        </is>
-      </c>
       <c r="F54" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/binary-search/</t>
-        </is>
-      </c>
-      <c r="G54" s="16" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="H54" s="14" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="I54" s="13" t="inlineStr">
-        <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J54" s="13" t="n"/>
-      <c r="K54" s="13" t="n"/>
-      <c r="L54" s="13" t="n"/>
+          <t>https://leetcode.com/problems/find-minimum-in-rotated-sorted-array/</t>
+        </is>
+      </c>
+      <c r="G54" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H54" s="14" t="inlineStr"/>
+      <c r="I54" s="13" t="inlineStr"/>
+      <c r="J54" s="13" t="inlineStr"/>
+      <c r="K54" s="13" t="inlineStr"/>
+      <c r="L54" s="13" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="17" t="n">
@@ -3323,47 +3335,39 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>Binary Search &amp; Sort</t>
+          <t>Arrays</t>
         </is>
       </c>
       <c r="C55" s="18" t="inlineStr">
         <is>
-          <t>Binary Search</t>
+          <t>Subarray</t>
         </is>
       </c>
       <c r="D55" s="18" t="inlineStr">
         <is>
-          <t>Search Insert Position</t>
+          <t>Maximum Subarray</t>
         </is>
       </c>
       <c r="E55" s="18" t="inlineStr">
         <is>
-          <t>Binary Search</t>
+          <t>Kadanes Algorithm</t>
         </is>
       </c>
       <c r="F55" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/search-insert-position/</t>
-        </is>
-      </c>
-      <c r="G55" s="20" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="H55" s="18" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="I55" s="17" t="inlineStr">
-        <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J55" s="17" t="n"/>
-      <c r="K55" s="17" t="n"/>
-      <c r="L55" s="17" t="n"/>
+          <t>https://leetcode.com/problems/maximum-subarray/</t>
+        </is>
+      </c>
+      <c r="G55" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H55" s="18" t="inlineStr"/>
+      <c r="I55" s="17" t="inlineStr"/>
+      <c r="J55" s="17" t="inlineStr"/>
+      <c r="K55" s="17" t="inlineStr"/>
+      <c r="L55" s="17" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="13" t="n">
@@ -3371,27 +3375,27 @@
       </c>
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t>Binary Search &amp; Sort</t>
+          <t>Arrays</t>
         </is>
       </c>
       <c r="C56" s="14" t="inlineStr">
         <is>
-          <t>Binary Search</t>
+          <t>Two Pointers</t>
         </is>
       </c>
       <c r="D56" s="14" t="inlineStr">
         <is>
-          <t>First Bad Version</t>
+          <t>Max Consecutive Ones</t>
         </is>
       </c>
       <c r="E56" s="14" t="inlineStr">
         <is>
-          <t>Binary Search</t>
+          <t>Two Pointers</t>
         </is>
       </c>
       <c r="F56" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/first-bad-version/</t>
+          <t>https://leetcode.com/problems/max-consecutive-ones/</t>
         </is>
       </c>
       <c r="G56" s="16" t="inlineStr">
@@ -3406,12 +3410,12 @@
       </c>
       <c r="I56" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J56" s="13" t="n"/>
-      <c r="K56" s="13" t="n"/>
-      <c r="L56" s="13" t="n"/>
+          <t>20-08-2026</t>
+        </is>
+      </c>
+      <c r="J56" s="13" t="inlineStr"/>
+      <c r="K56" s="13" t="inlineStr"/>
+      <c r="L56" s="13" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="17" t="n">
@@ -3419,27 +3423,27 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>Binary Search &amp; Sort</t>
+          <t>Arrays</t>
         </is>
       </c>
       <c r="C57" s="18" t="inlineStr">
         <is>
-          <t>Binary Search</t>
+          <t>Two Pointers</t>
         </is>
       </c>
       <c r="D57" s="18" t="inlineStr">
         <is>
-          <t>Sqrt(x)</t>
+          <t>Remove Duplicates from Sorted Array</t>
         </is>
       </c>
       <c r="E57" s="18" t="inlineStr">
         <is>
-          <t>Binary Search</t>
+          <t>Two Pointers</t>
         </is>
       </c>
       <c r="F57" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/sqrtx/</t>
+          <t>https://leetcode.com/problems/remove-duplicates-from-sorted-array/</t>
         </is>
       </c>
       <c r="G57" s="20" t="inlineStr">
@@ -3454,12 +3458,12 @@
       </c>
       <c r="I57" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J57" s="17" t="n"/>
-      <c r="K57" s="17" t="n"/>
-      <c r="L57" s="17" t="n"/>
+          <t>05-08-2026</t>
+        </is>
+      </c>
+      <c r="J57" s="17" t="inlineStr"/>
+      <c r="K57" s="17" t="inlineStr"/>
+      <c r="L57" s="17" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="13" t="n">
@@ -3467,27 +3471,27 @@
       </c>
       <c r="B58" s="14" t="inlineStr">
         <is>
-          <t>Hashing</t>
+          <t>Arrays - Two Pointers</t>
         </is>
       </c>
       <c r="C58" s="14" t="inlineStr">
         <is>
-          <t>HashMaps &amp; HashSets</t>
+          <t>Two Pointers Technique</t>
         </is>
       </c>
       <c r="D58" s="14" t="inlineStr">
         <is>
-          <t>Jewels and Stones</t>
+          <t>Move Zeroes</t>
         </is>
       </c>
       <c r="E58" s="14" t="inlineStr">
         <is>
-          <t>HashSet</t>
+          <t>Two Pointers (Slow/Fast)</t>
         </is>
       </c>
       <c r="F58" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/jewels-and-stones/</t>
+          <t>https://leetcode.com/problems/move-zeroes/</t>
         </is>
       </c>
       <c r="G58" s="16" t="inlineStr">
@@ -3502,12 +3506,20 @@
       </c>
       <c r="I58" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J58" s="13" t="n"/>
-      <c r="K58" s="13" t="n"/>
-      <c r="L58" s="13" t="n"/>
+          <t>26-07-2026</t>
+        </is>
+      </c>
+      <c r="J58" s="13" t="inlineStr">
+        <is>
+          <t>26-07-2026</t>
+        </is>
+      </c>
+      <c r="K58" s="13" t="inlineStr">
+        <is>
+          <t>01-08-2026</t>
+        </is>
+      </c>
+      <c r="L58" s="13" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="17" t="n">
@@ -3515,27 +3527,27 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>Hashing</t>
+          <t>Arrays - Two Pointers</t>
         </is>
       </c>
       <c r="C59" s="18" t="inlineStr">
         <is>
-          <t>HashMaps &amp; HashSets</t>
+          <t>Two Pointers Technique</t>
         </is>
       </c>
       <c r="D59" s="18" t="inlineStr">
         <is>
-          <t>How Many Numbers Are Smaller Than the Current Number</t>
+          <t>Remove Element</t>
         </is>
       </c>
       <c r="E59" s="18" t="inlineStr">
         <is>
-          <t>Frequency Array</t>
+          <t>Two Pointers (Slow/Fast)</t>
         </is>
       </c>
       <c r="F59" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/how-many-numbers-are-smaller-than-the-current-number/</t>
+          <t>https://leetcode.com/problems/remove-element/</t>
         </is>
       </c>
       <c r="G59" s="20" t="inlineStr">
@@ -3543,11 +3555,11 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H59" s="18" t="n"/>
-      <c r="I59" s="17" t="n"/>
-      <c r="J59" s="17" t="n"/>
-      <c r="K59" s="17" t="n"/>
-      <c r="L59" s="17" t="n"/>
+      <c r="H59" s="18" t="inlineStr"/>
+      <c r="I59" s="17" t="inlineStr"/>
+      <c r="J59" s="17" t="inlineStr"/>
+      <c r="K59" s="17" t="inlineStr"/>
+      <c r="L59" s="17" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="13" t="n">
@@ -3555,27 +3567,27 @@
       </c>
       <c r="B60" s="14" t="inlineStr">
         <is>
-          <t>Hashing</t>
+          <t>Arrays - Two Pointers</t>
         </is>
       </c>
       <c r="C60" s="14" t="inlineStr">
         <is>
-          <t>HashMaps &amp; HashSets</t>
+          <t>Two Pointers Technique</t>
         </is>
       </c>
       <c r="D60" s="14" t="inlineStr">
         <is>
-          <t>Contains Duplicate</t>
+          <t>Reverse String</t>
         </is>
       </c>
       <c r="E60" s="14" t="inlineStr">
         <is>
-          <t>HashSet</t>
+          <t>Two Pointers (Left/Right)</t>
         </is>
       </c>
       <c r="F60" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/contains-duplicate/</t>
+          <t>https://leetcode.com/problems/reverse-string/</t>
         </is>
       </c>
       <c r="G60" s="16" t="inlineStr">
@@ -3583,11 +3595,19 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H60" s="14" t="n"/>
-      <c r="I60" s="13" t="n"/>
-      <c r="J60" s="13" t="n"/>
-      <c r="K60" s="13" t="n"/>
-      <c r="L60" s="13" t="n"/>
+      <c r="H60" s="14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I60" s="13" t="inlineStr">
+        <is>
+          <t>10-08-2026</t>
+        </is>
+      </c>
+      <c r="J60" s="13" t="inlineStr"/>
+      <c r="K60" s="13" t="inlineStr"/>
+      <c r="L60" s="13" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="17" t="n">
@@ -3595,27 +3615,27 @@
       </c>
       <c r="B61" s="18" t="inlineStr">
         <is>
-          <t>Hashing</t>
+          <t>Arrays - Two Pointers</t>
         </is>
       </c>
       <c r="C61" s="18" t="inlineStr">
         <is>
-          <t>HashMaps &amp; HashSets</t>
+          <t>Two Pointers Technique</t>
         </is>
       </c>
       <c r="D61" s="18" t="inlineStr">
         <is>
-          <t>Valid Anagram</t>
+          <t>Squares of a Sorted Array</t>
         </is>
       </c>
       <c r="E61" s="18" t="inlineStr">
         <is>
-          <t>HashMap / Frequency Array</t>
+          <t>Two Pointers (Left/Right)</t>
         </is>
       </c>
       <c r="F61" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/valid-anagram/</t>
+          <t>https://leetcode.com/problems/squares-of-a-sorted-array/</t>
         </is>
       </c>
       <c r="G61" s="20" t="inlineStr">
@@ -3630,12 +3650,20 @@
       </c>
       <c r="I61" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J61" s="17" t="n"/>
-      <c r="K61" s="17" t="n"/>
-      <c r="L61" s="17" t="n"/>
+          <t>27-07-2026</t>
+        </is>
+      </c>
+      <c r="J61" s="17" t="inlineStr">
+        <is>
+          <t>27-07-2026</t>
+        </is>
+      </c>
+      <c r="K61" s="17" t="inlineStr">
+        <is>
+          <t>02-08-2026</t>
+        </is>
+      </c>
+      <c r="L61" s="17" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="13" t="n">
@@ -3643,32 +3671,32 @@
       </c>
       <c r="B62" s="14" t="inlineStr">
         <is>
-          <t>Hashing</t>
+          <t>Arrays - Two Pointers</t>
         </is>
       </c>
       <c r="C62" s="14" t="inlineStr">
         <is>
-          <t>HashMaps &amp; HashSets</t>
+          <t>Two Pointers Technique</t>
         </is>
       </c>
       <c r="D62" s="14" t="inlineStr">
         <is>
-          <t>Two Sum</t>
+          <t>Trapping Rain Water</t>
         </is>
       </c>
       <c r="E62" s="14" t="inlineStr">
         <is>
-          <t>HashMap</t>
+          <t>Two Pointers</t>
         </is>
       </c>
       <c r="F62" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/two-sum/</t>
-        </is>
-      </c>
-      <c r="G62" s="16" t="inlineStr">
-        <is>
-          <t>Easy</t>
+          <t>https://leetcode.com/problems/trapping-rain-water/</t>
+        </is>
+      </c>
+      <c r="G62" s="24" t="inlineStr">
+        <is>
+          <t>Hard</t>
         </is>
       </c>
       <c r="H62" s="14" t="inlineStr">
@@ -3678,20 +3706,12 @@
       </c>
       <c r="I62" s="13" t="inlineStr">
         <is>
-          <t>25-07-2026</t>
-        </is>
-      </c>
-      <c r="J62" s="13" t="inlineStr">
-        <is>
-          <t>26-07-2026</t>
-        </is>
-      </c>
-      <c r="K62" s="13" t="inlineStr">
-        <is>
-          <t>01-08-2026</t>
-        </is>
-      </c>
-      <c r="L62" s="13" t="n"/>
+          <t>12-08-2026</t>
+        </is>
+      </c>
+      <c r="J62" s="13" t="inlineStr"/>
+      <c r="K62" s="13" t="inlineStr"/>
+      <c r="L62" s="13" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="17" t="n">
@@ -3699,27 +3719,27 @@
       </c>
       <c r="B63" s="18" t="inlineStr">
         <is>
-          <t>Hashing</t>
+          <t>Binary Search &amp; Sort</t>
         </is>
       </c>
       <c r="C63" s="18" t="inlineStr">
         <is>
-          <t>HashMaps &amp; HashSets</t>
+          <t>Binary Search</t>
         </is>
       </c>
       <c r="D63" s="18" t="inlineStr">
         <is>
-          <t>Majority Element</t>
+          <t>Binary Search</t>
         </is>
       </c>
       <c r="E63" s="18" t="inlineStr">
         <is>
-          <t>Moore's Voting Algorithm</t>
+          <t>Binary Search</t>
         </is>
       </c>
       <c r="F63" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/majority-element/</t>
+          <t>https://leetcode.com/problems/binary-search/</t>
         </is>
       </c>
       <c r="G63" s="20" t="inlineStr">
@@ -3734,20 +3754,12 @@
       </c>
       <c r="I63" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J63" s="17" t="inlineStr">
-        <is>
-          <t>28-07-2026</t>
-        </is>
-      </c>
-      <c r="K63" s="17" t="inlineStr">
-        <is>
-          <t>03-08-2026</t>
-        </is>
-      </c>
-      <c r="L63" s="17" t="n"/>
+          <t>04-08-2026</t>
+        </is>
+      </c>
+      <c r="J63" s="17" t="inlineStr"/>
+      <c r="K63" s="17" t="inlineStr"/>
+      <c r="L63" s="17" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="13" t="n">
@@ -3755,27 +3767,27 @@
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>Hashing</t>
+          <t>Binary Search &amp; Sort</t>
         </is>
       </c>
       <c r="C64" s="14" t="inlineStr">
         <is>
-          <t>HashMaps &amp; HashSets</t>
+          <t>Binary Search</t>
         </is>
       </c>
       <c r="D64" s="14" t="inlineStr">
         <is>
-          <t>Find the Difference</t>
+          <t>Find Target Indices After Sorting Array</t>
         </is>
       </c>
       <c r="E64" s="14" t="inlineStr">
         <is>
-          <t>HashMap</t>
+          <t>Sorting</t>
         </is>
       </c>
       <c r="F64" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/find-the-difference/</t>
+          <t>https://leetcode.com/problems/find-target-indices-after-sorting-array/</t>
         </is>
       </c>
       <c r="G64" s="16" t="inlineStr">
@@ -3783,19 +3795,11 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H64" s="14" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="I64" s="13" t="inlineStr">
-        <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J64" s="13" t="n"/>
-      <c r="K64" s="13" t="n"/>
-      <c r="L64" s="13" t="n"/>
+      <c r="H64" s="14" t="inlineStr"/>
+      <c r="I64" s="13" t="inlineStr"/>
+      <c r="J64" s="13" t="inlineStr"/>
+      <c r="K64" s="13" t="inlineStr"/>
+      <c r="L64" s="13" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="17" t="n">
@@ -3803,27 +3807,27 @@
       </c>
       <c r="B65" s="18" t="inlineStr">
         <is>
-          <t>Hashing</t>
+          <t>Binary Search &amp; Sort</t>
         </is>
       </c>
       <c r="C65" s="18" t="inlineStr">
         <is>
-          <t>HashMaps &amp; HashSets</t>
+          <t>Binary Search</t>
         </is>
       </c>
       <c r="D65" s="18" t="inlineStr">
         <is>
-          <t>Keyboard Row</t>
+          <t>First Bad Version</t>
         </is>
       </c>
       <c r="E65" s="18" t="inlineStr">
         <is>
-          <t>HashSet</t>
+          <t>Binary Search</t>
         </is>
       </c>
       <c r="F65" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/keyboard-row/</t>
+          <t>https://leetcode.com/problems/first-bad-version/</t>
         </is>
       </c>
       <c r="G65" s="20" t="inlineStr">
@@ -3838,12 +3842,12 @@
       </c>
       <c r="I65" s="17" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J65" s="17" t="n"/>
-      <c r="K65" s="17" t="n"/>
-      <c r="L65" s="17" t="n"/>
+          <t>06-08-2026</t>
+        </is>
+      </c>
+      <c r="J65" s="17" t="inlineStr"/>
+      <c r="K65" s="17" t="inlineStr"/>
+      <c r="L65" s="17" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="13" t="n">
@@ -3851,27 +3855,27 @@
       </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>Hashing</t>
+          <t>Binary Search &amp; Sort</t>
         </is>
       </c>
       <c r="C66" s="14" t="inlineStr">
         <is>
-          <t>HashMaps &amp; HashSets</t>
+          <t>Binary Search</t>
         </is>
       </c>
       <c r="D66" s="14" t="inlineStr">
         <is>
-          <t>Happy Number</t>
+          <t>Search Insert Position</t>
         </is>
       </c>
       <c r="E66" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Binary Search</t>
         </is>
       </c>
       <c r="F66" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/happy-number/</t>
+          <t>https://leetcode.com/problems/search-insert-position/</t>
         </is>
       </c>
       <c r="G66" s="16" t="inlineStr">
@@ -3886,7 +3890,7 @@
       </c>
       <c r="I66" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
+          <t>04-08-2026</t>
         </is>
       </c>
       <c r="J66" s="13" t="inlineStr"/>
@@ -3899,27 +3903,27 @@
       </c>
       <c r="B67" s="18" t="inlineStr">
         <is>
-          <t>Linked Lists</t>
+          <t>Binary Search &amp; Sort</t>
         </is>
       </c>
       <c r="C67" s="18" t="inlineStr">
         <is>
-          <t>Merging</t>
+          <t>Binary Search</t>
         </is>
       </c>
       <c r="D67" s="18" t="inlineStr">
         <is>
-          <t>Merge Two Sorted Lists</t>
+          <t>Sqrt(x)</t>
         </is>
       </c>
       <c r="E67" s="18" t="inlineStr">
         <is>
-          <t>Two Pointers</t>
+          <t>Binary Search</t>
         </is>
       </c>
       <c r="F67" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/merge-two-sorted-lists/</t>
+          <t>https://leetcode.com/problems/sqrtx/</t>
         </is>
       </c>
       <c r="G67" s="20" t="inlineStr">
@@ -3927,11 +3931,19 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H67" s="18" t="n"/>
-      <c r="I67" s="17" t="n"/>
-      <c r="J67" s="17" t="n"/>
-      <c r="K67" s="17" t="n"/>
-      <c r="L67" s="17" t="n"/>
+      <c r="H67" s="18" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I67" s="17" t="inlineStr">
+        <is>
+          <t>11-08-2026</t>
+        </is>
+      </c>
+      <c r="J67" s="17" t="inlineStr"/>
+      <c r="K67" s="17" t="inlineStr"/>
+      <c r="L67" s="17" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="13" t="n">
@@ -3939,27 +3951,27 @@
       </c>
       <c r="B68" s="14" t="inlineStr">
         <is>
-          <t>Linked Lists</t>
+          <t>Hashing</t>
         </is>
       </c>
       <c r="C68" s="14" t="inlineStr">
         <is>
-          <t>Modification</t>
+          <t>HashMaps &amp; HashSets</t>
         </is>
       </c>
       <c r="D68" s="14" t="inlineStr">
         <is>
-          <t>Remove Linked List Elements</t>
+          <t>Contains Duplicate</t>
         </is>
       </c>
       <c r="E68" s="14" t="inlineStr">
         <is>
-          <t>Iteration</t>
+          <t>HashSet</t>
         </is>
       </c>
       <c r="F68" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/remove-linked-list-elements/</t>
+          <t>https://leetcode.com/problems/contains-duplicate/</t>
         </is>
       </c>
       <c r="G68" s="16" t="inlineStr">
@@ -3967,11 +3979,11 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H68" s="14" t="n"/>
-      <c r="I68" s="13" t="n"/>
-      <c r="J68" s="13" t="n"/>
-      <c r="K68" s="13" t="n"/>
-      <c r="L68" s="13" t="n"/>
+      <c r="H68" s="14" t="inlineStr"/>
+      <c r="I68" s="13" t="inlineStr"/>
+      <c r="J68" s="13" t="inlineStr"/>
+      <c r="K68" s="13" t="inlineStr"/>
+      <c r="L68" s="13" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="17" t="n">
@@ -3979,27 +3991,27 @@
       </c>
       <c r="B69" s="18" t="inlineStr">
         <is>
-          <t>Linked Lists</t>
+          <t>Hashing</t>
         </is>
       </c>
       <c r="C69" s="18" t="inlineStr">
         <is>
-          <t>Modification</t>
+          <t>HashMaps &amp; HashSets</t>
         </is>
       </c>
       <c r="D69" s="18" t="inlineStr">
         <is>
-          <t>Remove Duplicates from Sorted List</t>
+          <t>Find the Difference</t>
         </is>
       </c>
       <c r="E69" s="18" t="inlineStr">
         <is>
-          <t>Iteration</t>
+          <t>HashMap</t>
         </is>
       </c>
       <c r="F69" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/remove-duplicates-from-sorted-list/</t>
+          <t>https://leetcode.com/problems/find-the-difference/</t>
         </is>
       </c>
       <c r="G69" s="20" t="inlineStr">
@@ -4007,11 +4019,19 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H69" s="18" t="n"/>
-      <c r="I69" s="17" t="n"/>
-      <c r="J69" s="17" t="n"/>
-      <c r="K69" s="17" t="n"/>
-      <c r="L69" s="17" t="n"/>
+      <c r="H69" s="18" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I69" s="17" t="inlineStr">
+        <is>
+          <t>27-08-2026</t>
+        </is>
+      </c>
+      <c r="J69" s="17" t="inlineStr"/>
+      <c r="K69" s="17" t="inlineStr"/>
+      <c r="L69" s="17" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="13" t="n">
@@ -4019,27 +4039,27 @@
       </c>
       <c r="B70" s="14" t="inlineStr">
         <is>
-          <t>Linked Lists</t>
+          <t>Hashing</t>
         </is>
       </c>
       <c r="C70" s="14" t="inlineStr">
         <is>
-          <t>Reversal</t>
+          <t>HashMaps &amp; HashSets</t>
         </is>
       </c>
       <c r="D70" s="14" t="inlineStr">
         <is>
-          <t>Reverse Linked List</t>
+          <t>Happy Number</t>
         </is>
       </c>
       <c r="E70" s="14" t="inlineStr">
         <is>
-          <t>Iterative/Recursive</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F70" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/reverse-linked-list/</t>
+          <t>https://leetcode.com/problems/happy-number/</t>
         </is>
       </c>
       <c r="G70" s="16" t="inlineStr">
@@ -4047,11 +4067,19 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H70" s="14" t="n"/>
-      <c r="I70" s="13" t="n"/>
-      <c r="J70" s="13" t="n"/>
-      <c r="K70" s="13" t="n"/>
-      <c r="L70" s="13" t="n"/>
+      <c r="H70" s="14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I70" s="13" t="inlineStr">
+        <is>
+          <t>13-08-2026</t>
+        </is>
+      </c>
+      <c r="J70" s="13" t="inlineStr"/>
+      <c r="K70" s="13" t="inlineStr"/>
+      <c r="L70" s="13" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="17" t="n">
@@ -4059,27 +4087,27 @@
       </c>
       <c r="B71" s="18" t="inlineStr">
         <is>
-          <t>Linked Lists</t>
+          <t>Hashing</t>
         </is>
       </c>
       <c r="C71" s="18" t="inlineStr">
         <is>
-          <t>Slow/Fast Ptr</t>
+          <t>HashMaps &amp; HashSets</t>
         </is>
       </c>
       <c r="D71" s="18" t="inlineStr">
         <is>
-          <t>Linked List Cycle</t>
+          <t>How Many Numbers Are Smaller Than the Current Number</t>
         </is>
       </c>
       <c r="E71" s="18" t="inlineStr">
         <is>
-          <t>Tortoise &amp; Hare</t>
+          <t>Frequency Array</t>
         </is>
       </c>
       <c r="F71" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/linked-list-cycle/</t>
+          <t>https://leetcode.com/problems/how-many-numbers-are-smaller-than-the-current-number/</t>
         </is>
       </c>
       <c r="G71" s="20" t="inlineStr">
@@ -4087,11 +4115,11 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H71" s="18" t="n"/>
-      <c r="I71" s="17" t="n"/>
-      <c r="J71" s="17" t="n"/>
-      <c r="K71" s="17" t="n"/>
-      <c r="L71" s="17" t="n"/>
+      <c r="H71" s="18" t="inlineStr"/>
+      <c r="I71" s="17" t="inlineStr"/>
+      <c r="J71" s="17" t="inlineStr"/>
+      <c r="K71" s="17" t="inlineStr"/>
+      <c r="L71" s="17" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="13" t="n">
@@ -4099,27 +4127,27 @@
       </c>
       <c r="B72" s="14" t="inlineStr">
         <is>
-          <t>Linked Lists</t>
+          <t>Hashing</t>
         </is>
       </c>
       <c r="C72" s="14" t="inlineStr">
         <is>
-          <t>Slow/Fast Ptr</t>
+          <t>HashMaps &amp; HashSets</t>
         </is>
       </c>
       <c r="D72" s="14" t="inlineStr">
         <is>
-          <t>Middle of the Linked List</t>
+          <t>Jewels and Stones</t>
         </is>
       </c>
       <c r="E72" s="14" t="inlineStr">
         <is>
-          <t>Tortoise &amp; Hare</t>
+          <t>HashSet</t>
         </is>
       </c>
       <c r="F72" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/middle-of-the-linked-list/</t>
+          <t>https://leetcode.com/problems/jewels-and-stones/</t>
         </is>
       </c>
       <c r="G72" s="16" t="inlineStr">
@@ -4127,11 +4155,19 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H72" s="14" t="n"/>
-      <c r="I72" s="13" t="n"/>
-      <c r="J72" s="13" t="n"/>
-      <c r="K72" s="13" t="n"/>
-      <c r="L72" s="13" t="n"/>
+      <c r="H72" s="14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I72" s="13" t="inlineStr">
+        <is>
+          <t>29-08-2026</t>
+        </is>
+      </c>
+      <c r="J72" s="13" t="inlineStr"/>
+      <c r="K72" s="13" t="inlineStr"/>
+      <c r="L72" s="13" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="17" t="n">
@@ -4139,27 +4175,27 @@
       </c>
       <c r="B73" s="18" t="inlineStr">
         <is>
-          <t>Linked Lists</t>
+          <t>Hashing</t>
         </is>
       </c>
       <c r="C73" s="18" t="inlineStr">
         <is>
-          <t>Slow/Fast Ptr</t>
+          <t>HashMaps &amp; HashSets</t>
         </is>
       </c>
       <c r="D73" s="18" t="inlineStr">
         <is>
-          <t>Palindrome Linked List</t>
+          <t>Keyboard Row</t>
         </is>
       </c>
       <c r="E73" s="18" t="inlineStr">
         <is>
-          <t>Reversal &amp; Pointers</t>
+          <t>HashSet</t>
         </is>
       </c>
       <c r="F73" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/palindrome-linked-list/</t>
+          <t>https://leetcode.com/problems/keyboard-row/</t>
         </is>
       </c>
       <c r="G73" s="20" t="inlineStr">
@@ -4167,11 +4203,19 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H73" s="18" t="n"/>
-      <c r="I73" s="17" t="n"/>
-      <c r="J73" s="17" t="n"/>
-      <c r="K73" s="17" t="n"/>
-      <c r="L73" s="17" t="n"/>
+      <c r="H73" s="18" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I73" s="17" t="inlineStr">
+        <is>
+          <t>21-08-2026</t>
+        </is>
+      </c>
+      <c r="J73" s="17" t="inlineStr"/>
+      <c r="K73" s="17" t="inlineStr"/>
+      <c r="L73" s="17" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="13" t="n">
@@ -4179,27 +4223,27 @@
       </c>
       <c r="B74" s="14" t="inlineStr">
         <is>
-          <t>Stacks</t>
+          <t>Hashing</t>
         </is>
       </c>
       <c r="C74" s="14" t="inlineStr">
         <is>
-          <t>Implementation</t>
+          <t>HashMaps &amp; HashSets</t>
         </is>
       </c>
       <c r="D74" s="14" t="inlineStr">
         <is>
-          <t>Implement Queue using Stacks</t>
+          <t>Majority Element</t>
         </is>
       </c>
       <c r="E74" s="14" t="inlineStr">
         <is>
-          <t>Two Stacks</t>
+          <t>Moore's Voting Algorithm</t>
         </is>
       </c>
       <c r="F74" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/implement-queue-using-stacks/</t>
+          <t>https://leetcode.com/problems/majority-element/</t>
         </is>
       </c>
       <c r="G74" s="16" t="inlineStr">
@@ -4207,11 +4251,27 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H74" s="14" t="n"/>
-      <c r="I74" s="13" t="n"/>
-      <c r="J74" s="13" t="n"/>
-      <c r="K74" s="13" t="n"/>
-      <c r="L74" s="13" t="n"/>
+      <c r="H74" s="14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I74" s="13" t="inlineStr">
+        <is>
+          <t>28-07-2026</t>
+        </is>
+      </c>
+      <c r="J74" s="13" t="inlineStr">
+        <is>
+          <t>28-07-2026</t>
+        </is>
+      </c>
+      <c r="K74" s="13" t="inlineStr">
+        <is>
+          <t>03-08-2026</t>
+        </is>
+      </c>
+      <c r="L74" s="13" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="17" t="n">
@@ -4219,27 +4279,27 @@
       </c>
       <c r="B75" s="18" t="inlineStr">
         <is>
-          <t>Stacks</t>
+          <t>Hashing</t>
         </is>
       </c>
       <c r="C75" s="18" t="inlineStr">
         <is>
-          <t>Implementation</t>
+          <t>HashMaps &amp; HashSets</t>
         </is>
       </c>
       <c r="D75" s="18" t="inlineStr">
         <is>
-          <t>Implement Stack using Queues</t>
+          <t>Two Sum</t>
         </is>
       </c>
       <c r="E75" s="18" t="inlineStr">
         <is>
-          <t>Two Queues</t>
+          <t>HashMap</t>
         </is>
       </c>
       <c r="F75" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/implement-stack-using-queues/</t>
+          <t>https://leetcode.com/problems/two-sum/</t>
         </is>
       </c>
       <c r="G75" s="20" t="inlineStr">
@@ -4247,11 +4307,27 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H75" s="18" t="n"/>
-      <c r="I75" s="17" t="n"/>
-      <c r="J75" s="17" t="n"/>
-      <c r="K75" s="17" t="n"/>
-      <c r="L75" s="17" t="n"/>
+      <c r="H75" s="18" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I75" s="17" t="inlineStr">
+        <is>
+          <t>25-07-2026</t>
+        </is>
+      </c>
+      <c r="J75" s="17" t="inlineStr">
+        <is>
+          <t>26-07-2026</t>
+        </is>
+      </c>
+      <c r="K75" s="17" t="inlineStr">
+        <is>
+          <t>01-08-2026</t>
+        </is>
+      </c>
+      <c r="L75" s="17" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="13" t="n">
@@ -4259,27 +4335,27 @@
       </c>
       <c r="B76" s="14" t="inlineStr">
         <is>
-          <t>Stacks</t>
+          <t>Hashing</t>
         </is>
       </c>
       <c r="C76" s="14" t="inlineStr">
         <is>
-          <t>Stack Data Structure</t>
+          <t>HashMaps &amp; HashSets</t>
         </is>
       </c>
       <c r="D76" s="14" t="inlineStr">
         <is>
-          <t>Valid Parentheses</t>
+          <t>Valid Anagram</t>
         </is>
       </c>
       <c r="E76" s="14" t="inlineStr">
         <is>
-          <t>Stack</t>
+          <t>HashMap / Frequency Array</t>
         </is>
       </c>
       <c r="F76" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/valid-parentheses/</t>
+          <t>https://leetcode.com/problems/valid-anagram/</t>
         </is>
       </c>
       <c r="G76" s="16" t="inlineStr">
@@ -4294,12 +4370,12 @@
       </c>
       <c r="I76" s="13" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J76" s="13" t="n"/>
-      <c r="K76" s="13" t="n"/>
-      <c r="L76" s="13" t="n"/>
+          <t>17-08-2026</t>
+        </is>
+      </c>
+      <c r="J76" s="13" t="inlineStr"/>
+      <c r="K76" s="13" t="inlineStr"/>
+      <c r="L76" s="13" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="17" t="n">
@@ -4307,27 +4383,27 @@
       </c>
       <c r="B77" s="18" t="inlineStr">
         <is>
-          <t>Stacks</t>
+          <t>Linked Lists</t>
         </is>
       </c>
       <c r="C77" s="18" t="inlineStr">
         <is>
-          <t>Stack Data Structure</t>
+          <t>Merging</t>
         </is>
       </c>
       <c r="D77" s="18" t="inlineStr">
         <is>
-          <t>Remove Outermost Parentheses</t>
+          <t>Merge Two Sorted Lists</t>
         </is>
       </c>
       <c r="E77" s="18" t="inlineStr">
         <is>
-          <t>Stack or Counter</t>
+          <t>Two Pointers</t>
         </is>
       </c>
       <c r="F77" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/remove-outermost-parentheses/</t>
+          <t>https://leetcode.com/problems/merge-two-sorted-lists/</t>
         </is>
       </c>
       <c r="G77" s="20" t="inlineStr">
@@ -4335,11 +4411,11 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H77" s="18" t="n"/>
-      <c r="I77" s="17" t="n"/>
-      <c r="J77" s="17" t="n"/>
-      <c r="K77" s="17" t="n"/>
-      <c r="L77" s="17" t="n"/>
+      <c r="H77" s="18" t="inlineStr"/>
+      <c r="I77" s="17" t="inlineStr"/>
+      <c r="J77" s="17" t="inlineStr"/>
+      <c r="K77" s="17" t="inlineStr"/>
+      <c r="L77" s="17" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="13" t="n">
@@ -4347,27 +4423,27 @@
       </c>
       <c r="B78" s="14" t="inlineStr">
         <is>
-          <t>Stacks</t>
+          <t>Linked Lists</t>
         </is>
       </c>
       <c r="C78" s="14" t="inlineStr">
         <is>
-          <t>Stack Data Structure</t>
+          <t>Modification</t>
         </is>
       </c>
       <c r="D78" s="14" t="inlineStr">
         <is>
-          <t>Remove All Adjacent Duplicates In String</t>
+          <t>Remove Duplicates from Sorted List</t>
         </is>
       </c>
       <c r="E78" s="14" t="inlineStr">
         <is>
-          <t>Stack</t>
+          <t>Iteration</t>
         </is>
       </c>
       <c r="F78" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/remove-all-adjacent-duplicates-in-string/</t>
+          <t>https://leetcode.com/problems/remove-duplicates-from-sorted-list/</t>
         </is>
       </c>
       <c r="G78" s="16" t="inlineStr">
@@ -4375,19 +4451,11 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H78" s="14" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="I78" s="13" t="inlineStr">
-        <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J78" s="13" t="n"/>
-      <c r="K78" s="13" t="n"/>
-      <c r="L78" s="13" t="n"/>
+      <c r="H78" s="14" t="inlineStr"/>
+      <c r="I78" s="13" t="inlineStr"/>
+      <c r="J78" s="13" t="inlineStr"/>
+      <c r="K78" s="13" t="inlineStr"/>
+      <c r="L78" s="13" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="17" t="n">
@@ -4395,39 +4463,39 @@
       </c>
       <c r="B79" s="18" t="inlineStr">
         <is>
-          <t>Stacks</t>
+          <t>Linked Lists</t>
         </is>
       </c>
       <c r="C79" s="18" t="inlineStr">
         <is>
-          <t>Stack Data Structure</t>
+          <t>Modification</t>
         </is>
       </c>
       <c r="D79" s="18" t="inlineStr">
         <is>
-          <t>Min Stack</t>
+          <t>Remove Linked List Elements</t>
         </is>
       </c>
       <c r="E79" s="18" t="inlineStr">
         <is>
-          <t>Two Stacks</t>
+          <t>Iteration</t>
         </is>
       </c>
       <c r="F79" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/min-stack/</t>
-        </is>
-      </c>
-      <c r="G79" s="22" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H79" s="18" t="n"/>
-      <c r="I79" s="17" t="n"/>
-      <c r="J79" s="17" t="n"/>
-      <c r="K79" s="17" t="n"/>
-      <c r="L79" s="17" t="n"/>
+          <t>https://leetcode.com/problems/remove-linked-list-elements/</t>
+        </is>
+      </c>
+      <c r="G79" s="20" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H79" s="18" t="inlineStr"/>
+      <c r="I79" s="17" t="inlineStr"/>
+      <c r="J79" s="17" t="inlineStr"/>
+      <c r="K79" s="17" t="inlineStr"/>
+      <c r="L79" s="17" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="13" t="n">
@@ -4435,39 +4503,39 @@
       </c>
       <c r="B80" s="14" t="inlineStr">
         <is>
-          <t>Stacks</t>
+          <t>Linked Lists</t>
         </is>
       </c>
       <c r="C80" s="14" t="inlineStr">
         <is>
-          <t>Stack Data Structure</t>
+          <t>Reversal</t>
         </is>
       </c>
       <c r="D80" s="14" t="inlineStr">
         <is>
-          <t>Evaluate Reverse Polish Notation</t>
+          <t>Reverse Linked List</t>
         </is>
       </c>
       <c r="E80" s="14" t="inlineStr">
         <is>
-          <t>Stack</t>
+          <t>Iterative/Recursive</t>
         </is>
       </c>
       <c r="F80" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/evaluate-reverse-polish-notation/</t>
-        </is>
-      </c>
-      <c r="G80" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H80" s="14" t="n"/>
-      <c r="I80" s="13" t="n"/>
-      <c r="J80" s="13" t="n"/>
-      <c r="K80" s="13" t="n"/>
-      <c r="L80" s="13" t="n"/>
+          <t>https://leetcode.com/problems/reverse-linked-list/</t>
+        </is>
+      </c>
+      <c r="G80" s="16" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H80" s="14" t="inlineStr"/>
+      <c r="I80" s="13" t="inlineStr"/>
+      <c r="J80" s="13" t="inlineStr"/>
+      <c r="K80" s="13" t="inlineStr"/>
+      <c r="L80" s="13" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="17" t="n">
@@ -4475,27 +4543,27 @@
       </c>
       <c r="B81" s="18" t="inlineStr">
         <is>
-          <t>Stacks</t>
+          <t>Linked Lists</t>
         </is>
       </c>
       <c r="C81" s="18" t="inlineStr">
         <is>
-          <t>Stack Data Structure</t>
+          <t>Slow/Fast Ptr</t>
         </is>
       </c>
       <c r="D81" s="18" t="inlineStr">
         <is>
-          <t>Next Greater Element I</t>
+          <t>Linked List Cycle</t>
         </is>
       </c>
       <c r="E81" s="18" t="inlineStr">
         <is>
-          <t>Monotonic Stack</t>
+          <t>Tortoise &amp; Hare</t>
         </is>
       </c>
       <c r="F81" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/next-greater-element-i/</t>
+          <t>https://leetcode.com/problems/linked-list-cycle/</t>
         </is>
       </c>
       <c r="G81" s="20" t="inlineStr">
@@ -4503,11 +4571,11 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H81" s="18" t="n"/>
-      <c r="I81" s="17" t="n"/>
-      <c r="J81" s="17" t="n"/>
-      <c r="K81" s="17" t="n"/>
-      <c r="L81" s="17" t="n"/>
+      <c r="H81" s="18" t="inlineStr"/>
+      <c r="I81" s="17" t="inlineStr"/>
+      <c r="J81" s="17" t="inlineStr"/>
+      <c r="K81" s="17" t="inlineStr"/>
+      <c r="L81" s="17" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="13" t="n">
@@ -4515,39 +4583,39 @@
       </c>
       <c r="B82" s="14" t="inlineStr">
         <is>
-          <t>Stacks</t>
+          <t>Linked Lists</t>
         </is>
       </c>
       <c r="C82" s="14" t="inlineStr">
         <is>
-          <t>Stack Data Structure</t>
+          <t>Slow/Fast Ptr</t>
         </is>
       </c>
       <c r="D82" s="14" t="inlineStr">
         <is>
-          <t>Daily Temperatures</t>
+          <t>Middle of the Linked List</t>
         </is>
       </c>
       <c r="E82" s="14" t="inlineStr">
         <is>
-          <t>Monotonic Stack</t>
+          <t>Tortoise &amp; Hare</t>
         </is>
       </c>
       <c r="F82" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/daily-temperatures/</t>
-        </is>
-      </c>
-      <c r="G82" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H82" s="14" t="n"/>
-      <c r="I82" s="13" t="n"/>
-      <c r="J82" s="13" t="n"/>
-      <c r="K82" s="13" t="n"/>
-      <c r="L82" s="13" t="n"/>
+          <t>https://leetcode.com/problems/middle-of-the-linked-list/</t>
+        </is>
+      </c>
+      <c r="G82" s="16" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H82" s="14" t="inlineStr"/>
+      <c r="I82" s="13" t="inlineStr"/>
+      <c r="J82" s="13" t="inlineStr"/>
+      <c r="K82" s="13" t="inlineStr"/>
+      <c r="L82" s="13" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="17" t="n">
@@ -4555,27 +4623,27 @@
       </c>
       <c r="B83" s="18" t="inlineStr">
         <is>
-          <t>Stacks</t>
+          <t>Linked Lists</t>
         </is>
       </c>
       <c r="C83" s="18" t="inlineStr">
         <is>
-          <t>String Ops</t>
+          <t>Slow/Fast Ptr</t>
         </is>
       </c>
       <c r="D83" s="18" t="inlineStr">
         <is>
-          <t>Backspace String Compare</t>
+          <t>Palindrome Linked List</t>
         </is>
       </c>
       <c r="E83" s="18" t="inlineStr">
         <is>
-          <t>Stack</t>
+          <t>Reversal &amp; Pointers</t>
         </is>
       </c>
       <c r="F83" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/backspace-string-compare/</t>
+          <t>https://leetcode.com/problems/palindrome-linked-list/</t>
         </is>
       </c>
       <c r="G83" s="20" t="inlineStr">
@@ -4583,11 +4651,11 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H83" s="18" t="n"/>
-      <c r="I83" s="17" t="n"/>
-      <c r="J83" s="17" t="n"/>
-      <c r="K83" s="17" t="n"/>
-      <c r="L83" s="17" t="n"/>
+      <c r="H83" s="18" t="inlineStr"/>
+      <c r="I83" s="17" t="inlineStr"/>
+      <c r="J83" s="17" t="inlineStr"/>
+      <c r="K83" s="17" t="inlineStr"/>
+      <c r="L83" s="17" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="13" t="n">
@@ -4595,27 +4663,27 @@
       </c>
       <c r="B84" s="14" t="inlineStr">
         <is>
-          <t>Recursion</t>
+          <t>Stacks</t>
         </is>
       </c>
       <c r="C84" s="14" t="inlineStr">
         <is>
-          <t>Logic/Math</t>
+          <t>Implementation</t>
         </is>
       </c>
       <c r="D84" s="14" t="inlineStr">
         <is>
-          <t>Power of Three</t>
+          <t>Implement Queue using Stacks</t>
         </is>
       </c>
       <c r="E84" s="14" t="inlineStr">
         <is>
-          <t>Recursion</t>
+          <t>Two Stacks</t>
         </is>
       </c>
       <c r="F84" s="15" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/power-of-three/</t>
+          <t>https://leetcode.com/problems/implement-queue-using-stacks/</t>
         </is>
       </c>
       <c r="G84" s="16" t="inlineStr">
@@ -4623,19 +4691,11 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H84" s="14" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="I84" s="13" t="inlineStr">
-        <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="J84" s="13" t="n"/>
-      <c r="K84" s="13" t="n"/>
-      <c r="L84" s="13" t="n"/>
+      <c r="H84" s="14" t="inlineStr"/>
+      <c r="I84" s="13" t="inlineStr"/>
+      <c r="J84" s="13" t="inlineStr"/>
+      <c r="K84" s="13" t="inlineStr"/>
+      <c r="L84" s="13" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="17" t="n">
@@ -4643,27 +4703,27 @@
       </c>
       <c r="B85" s="18" t="inlineStr">
         <is>
-          <t>Recursion</t>
+          <t>Stacks</t>
         </is>
       </c>
       <c r="C85" s="18" t="inlineStr">
         <is>
-          <t>Logic/Math</t>
+          <t>Implementation</t>
         </is>
       </c>
       <c r="D85" s="18" t="inlineStr">
         <is>
-          <t>Power of Four</t>
+          <t>Implement Stack using Queues</t>
         </is>
       </c>
       <c r="E85" s="18" t="inlineStr">
         <is>
-          <t>Recursion</t>
+          <t>Two Queues</t>
         </is>
       </c>
       <c r="F85" s="19" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problems/power-of-four/</t>
+          <t>https://leetcode.com/problems/implement-stack-using-queues/</t>
         </is>
       </c>
       <c r="G85" s="20" t="inlineStr">
@@ -4671,11 +4731,11 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H85" s="18" t="n"/>
-      <c r="I85" s="17" t="n"/>
-      <c r="J85" s="17" t="n"/>
-      <c r="K85" s="17" t="n"/>
-      <c r="L85" s="17" t="n"/>
+      <c r="H85" s="18" t="inlineStr"/>
+      <c r="I85" s="17" t="inlineStr"/>
+      <c r="J85" s="17" t="inlineStr"/>
+      <c r="K85" s="17" t="inlineStr"/>
+      <c r="L85" s="17" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="13" t="n">
@@ -4683,42 +4743,610 @@
       </c>
       <c r="B86" s="14" t="inlineStr">
         <is>
+          <t>Stacks</t>
+        </is>
+      </c>
+      <c r="C86" s="14" t="inlineStr">
+        <is>
+          <t>Stack Data Structure</t>
+        </is>
+      </c>
+      <c r="D86" s="14" t="inlineStr">
+        <is>
+          <t>Daily Temperatures</t>
+        </is>
+      </c>
+      <c r="E86" s="14" t="inlineStr">
+        <is>
+          <t>Monotonic Stack</t>
+        </is>
+      </c>
+      <c r="F86" s="15" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/daily-temperatures/</t>
+        </is>
+      </c>
+      <c r="G86" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H86" s="14" t="inlineStr"/>
+      <c r="I86" s="13" t="inlineStr"/>
+      <c r="J86" s="13" t="inlineStr"/>
+      <c r="K86" s="13" t="inlineStr"/>
+      <c r="L86" s="13" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="17" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="18" t="inlineStr">
+        <is>
+          <t>Stacks</t>
+        </is>
+      </c>
+      <c r="C87" s="18" t="inlineStr">
+        <is>
+          <t>Stack Data Structure</t>
+        </is>
+      </c>
+      <c r="D87" s="18" t="inlineStr">
+        <is>
+          <t>Evaluate Reverse Polish Notation</t>
+        </is>
+      </c>
+      <c r="E87" s="18" t="inlineStr">
+        <is>
+          <t>Stack</t>
+        </is>
+      </c>
+      <c r="F87" s="19" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/evaluate-reverse-polish-notation/</t>
+        </is>
+      </c>
+      <c r="G87" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H87" s="18" t="inlineStr"/>
+      <c r="I87" s="17" t="inlineStr"/>
+      <c r="J87" s="17" t="inlineStr"/>
+      <c r="K87" s="17" t="inlineStr"/>
+      <c r="L87" s="17" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="13" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="14" t="inlineStr">
+        <is>
+          <t>Stacks</t>
+        </is>
+      </c>
+      <c r="C88" s="14" t="inlineStr">
+        <is>
+          <t>Stack Data Structure</t>
+        </is>
+      </c>
+      <c r="D88" s="14" t="inlineStr">
+        <is>
+          <t>Min Stack</t>
+        </is>
+      </c>
+      <c r="E88" s="14" t="inlineStr">
+        <is>
+          <t>Two Stacks</t>
+        </is>
+      </c>
+      <c r="F88" s="15" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/min-stack/</t>
+        </is>
+      </c>
+      <c r="G88" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H88" s="14" t="inlineStr"/>
+      <c r="I88" s="13" t="inlineStr"/>
+      <c r="J88" s="13" t="inlineStr"/>
+      <c r="K88" s="13" t="inlineStr"/>
+      <c r="L88" s="13" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="17" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="18" t="inlineStr">
+        <is>
+          <t>Stacks</t>
+        </is>
+      </c>
+      <c r="C89" s="18" t="inlineStr">
+        <is>
+          <t>Stack Data Structure</t>
+        </is>
+      </c>
+      <c r="D89" s="18" t="inlineStr">
+        <is>
+          <t>Next Greater Element I</t>
+        </is>
+      </c>
+      <c r="E89" s="18" t="inlineStr">
+        <is>
+          <t>Monotonic Stack</t>
+        </is>
+      </c>
+      <c r="F89" s="19" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/next-greater-element-i/</t>
+        </is>
+      </c>
+      <c r="G89" s="20" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H89" s="18" t="inlineStr"/>
+      <c r="I89" s="17" t="inlineStr"/>
+      <c r="J89" s="17" t="inlineStr"/>
+      <c r="K89" s="17" t="inlineStr"/>
+      <c r="L89" s="17" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="13" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="14" t="inlineStr">
+        <is>
+          <t>Stacks</t>
+        </is>
+      </c>
+      <c r="C90" s="14" t="inlineStr">
+        <is>
+          <t>Stack Data Structure</t>
+        </is>
+      </c>
+      <c r="D90" s="14" t="inlineStr">
+        <is>
+          <t>Remove All Adjacent Duplicates In String</t>
+        </is>
+      </c>
+      <c r="E90" s="14" t="inlineStr">
+        <is>
+          <t>Stack</t>
+        </is>
+      </c>
+      <c r="F90" s="15" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/remove-all-adjacent-duplicates-in-string/</t>
+        </is>
+      </c>
+      <c r="G90" s="16" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H90" s="14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I90" s="13" t="inlineStr">
+        <is>
+          <t>08-08-2026</t>
+        </is>
+      </c>
+      <c r="J90" s="13" t="inlineStr"/>
+      <c r="K90" s="13" t="inlineStr"/>
+      <c r="L90" s="13" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="17" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="18" t="inlineStr">
+        <is>
+          <t>Stacks</t>
+        </is>
+      </c>
+      <c r="C91" s="18" t="inlineStr">
+        <is>
+          <t>Stack Data Structure</t>
+        </is>
+      </c>
+      <c r="D91" s="18" t="inlineStr">
+        <is>
+          <t>Remove Outermost Parentheses</t>
+        </is>
+      </c>
+      <c r="E91" s="18" t="inlineStr">
+        <is>
+          <t>Stack or Counter</t>
+        </is>
+      </c>
+      <c r="F91" s="19" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/remove-outermost-parentheses/</t>
+        </is>
+      </c>
+      <c r="G91" s="20" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H91" s="18" t="inlineStr"/>
+      <c r="I91" s="17" t="inlineStr"/>
+      <c r="J91" s="17" t="inlineStr"/>
+      <c r="K91" s="17" t="inlineStr"/>
+      <c r="L91" s="17" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="13" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="14" t="inlineStr">
+        <is>
+          <t>Stacks</t>
+        </is>
+      </c>
+      <c r="C92" s="14" t="inlineStr">
+        <is>
+          <t>Stack Data Structure</t>
+        </is>
+      </c>
+      <c r="D92" s="14" t="inlineStr">
+        <is>
+          <t>Valid Parentheses</t>
+        </is>
+      </c>
+      <c r="E92" s="14" t="inlineStr">
+        <is>
+          <t>Stack</t>
+        </is>
+      </c>
+      <c r="F92" s="15" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/valid-parentheses/</t>
+        </is>
+      </c>
+      <c r="G92" s="16" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H92" s="14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I92" s="13" t="inlineStr">
+        <is>
+          <t>04-08-2026</t>
+        </is>
+      </c>
+      <c r="J92" s="13" t="inlineStr"/>
+      <c r="K92" s="13" t="inlineStr"/>
+      <c r="L92" s="13" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="17" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="18" t="inlineStr">
+        <is>
+          <t>Stacks</t>
+        </is>
+      </c>
+      <c r="C93" s="18" t="inlineStr">
+        <is>
+          <t>String Ops</t>
+        </is>
+      </c>
+      <c r="D93" s="18" t="inlineStr">
+        <is>
+          <t>Backspace String Compare</t>
+        </is>
+      </c>
+      <c r="E93" s="18" t="inlineStr">
+        <is>
+          <t>Stack</t>
+        </is>
+      </c>
+      <c r="F93" s="19" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/backspace-string-compare/</t>
+        </is>
+      </c>
+      <c r="G93" s="20" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H93" s="18" t="inlineStr"/>
+      <c r="I93" s="17" t="inlineStr"/>
+      <c r="J93" s="17" t="inlineStr"/>
+      <c r="K93" s="17" t="inlineStr"/>
+      <c r="L93" s="17" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="13" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="14" t="inlineStr">
+        <is>
           <t>Recursion</t>
         </is>
       </c>
-      <c r="C86" s="14" t="inlineStr">
+      <c r="C94" s="14" t="inlineStr">
+        <is>
+          <t>Logic/Math</t>
+        </is>
+      </c>
+      <c r="D94" s="14" t="inlineStr">
+        <is>
+          <t>Power of Four</t>
+        </is>
+      </c>
+      <c r="E94" s="14" t="inlineStr">
+        <is>
+          <t>Recursion</t>
+        </is>
+      </c>
+      <c r="F94" s="15" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/power-of-four/</t>
+        </is>
+      </c>
+      <c r="G94" s="16" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H94" s="14" t="inlineStr"/>
+      <c r="I94" s="13" t="inlineStr"/>
+      <c r="J94" s="13" t="inlineStr"/>
+      <c r="K94" s="13" t="inlineStr"/>
+      <c r="L94" s="13" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="17" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="18" t="inlineStr">
+        <is>
+          <t>Recursion</t>
+        </is>
+      </c>
+      <c r="C95" s="18" t="inlineStr">
+        <is>
+          <t>Logic/Math</t>
+        </is>
+      </c>
+      <c r="D95" s="18" t="inlineStr">
+        <is>
+          <t>Power of Three</t>
+        </is>
+      </c>
+      <c r="E95" s="18" t="inlineStr">
+        <is>
+          <t>Recursion</t>
+        </is>
+      </c>
+      <c r="F95" s="19" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/power-of-three/</t>
+        </is>
+      </c>
+      <c r="G95" s="20" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H95" s="18" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I95" s="17" t="inlineStr">
+        <is>
+          <t>21-08-2026</t>
+        </is>
+      </c>
+      <c r="J95" s="17" t="inlineStr"/>
+      <c r="K95" s="17" t="inlineStr"/>
+      <c r="L95" s="17" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="13" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="14" t="inlineStr">
+        <is>
+          <t>Recursion</t>
+        </is>
+      </c>
+      <c r="C96" s="14" t="inlineStr">
         <is>
           <t>Power</t>
         </is>
       </c>
-      <c r="D86" s="14" t="inlineStr">
+      <c r="D96" s="14" t="inlineStr">
         <is>
           <t>Pow(x, n)</t>
         </is>
       </c>
-      <c r="E86" s="14" t="inlineStr">
+      <c r="E96" s="14" t="inlineStr">
         <is>
           <t>Recursion</t>
         </is>
       </c>
-      <c r="F86" s="15" t="inlineStr">
+      <c r="F96" s="15" t="inlineStr">
         <is>
           <t>https://leetcode.com/problems/powx-n/</t>
         </is>
       </c>
-      <c r="G86" s="21" t="inlineStr">
+      <c r="G96" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H86" s="14" t="n"/>
-      <c r="I86" s="13" t="n"/>
-      <c r="J86" s="13" t="n"/>
-      <c r="K86" s="13" t="n"/>
-      <c r="L86" s="13" t="n"/>
+      <c r="H96" s="14" t="inlineStr"/>
+      <c r="I96" s="13" t="inlineStr"/>
+      <c r="J96" s="13" t="inlineStr"/>
+      <c r="K96" s="13" t="inlineStr"/>
+      <c r="L96" s="13" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="17" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="18" t="inlineStr">
+        <is>
+          <t>Trees</t>
+        </is>
+      </c>
+      <c r="C97" s="18" t="inlineStr">
+        <is>
+          <t>Binary Tree DFS</t>
+        </is>
+      </c>
+      <c r="D97" s="18" t="inlineStr">
+        <is>
+          <t>Count Nodes Equal to Average of Subtree</t>
+        </is>
+      </c>
+      <c r="E97" s="18" t="inlineStr">
+        <is>
+          <t>Postorder Traversal</t>
+        </is>
+      </c>
+      <c r="F97" s="19" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/count-nodes-equal-to-average-of-subtree/</t>
+        </is>
+      </c>
+      <c r="G97" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H97" s="18" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I97" s="17" t="inlineStr">
+        <is>
+          <t>10-09-2026</t>
+        </is>
+      </c>
+      <c r="J97" s="17" t="inlineStr"/>
+      <c r="K97" s="17" t="inlineStr"/>
+      <c r="L97" s="17" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="13" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="14" t="inlineStr">
+        <is>
+          <t>Dynamic Programming</t>
+        </is>
+      </c>
+      <c r="C98" s="14" t="inlineStr">
+        <is>
+          <t>String DP</t>
+        </is>
+      </c>
+      <c r="D98" s="14" t="inlineStr">
+        <is>
+          <t>Distinct Subsequences</t>
+        </is>
+      </c>
+      <c r="E98" s="14" t="inlineStr">
+        <is>
+          <t>2D DP</t>
+        </is>
+      </c>
+      <c r="F98" s="15" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/distinct-subsequences/</t>
+        </is>
+      </c>
+      <c r="G98" s="24" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H98" s="14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I98" s="13" t="inlineStr">
+        <is>
+          <t>06-09-2026</t>
+        </is>
+      </c>
+      <c r="J98" s="13" t="inlineStr"/>
+      <c r="K98" s="13" t="inlineStr"/>
+      <c r="L98" s="13" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="17" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="18" t="inlineStr">
+        <is>
+          <t>Dynamic Programming</t>
+        </is>
+      </c>
+      <c r="C99" s="18" t="inlineStr">
+        <is>
+          <t>String DP</t>
+        </is>
+      </c>
+      <c r="D99" s="18" t="inlineStr">
+        <is>
+          <t>Distinct Subsequences II</t>
+        </is>
+      </c>
+      <c r="E99" s="18" t="inlineStr">
+        <is>
+          <t>1D DP / Prefix Sum</t>
+        </is>
+      </c>
+      <c r="F99" s="19" t="inlineStr">
+        <is>
+          <t>https://leetcode.com/problems/distinct-subsequences-ii/</t>
+        </is>
+      </c>
+      <c r="G99" s="23" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H99" s="18" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I99" s="17" t="inlineStr">
+        <is>
+          <t>07-09-2026</t>
+        </is>
+      </c>
+      <c r="J99" s="17" t="inlineStr"/>
+      <c r="K99" s="17" t="inlineStr"/>
+      <c r="L99" s="17" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L69"/>
+  <autoFilter ref="A1:L99"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
@@ -4805,6 +5433,19 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F84" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F85" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F99" r:id="rId98"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>